<commit_message>
Fix hip-hop periodic table data errors
- hiphop_artists.xlsx (drives the site):
  - Fill all 139 blank Composite Scores (mean of the 5 lyrical dims);
    previously every tile's score bar rendered as 0
  - Fix Era typo "Late 99s" -> "Late 90s"
  - Enrich 136 artist descriptions from the 5-dimension dataset
- HipHop_150_5Dim.xlsx:
  - Fix 10 "late 99s" -> "late 90s" Era typos
  - Rebuild corrupted "Era x Dimension Averages" sheet (Late 90s era was
    split into two rows by the typo) -> one clean row per era

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artist Database" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Artist Database" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Artist Database'!$A$1:$R$1</definedName>
@@ -741,9 +741,8 @@
       <c r="N2" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O2" s="6">
-        <f>AVERAGE(J2:N2)</f>
-        <v/>
+      <c r="O2" s="6" t="n">
+        <v>3</v>
       </c>
       <c r="P2" s="7" t="inlineStr">
         <is>
@@ -814,9 +813,8 @@
       <c r="N3" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O3" s="6">
-        <f>AVERAGE(J3:N3)</f>
-        <v/>
+      <c r="O3" s="6" t="n">
+        <v>5.6</v>
       </c>
       <c r="P3" s="7" t="inlineStr">
         <is>
@@ -887,9 +885,8 @@
       <c r="N4" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O4" s="6">
-        <f>AVERAGE(J4:N4)</f>
-        <v/>
+      <c r="O4" s="6" t="n">
+        <v>7.6</v>
       </c>
       <c r="P4" s="7" t="inlineStr">
         <is>
@@ -899,7 +896,7 @@
       <c r="Q4" s="2" t="inlineStr"/>
       <c r="R4" s="2" t="inlineStr">
         <is>
-          <t>'The Message' redefined what rap could say.</t>
+          <t>'The Message' — first truly serious rap lyric. Dark imagery of urban decay.</t>
         </is>
       </c>
     </row>
@@ -960,9 +957,8 @@
       <c r="N5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="O5" s="6">
-        <f>AVERAGE(J5:N5)</f>
-        <v/>
+      <c r="O5" s="6" t="n">
+        <v>3.2</v>
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
@@ -972,7 +968,7 @@
       <c r="Q5" s="2" t="inlineStr"/>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>First commercial rap hit.</t>
+          <t>Brought hip-hop mainstream with 'Rapper's Delight'.</t>
         </is>
       </c>
     </row>
@@ -1033,9 +1029,8 @@
       <c r="N6" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O6" s="6">
-        <f>AVERAGE(J6:N6)</f>
-        <v/>
+      <c r="O6" s="6" t="n">
+        <v>4.4</v>
       </c>
       <c r="P6" s="7" t="inlineStr">
         <is>
@@ -1045,7 +1040,7 @@
       <c r="Q6" s="2" t="inlineStr"/>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>Zulu Nation founder. Bridged hip-hop to electronic music.</t>
+          <t>'Planet Rock' visionary. Pan-African ideology in party form.</t>
         </is>
       </c>
     </row>
@@ -1106,9 +1101,8 @@
       <c r="N7" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O7" s="6">
-        <f>AVERAGE(J7:N7)</f>
-        <v/>
+      <c r="O7" s="6" t="n">
+        <v>5.4</v>
       </c>
       <c r="P7" s="7" t="inlineStr">
         <is>
@@ -1118,7 +1112,7 @@
       <c r="Q7" s="2" t="inlineStr"/>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>Defied rock and roll skeptics. First major Def Jam artist.</t>
+          <t>Def Jam's first star. Swagger as technique.</t>
         </is>
       </c>
     </row>
@@ -1179,9 +1173,8 @@
       <c r="N8" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O8" s="6">
-        <f>AVERAGE(J8:N8)</f>
-        <v/>
+      <c r="O8" s="6" t="n">
+        <v>5.2</v>
       </c>
       <c r="P8" s="7" t="inlineStr">
         <is>
@@ -1191,7 +1184,7 @@
       <c r="Q8" s="2" t="inlineStr"/>
       <c r="R8" s="2" t="inlineStr">
         <is>
-          <t>Integrated rock into rap. Made Adidas iconic.</t>
+          <t>Merged rock and rap. Iconic minimalism.</t>
         </is>
       </c>
     </row>
@@ -1252,9 +1245,8 @@
       <c r="N9" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O9" s="6">
-        <f>AVERAGE(J9:N9)</f>
-        <v/>
+      <c r="O9" s="6" t="n">
+        <v>5.8</v>
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
@@ -1264,7 +1256,7 @@
       <c r="Q9" s="2" t="inlineStr"/>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>Crossover kings. Made rap acceptable to white rock audiences.</t>
+          <t>Frenetic cultural collage. Grew into genuine experimental sophistication.</t>
         </is>
       </c>
     </row>
@@ -1325,9 +1317,8 @@
       <c r="N10" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O10" s="6">
-        <f>AVERAGE(J10:N10)</f>
-        <v/>
+      <c r="O10" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P10" s="7" t="inlineStr">
         <is>
@@ -1337,7 +1328,7 @@
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>The Teacha. 'South Bronx' battle classic.</t>
+          <t>'The Teacha.' Hip-hop philosopher-MC.</t>
         </is>
       </c>
     </row>
@@ -1398,9 +1389,8 @@
       <c r="N11" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="O11" s="6">
-        <f>AVERAGE(J11:N11)</f>
-        <v/>
+      <c r="O11" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
@@ -1410,7 +1400,7 @@
       <c r="Q11" s="2" t="inlineStr"/>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>Most politically explosive group in rap history.</t>
+          <t>Maximum political rage. Bomb Squad production as sonic warfare.</t>
         </is>
       </c>
     </row>
@@ -1471,9 +1461,8 @@
       <c r="N12" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O12" s="6">
-        <f>AVERAGE(J12:N12)</f>
-        <v/>
+      <c r="O12" s="6" t="n">
+        <v>6.2</v>
       </c>
       <c r="P12" s="14" t="inlineStr">
         <is>
@@ -1487,7 +1476,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>First female voice in a rap beef. Battle rap pioneer.</t>
+          <t>Pioneer female MC. Battle rap legend at age 14. Foundational for women in hip-hop.</t>
         </is>
       </c>
     </row>
@@ -1548,9 +1537,8 @@
       <c r="N13" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O13" s="6">
-        <f>AVERAGE(J13:N13)</f>
-        <v/>
+      <c r="O13" s="6" t="n">
+        <v>6.8</v>
       </c>
       <c r="P13" s="14" t="inlineStr">
         <is>
@@ -1564,7 +1552,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>First female rapper to release a full solo album.</t>
+          <t>First solo female rapper to release a full album. Sharp, authoritative delivery.</t>
         </is>
       </c>
     </row>
@@ -1625,9 +1613,8 @@
       <c r="N14" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O14" s="6">
-        <f>AVERAGE(J14:N14)</f>
-        <v/>
+      <c r="O14" s="6" t="n">
+        <v>5.4</v>
       </c>
       <c r="P14" s="14" t="inlineStr">
         <is>
@@ -1641,7 +1628,7 @@
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Godfather of gangsta rap. Influence often unacknowledged.</t>
+          <t>Philadelphia proto-gangsta rapper. Predates N.W.A's gangsta template.</t>
         </is>
       </c>
     </row>
@@ -1702,9 +1689,8 @@
       <c r="N15" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="O15" s="6">
-        <f>AVERAGE(J15:N15)</f>
-        <v/>
+      <c r="O15" s="6" t="n">
+        <v>3.6</v>
       </c>
       <c r="P15" s="15" t="inlineStr">
         <is>
@@ -1718,7 +1704,7 @@
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Supersonic. Early Ruthless Records female act.</t>
+          <t>First rap group Grammy-nominated. Female-fronted electro-hop novelty hit.</t>
         </is>
       </c>
     </row>
@@ -1779,9 +1765,8 @@
       <c r="N16" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O16" s="6">
-        <f>AVERAGE(J16:N16)</f>
-        <v/>
+      <c r="O16" s="6" t="n">
+        <v>4.6</v>
       </c>
       <c r="P16" s="14" t="inlineStr">
         <is>
@@ -1795,7 +1780,7 @@
       </c>
       <c r="R16" s="2" t="inlineStr">
         <is>
-          <t>Crossover R&amp;B-rap. Smooth sophistication in Old School era.</t>
+          <t>Early electro-rap crossover. Bridged disco and hip-hop aesthetics.</t>
         </is>
       </c>
     </row>
@@ -1856,9 +1841,8 @@
       <c r="N17" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O17" s="6">
-        <f>AVERAGE(J17:N17)</f>
-        <v/>
+      <c r="O17" s="6" t="n">
+        <v>5.4</v>
       </c>
       <c r="P17" s="14" t="inlineStr">
         <is>
@@ -1872,7 +1856,7 @@
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>Human beatbox originator. 'La Di Da Di' with Slick Rick.</t>
+          <t>Human beatbox pioneer. 'La Di Da Di' a canonical party rap text.</t>
         </is>
       </c>
     </row>
@@ -1933,9 +1917,8 @@
       <c r="N18" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O18" s="6">
-        <f>AVERAGE(J18:N18)</f>
-        <v/>
+      <c r="O18" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
@@ -1945,7 +1928,7 @@
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="inlineStr">
         <is>
-          <t>Master storyteller. 'Children's Story' is a narrative benchmark.</t>
+          <t>Master storyteller. Cockney-inflected delivery, vivid street fables.</t>
         </is>
       </c>
     </row>
@@ -2006,9 +1989,8 @@
       <c r="N19" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O19" s="6">
-        <f>AVERAGE(J19:N19)</f>
-        <v/>
+      <c r="O19" s="6" t="n">
+        <v>5.8</v>
       </c>
       <c r="P19" s="15" t="inlineStr">
         <is>
@@ -2022,7 +2004,7 @@
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Slick Rick adjacent storyteller. Underrated narrative voice.</t>
+          <t>Storytelling peer to Slick Rick. Underrated narrative rapper.</t>
         </is>
       </c>
     </row>
@@ -2083,9 +2065,8 @@
       <c r="N20" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O20" s="6">
-        <f>AVERAGE(J20:N20)</f>
-        <v/>
+      <c r="O20" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
@@ -2095,7 +2076,7 @@
       <c r="Q20" s="2" t="inlineStr"/>
       <c r="R20" s="2" t="inlineStr">
         <is>
-          <t>Smoothed battle rap into an art form. Influenced Jay-Z directly.</t>
+          <t>Velvet-glove delivery hiding razor-sharp multisyllabic patterns.</t>
         </is>
       </c>
     </row>
@@ -2156,9 +2137,8 @@
       <c r="N21" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O21" s="6">
-        <f>AVERAGE(J21:N21)</f>
-        <v/>
+      <c r="O21" s="6" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
@@ -2168,7 +2148,7 @@
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>Rewired how MCs thought about flow. The God MC.</t>
+          <t>Invented internal rhyme as default mode. The God MC.</t>
         </is>
       </c>
     </row>
@@ -2229,9 +2209,8 @@
       <c r="N22" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O22" s="6">
-        <f>AVERAGE(J22:N22)</f>
-        <v/>
+      <c r="O22" s="6" t="n">
+        <v>7.6</v>
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
@@ -2241,7 +2220,7 @@
       <c r="Q22" s="2" t="inlineStr"/>
       <c r="R22" s="2" t="inlineStr">
         <is>
-          <t>U.N.I.T.Y. feminist anthem. First lady of hip-hop royalty.</t>
+          <t>Regal feminist authority. Foundational for women in rap.</t>
         </is>
       </c>
     </row>
@@ -2302,9 +2281,8 @@
       <c r="N23" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O23" s="6">
-        <f>AVERAGE(J23:N23)</f>
-        <v/>
+      <c r="O23" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
@@ -2314,7 +2292,7 @@
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="inlineStr">
         <is>
-          <t>Straight Outta Compton. Made the coasts speak different languages.</t>
+          <t>Invented gangsta rap. Vérité street journalism.</t>
         </is>
       </c>
     </row>
@@ -2375,9 +2353,8 @@
       <c r="N24" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O24" s="6">
-        <f>AVERAGE(J24:N24)</f>
-        <v/>
+      <c r="O24" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
@@ -2387,7 +2364,7 @@
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="inlineStr">
         <is>
-          <t>N.W.A pen. AmeriKKKa's Most Wanted is a lyrical high-water mark.</t>
+          <t>N.W.A's sharpest writer. Furious precision.</t>
         </is>
       </c>
     </row>
@@ -2448,9 +2425,8 @@
       <c r="N25" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O25" s="6">
-        <f>AVERAGE(J25:N25)</f>
-        <v/>
+      <c r="O25" s="6" t="n">
+        <v>7.6</v>
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
@@ -2460,7 +2436,7 @@
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="inlineStr">
         <is>
-          <t>3 Feet High and Rising. Made sampling feel like art.</t>
+          <t>Playful polymaths. Vast vocabulary with absurdist wit.</t>
         </is>
       </c>
     </row>
@@ -2521,9 +2497,8 @@
       <c r="N26" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O26" s="6">
-        <f>AVERAGE(J26:N26)</f>
-        <v/>
+      <c r="O26" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P26" s="7" t="inlineStr">
         <is>
@@ -2533,7 +2508,7 @@
       <c r="Q26" s="2" t="inlineStr"/>
       <c r="R26" s="2" t="inlineStr">
         <is>
-          <t>Married jazz and hip-hop elegantly. The Low End Theory is essential.</t>
+          <t>Q-Tip's conversational genius. Jazz improvisation in verse.</t>
         </is>
       </c>
     </row>
@@ -2594,9 +2569,8 @@
       <c r="N27" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O27" s="6">
-        <f>AVERAGE(J27:N27)</f>
-        <v/>
+      <c r="O27" s="6" t="n">
+        <v>9.4</v>
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
@@ -2606,7 +2580,7 @@
       <c r="Q27" s="2" t="inlineStr"/>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>Illmatic remains the most critically studied debut in rap.</t>
+          <t>'Illmatic' distilled Queensbridge into literary art.</t>
         </is>
       </c>
     </row>
@@ -2667,9 +2641,8 @@
       <c r="N28" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O28" s="6">
-        <f>AVERAGE(J28:N28)</f>
-        <v/>
+      <c r="O28" s="6" t="n">
+        <v>9</v>
       </c>
       <c r="P28" s="7" t="inlineStr">
         <is>
@@ -2679,7 +2652,7 @@
       <c r="Q28" s="2" t="inlineStr"/>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>Lyrical density and narrative gift in equal measure.</t>
+          <t>Greatest natural storyteller. Cinematic scenes, effortless charisma.</t>
         </is>
       </c>
     </row>
@@ -2740,9 +2713,8 @@
       <c r="N29" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O29" s="6">
-        <f>AVERAGE(J29:N29)</f>
-        <v/>
+      <c r="O29" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
@@ -2752,7 +2724,7 @@
       <c r="Q29" s="2" t="inlineStr"/>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>Enter the 36 Chambers. Martial arts mythology meets Shaolin New York.</t>
+          <t>Nine MCs, nine styles. Martial mythology meets grim NY street.</t>
         </is>
       </c>
     </row>
@@ -2813,9 +2785,8 @@
       <c r="N30" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O30" s="6">
-        <f>AVERAGE(J30:N30)</f>
-        <v/>
+      <c r="O30" s="6" t="n">
+        <v>6.6</v>
       </c>
       <c r="P30" s="7" t="inlineStr">
         <is>
@@ -2825,7 +2796,7 @@
       <c r="Q30" s="2" t="inlineStr"/>
       <c r="R30" s="2" t="inlineStr">
         <is>
-          <t>Iconic delivery over Dre's G-Funk. Doggystyle defined an era.</t>
+          <t>Flow as personality. Delivery transcends lyrical content.</t>
         </is>
       </c>
     </row>
@@ -2886,9 +2857,8 @@
       <c r="N31" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O31" s="6">
-        <f>AVERAGE(J31:N31)</f>
-        <v/>
+      <c r="O31" s="6" t="n">
+        <v>5.6</v>
       </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
@@ -2898,7 +2868,7 @@
       <c r="Q31" s="2" t="inlineStr"/>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>G-Funk architect. The Chronic changed West Coast sound globally.</t>
+          <t>Producer-first. Lyricism secondary to sonic architecture.</t>
         </is>
       </c>
     </row>
@@ -2959,9 +2929,8 @@
       <c r="N32" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O32" s="6">
-        <f>AVERAGE(J32:N32)</f>
-        <v/>
+      <c r="O32" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P32" s="7" t="inlineStr">
         <is>
@@ -2971,7 +2940,7 @@
       <c r="Q32" s="2" t="inlineStr"/>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>Bizarre Ride II. Quirky alternative to gangsta dominance.</t>
+          <t>Acrobatic, joyful wordplay. LA's alternative answer to De La Soul.</t>
         </is>
       </c>
     </row>
@@ -3032,9 +3001,8 @@
       <c r="N33" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O33" s="6">
-        <f>AVERAGE(J33:N33)</f>
-        <v/>
+      <c r="O33" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
@@ -3044,7 +3012,7 @@
       <c r="Q33" s="2" t="inlineStr"/>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>The Infamous is peak Queens gothic menace.</t>
+          <t>Prodigy's paranoid poetry over Havoc's glacial loops.</t>
         </is>
       </c>
     </row>
@@ -3105,9 +3073,8 @@
       <c r="N34" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O34" s="6">
-        <f>AVERAGE(J34:N34)</f>
-        <v/>
+      <c r="O34" s="6" t="n">
+        <v>6.8</v>
       </c>
       <c r="P34" s="7" t="inlineStr">
         <is>
@@ -3117,7 +3084,7 @@
       <c r="Q34" s="2" t="inlineStr"/>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>Dictionary of Bay slang. Slanguistics pioneer.</t>
+          <t>Slang inventor. Vocabulary innovation as primary art form.</t>
         </is>
       </c>
     </row>
@@ -3178,9 +3145,8 @@
       <c r="N35" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O35" s="6">
-        <f>AVERAGE(J35:N35)</f>
-        <v/>
+      <c r="O35" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P35" s="14" t="inlineStr">
         <is>
@@ -3194,7 +3160,7 @@
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>Mecca and the Soul Brother. CL Smooth's introspection over Pete's soul.</t>
+          <t>Pete Rock's jazz-inflected production plus CL Smooth's introspective flows.</t>
         </is>
       </c>
     </row>
@@ -3255,9 +3221,8 @@
       <c r="N36" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O36" s="6">
-        <f>AVERAGE(J36:N36)</f>
-        <v/>
+      <c r="O36" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P36" s="7" t="inlineStr">
         <is>
@@ -3267,7 +3232,7 @@
       <c r="Q36" s="2" t="inlineStr"/>
       <c r="R36" s="2" t="inlineStr">
         <is>
-          <t>Guru's flat-affect wisdom over Primo's chopped jazz. Step In the Arena.</t>
+          <t>Guru's monotone wisdom over DJ Premier's crate-dug perfection.</t>
         </is>
       </c>
     </row>
@@ -3328,9 +3293,8 @@
       <c r="N37" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O37" s="6">
-        <f>AVERAGE(J37:N37)</f>
-        <v/>
+      <c r="O37" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P37" s="14" t="inlineStr">
         <is>
@@ -3344,7 +3308,7 @@
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>5% Nation theology in hip-hop. One for All is a conscious landmark.</t>
+          <t>5 Percenter theology meets Afrocentric fury. Sadat X and Grand Puba.</t>
         </is>
       </c>
     </row>
@@ -3405,9 +3369,8 @@
       <c r="N38" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O38" s="6">
-        <f>AVERAGE(J38:N38)</f>
-        <v/>
+      <c r="O38" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="P38" s="14" t="inlineStr">
         <is>
@@ -3421,7 +3384,7 @@
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>To the East Blackwards. Black nationalist aesthetics in full bloom.</t>
+          <t>Black nationalist imagery and Afrocentric symbolism at maximum.</t>
         </is>
       </c>
     </row>
@@ -3482,9 +3445,8 @@
       <c r="N39" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O39" s="6">
-        <f>AVERAGE(J39:N39)</f>
-        <v/>
+      <c r="O39" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
@@ -3494,7 +3456,7 @@
       <c r="Q39" s="2" t="inlineStr"/>
       <c r="R39" s="2" t="inlineStr">
         <is>
-          <t>Punchline king. Lifestylez ov da Poor &amp; Dangerous is criminally slept on.</t>
+          <t>Punchline architect. Harlem's greatest. Wordplay density rivals anyone.</t>
         </is>
       </c>
     </row>
@@ -3555,9 +3517,8 @@
       <c r="N40" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O40" s="6">
-        <f>AVERAGE(J40:N40)</f>
-        <v/>
+      <c r="O40" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P40" s="7" t="inlineStr">
         <is>
@@ -3567,7 +3528,7 @@
       <c r="Q40" s="2" t="inlineStr"/>
       <c r="R40" s="2" t="inlineStr">
         <is>
-          <t>My Mind Playing Tricks on Me. Southern rap's dark psychological turn.</t>
+          <t>Pioneered Southern horror-gangsta. Scarface's lyrical foundation.</t>
         </is>
       </c>
     </row>
@@ -3628,9 +3589,8 @@
       <c r="N41" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O41" s="6">
-        <f>AVERAGE(J41:N41)</f>
-        <v/>
+      <c r="O41" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P41" s="14" t="inlineStr">
         <is>
@@ -3644,7 +3604,7 @@
       </c>
       <c r="R41" s="2" t="inlineStr">
         <is>
-          <t>Innercity Griots. Improvised lyricism from the Good Life Café scene.</t>
+          <t>LA's jazz-rap underground. Aceyalone among the most technically gifted MCs ever.</t>
         </is>
       </c>
     </row>
@@ -3705,9 +3665,8 @@
       <c r="N42" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O42" s="6">
-        <f>AVERAGE(J42:N42)</f>
-        <v/>
+      <c r="O42" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="P42" s="14" t="inlineStr">
         <is>
@@ -3721,7 +3680,7 @@
       </c>
       <c r="R42" s="2" t="inlineStr">
         <is>
-          <t>Reachin' (A New Refutation of Time and Space). Bohemian cool jazz.</t>
+          <t>Cool jazz-rap fusion. Ladybug Mecca one of the era's sharpest female voices.</t>
         </is>
       </c>
     </row>
@@ -3782,9 +3741,8 @@
       <c r="N43" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O43" s="6">
-        <f>AVERAGE(J43:N43)</f>
-        <v/>
+      <c r="O43" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P43" s="14" t="inlineStr">
         <is>
@@ -3798,7 +3756,7 @@
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>A Future Without a Past. Busta Rhymes's stage before his solo explosions.</t>
+          <t>Launched Busta Rhymes. Charlie Brown and Dinco D also strong voices.</t>
         </is>
       </c>
     </row>
@@ -3859,9 +3817,8 @@
       <c r="N44" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O44" s="6">
-        <f>AVERAGE(J44:N44)</f>
-        <v/>
+      <c r="O44" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P44" s="7" t="inlineStr">
         <is>
@@ -3871,7 +3828,7 @@
       <c r="Q44" s="2" t="inlineStr"/>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>Hyperkinetic flow and energy. The Coming announced a superstar.</t>
+          <t>Hyper-kinetic delivery and flow complexity. One of the fastest MCs ever.</t>
         </is>
       </c>
     </row>
@@ -3932,9 +3889,8 @@
       <c r="N45" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O45" s="6">
-        <f>AVERAGE(J45:N45)</f>
-        <v/>
+      <c r="O45" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P45" s="7" t="inlineStr">
         <is>
@@ -3944,7 +3900,7 @@
       <c r="Q45" s="2" t="inlineStr"/>
       <c r="R45" s="2" t="inlineStr">
         <is>
-          <t>Me Against the World / All Eyez on Me. Embodied generational pain.</t>
+          <t>Raw emotional intelligence. Political rage and personal vulnerability.</t>
         </is>
       </c>
     </row>
@@ -4005,9 +3961,8 @@
       <c r="N46" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O46" s="6">
-        <f>AVERAGE(J46:N46)</f>
-        <v/>
+      <c r="O46" s="6" t="n">
+        <v>8.6</v>
       </c>
       <c r="P46" s="7" t="inlineStr">
         <is>
@@ -4017,7 +3972,7 @@
       <c r="Q46" s="2" t="inlineStr"/>
       <c r="R46" s="2" t="inlineStr">
         <is>
-          <t>Reasonable Doubt to Blueprint. Business and artistry in concert.</t>
+          <t>Effortless mastery. Hustler's autobiography as album architecture.</t>
         </is>
       </c>
     </row>
@@ -4078,9 +4033,8 @@
       <c r="N47" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O47" s="6">
-        <f>AVERAGE(J47:N47)</f>
-        <v/>
+      <c r="O47" s="6" t="n">
+        <v>9.199999999999999</v>
       </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
@@ -4090,7 +4044,7 @@
       <c r="Q47" s="2" t="inlineStr"/>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>Slim Shady LP. Technical rhyme density unchallenged in any era.</t>
+          <t>Most technically precise rapper. Internal rhyme density off the charts.</t>
         </is>
       </c>
     </row>
@@ -4151,9 +4105,8 @@
       <c r="N48" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O48" s="6">
-        <f>AVERAGE(J48:N48)</f>
-        <v/>
+      <c r="O48" s="6" t="n">
+        <v>6.2</v>
       </c>
       <c r="P48" s="7" t="inlineStr">
         <is>
@@ -4163,7 +4116,7 @@
       <c r="Q48" s="2" t="inlineStr"/>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>Barking aggression as spiritual crisis. It's Dark and Hell Is Hot.</t>
+          <t>Primal confessional fury. Power through raw emotional delivery.</t>
         </is>
       </c>
     </row>
@@ -4224,9 +4177,8 @@
       <c r="N49" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O49" s="6">
-        <f>AVERAGE(J49:N49)</f>
-        <v/>
+      <c r="O49" s="6" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
@@ -4236,7 +4188,7 @@
       <c r="Q49" s="2" t="inlineStr"/>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>Miseducation is the high point of rap-soul fusion.</t>
+          <t>'Miseducation' — radical emotional honesty + technical precision.</t>
         </is>
       </c>
     </row>
@@ -4297,9 +4249,8 @@
       <c r="N50" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O50" s="6">
-        <f>AVERAGE(J50:N50)</f>
-        <v/>
+      <c r="O50" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P50" s="7" t="inlineStr">
         <is>
@@ -4309,7 +4260,7 @@
       <c r="Q50" s="2" t="inlineStr"/>
       <c r="R50" s="2" t="inlineStr">
         <is>
-          <t>Supa Dupa Fly. Avant-garde Southern vision over Timbaland.</t>
+          <t>Flow as futurist sculpture. Rhythm manipulation over traditional lyricism.</t>
         </is>
       </c>
     </row>
@@ -4370,9 +4321,8 @@
       <c r="N51" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O51" s="6">
-        <f>AVERAGE(J51:N51)</f>
-        <v/>
+      <c r="O51" s="6" t="n">
+        <v>8.6</v>
       </c>
       <c r="P51" s="7" t="inlineStr">
         <is>
@@ -4382,7 +4332,7 @@
       <c r="Q51" s="2" t="inlineStr"/>
       <c r="R51" s="2" t="inlineStr">
         <is>
-          <t>Black on Both Sides. Renaissance man MC.</t>
+          <t>'Black on Both Sides' — blues, jazz, politics in one voice.</t>
         </is>
       </c>
     </row>
@@ -4443,9 +4393,8 @@
       <c r="N52" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O52" s="6">
-        <f>AVERAGE(J52:N52)</f>
-        <v/>
+      <c r="O52" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P52" s="7" t="inlineStr">
         <is>
@@ -4455,7 +4404,7 @@
       <c r="Q52" s="2" t="inlineStr"/>
       <c r="R52" s="2" t="inlineStr">
         <is>
-          <t>Reflection Eternal. Wordy, dense, deeply political.</t>
+          <t>Brooklyn's dense intellectual. Every bar packed with history.</t>
         </is>
       </c>
     </row>
@@ -4516,9 +4465,8 @@
       <c r="N53" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O53" s="6">
-        <f>AVERAGE(J53:N53)</f>
-        <v/>
+      <c r="O53" s="6" t="n">
+        <v>8.6</v>
       </c>
       <c r="P53" s="7" t="inlineStr">
         <is>
@@ -4528,7 +4476,7 @@
       <c r="Q53" s="2" t="inlineStr"/>
       <c r="R53" s="2" t="inlineStr">
         <is>
-          <t>Aquemini. Andre 3000 is a singular artistic voice.</t>
+          <t>Andre 3000: genre-defying poet. Big Boi: underrated technical master.</t>
         </is>
       </c>
     </row>
@@ -4589,9 +4537,8 @@
       <c r="N54" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O54" s="6">
-        <f>AVERAGE(J54:N54)</f>
-        <v/>
+      <c r="O54" s="6" t="n">
+        <v>3.8</v>
       </c>
       <c r="P54" s="7" t="inlineStr">
         <is>
@@ -4601,7 +4548,7 @@
       <c r="Q54" s="2" t="inlineStr"/>
       <c r="R54" s="2" t="inlineStr">
         <is>
-          <t>Ghetto D. Cash Money architect. Business over lyricism.</t>
+          <t>Mogul over MC. Influence is business, not bars.</t>
         </is>
       </c>
     </row>
@@ -4662,9 +4609,8 @@
       <c r="N55" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O55" s="6">
-        <f>AVERAGE(J55:N55)</f>
-        <v/>
+      <c r="O55" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="P55" s="14" t="inlineStr">
         <is>
@@ -4678,7 +4624,7 @@
       </c>
       <c r="R55" s="2" t="inlineStr">
         <is>
-          <t>Come Home with Me. Pink fur and oblique rap logic.</t>
+          <t>Pink fur and slant rhymes. Harlem's most stylistically eccentric MC.</t>
         </is>
       </c>
     </row>
@@ -4739,9 +4685,8 @@
       <c r="N56" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O56" s="6">
-        <f>AVERAGE(J56:N56)</f>
-        <v/>
+      <c r="O56" s="6" t="n">
+        <v>6.8</v>
       </c>
       <c r="P56" s="14" t="inlineStr">
         <is>
@@ -4755,7 +4700,7 @@
       </c>
       <c r="R56" s="2" t="inlineStr">
         <is>
-          <t>Ill Na Na. Mafioso rap via the female gaze.</t>
+          <t>Aggressive feminine sexuality as lyrical weapon. Def Jam's answer to Lil Kim.</t>
         </is>
       </c>
     </row>
@@ -4816,9 +4761,8 @@
       <c r="N57" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O57" s="6">
-        <f>AVERAGE(J57:N57)</f>
-        <v/>
+      <c r="O57" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="P57" s="7" t="inlineStr">
         <is>
@@ -4828,7 +4772,7 @@
       <c r="Q57" s="2" t="inlineStr"/>
       <c r="R57" s="2" t="inlineStr">
         <is>
-          <t>Hard Core. Explicit female sexuality as power and disruption.</t>
+          <t>Radical sexual candor. Graphic feminism that rewrote what women could say in rap.</t>
         </is>
       </c>
     </row>
@@ -4853,7 +4797,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Late 99s</t>
+          <t>Late 90s</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -4889,9 +4833,8 @@
       <c r="N58" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O58" s="6">
-        <f>AVERAGE(J58:N58)</f>
-        <v/>
+      <c r="O58" s="6" t="n">
+        <v>5.8</v>
       </c>
       <c r="P58" s="14" t="inlineStr">
         <is>
@@ -4905,7 +4848,7 @@
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>400 Degreez. Cash Money's breakout moment.</t>
+          <t>Cash Money's first star. New Orleans bounce meets street narrative.</t>
         </is>
       </c>
     </row>
@@ -4966,9 +4909,8 @@
       <c r="N59" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O59" s="6">
-        <f>AVERAGE(J59:N59)</f>
-        <v/>
+      <c r="O59" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="P59" s="14" t="inlineStr">
         <is>
@@ -4982,7 +4924,7 @@
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>Syllable count obsessive. Battle loss to LL never fully recovered from.</t>
+          <t>Battle rap legend. Technical skill occasionally undermined by ego.</t>
         </is>
       </c>
     </row>
@@ -5043,9 +4985,8 @@
       <c r="N60" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O60" s="6">
-        <f>AVERAGE(J60:N60)</f>
-        <v/>
+      <c r="O60" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P60" s="15" t="inlineStr">
         <is>
@@ -5059,7 +5000,7 @@
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>Violent by Design. Horror-core meets political paranoia underground.</t>
+          <t>Philadelphia underground. Vinnie Paz's dense, conspiratorial lyricism.</t>
         </is>
       </c>
     </row>
@@ -5120,9 +5061,8 @@
       <c r="N61" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O61" s="6">
-        <f>AVERAGE(J61:N61)</f>
-        <v/>
+      <c r="O61" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
@@ -5132,7 +5072,7 @@
       <c r="Q61" s="2" t="inlineStr"/>
       <c r="R61" s="2" t="inlineStr">
         <is>
-          <t>Capital Punishment. First Latino rapper to go platinum solo.</t>
+          <t>First Latin rapper to go platinum solo. Multisyllabic rhyme virtuoso.</t>
         </is>
       </c>
     </row>
@@ -5193,9 +5133,8 @@
       <c r="N62" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O62" s="6">
-        <f>AVERAGE(J62:N62)</f>
-        <v/>
+      <c r="O62" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P62" s="14" t="inlineStr">
         <is>
@@ -5209,7 +5148,7 @@
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>Life's a Bitch collab. AZ's verse is among the finest in rap history.</t>
+          <t>AZ: One of the most underrated MCs of the era. 'Sugarhill' an all-time verse.</t>
         </is>
       </c>
     </row>
@@ -5270,9 +5209,8 @@
       <c r="N63" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="O63" s="6">
-        <f>AVERAGE(J63:N63)</f>
-        <v/>
+      <c r="O63" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P63" s="7" t="inlineStr">
         <is>
@@ -5282,7 +5220,7 @@
       <c r="Q63" s="2" t="inlineStr"/>
       <c r="R63" s="2" t="inlineStr">
         <is>
-          <t>College Dropout to 808s. Artistic ambition reshapes each era.</t>
+          <t>Conceptual ambition as primary engine. Each album a reinvention.</t>
         </is>
       </c>
     </row>
@@ -5343,9 +5281,8 @@
       <c r="N64" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O64" s="6">
-        <f>AVERAGE(J64:N64)</f>
-        <v/>
+      <c r="O64" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P64" s="7" t="inlineStr">
         <is>
@@ -5355,7 +5292,7 @@
       <c r="Q64" s="2" t="inlineStr"/>
       <c r="R64" s="2" t="inlineStr">
         <is>
-          <t>Tha Carter III. Mixtape era Wayne is the definition of peak lyricism.</t>
+          <t>Simile machine at peak. Abstract metaphor-stacking as freestyle sport.</t>
         </is>
       </c>
     </row>
@@ -5416,9 +5353,8 @@
       <c r="N65" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O65" s="6">
-        <f>AVERAGE(J65:N65)</f>
-        <v/>
+      <c r="O65" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P65" s="7" t="inlineStr">
         <is>
@@ -5428,7 +5364,7 @@
       <c r="Q65" s="2" t="inlineStr"/>
       <c r="R65" s="2" t="inlineStr">
         <is>
-          <t>King. Claimed the ATL throne and the trap blueprint.</t>
+          <t>King of the South. Trap's emotional architect.</t>
         </is>
       </c>
     </row>
@@ -5489,9 +5425,8 @@
       <c r="N66" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O66" s="6">
-        <f>AVERAGE(J66:N66)</f>
-        <v/>
+      <c r="O66" s="6" t="n">
+        <v>4.8</v>
       </c>
       <c r="P66" s="7" t="inlineStr">
         <is>
@@ -5501,7 +5436,7 @@
       <c r="Q66" s="2" t="inlineStr"/>
       <c r="R66" s="2" t="inlineStr">
         <is>
-          <t>Trap God. Prolific mixtape movement godfather.</t>
+          <t>Vibe and charisma over craft. Trap music's spiritual godfather.</t>
         </is>
       </c>
     </row>
@@ -5562,9 +5497,8 @@
       <c r="N67" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O67" s="6">
-        <f>AVERAGE(J67:N67)</f>
-        <v/>
+      <c r="O67" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P67" s="7" t="inlineStr">
         <is>
@@ -5574,7 +5508,7 @@
       <c r="Q67" s="2" t="inlineStr"/>
       <c r="R67" s="2" t="inlineStr">
         <is>
-          <t>Supreme Clientele. Dense, dazzling, associative.</t>
+          <t>Stream-of-consciousness genius. Dense slang, vivid scene-painting.</t>
         </is>
       </c>
     </row>
@@ -5635,9 +5569,8 @@
       <c r="N68" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O68" s="6">
-        <f>AVERAGE(J68:N68)</f>
-        <v/>
+      <c r="O68" s="6" t="n">
+        <v>9.199999999999999</v>
       </c>
       <c r="P68" s="7" t="inlineStr">
         <is>
@@ -5647,7 +5580,7 @@
       <c r="Q68" s="2" t="inlineStr"/>
       <c r="R68" s="2" t="inlineStr">
         <is>
-          <t>Madvillainy. The mask, the myth, the syllable wizardry.</t>
+          <t>The supervillain. Labyrinths of internal rhyme no one has fully mapped.</t>
         </is>
       </c>
     </row>
@@ -5708,9 +5641,8 @@
       <c r="N69" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O69" s="6">
-        <f>AVERAGE(J69:N69)</f>
-        <v/>
+      <c r="O69" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P69" s="7" t="inlineStr">
         <is>
@@ -5720,7 +5652,7 @@
       <c r="Q69" s="2" t="inlineStr"/>
       <c r="R69" s="2" t="inlineStr">
         <is>
-          <t>Be. Elevated conscious rap into mainstream Grammy territory.</t>
+          <t>Chicago's philosopher-MC. Ernie Barnes paintings in verse form.</t>
         </is>
       </c>
     </row>
@@ -5781,9 +5713,8 @@
       <c r="N70" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O70" s="6">
-        <f>AVERAGE(J70:N70)</f>
-        <v/>
+      <c r="O70" s="6" t="n">
+        <v>6.6</v>
       </c>
       <c r="P70" s="7" t="inlineStr">
         <is>
@@ -5793,7 +5724,7 @@
       <c r="Q70" s="2" t="inlineStr"/>
       <c r="R70" s="2" t="inlineStr">
         <is>
-          <t>Word of Mouf. Playful Southern rapping with genuine lyrical edge.</t>
+          <t>Comic virtuosity. Punchline timing as precision instrument.</t>
         </is>
       </c>
     </row>
@@ -5854,9 +5785,8 @@
       <c r="N71" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O71" s="6">
-        <f>AVERAGE(J71:N71)</f>
-        <v/>
+      <c r="O71" s="6" t="n">
+        <v>5.4</v>
       </c>
       <c r="P71" s="7" t="inlineStr">
         <is>
@@ -5866,7 +5796,7 @@
       <c r="Q71" s="2" t="inlineStr"/>
       <c r="R71" s="2" t="inlineStr">
         <is>
-          <t>Let's Get It: Thug Motivation 101. Trap's motivational speaker.</t>
+          <t>Trap's motivational orator. Delivery and charisma over craft.</t>
         </is>
       </c>
     </row>
@@ -5927,9 +5857,8 @@
       <c r="N72" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="O72" s="6">
-        <f>AVERAGE(J72:N72)</f>
-        <v/>
+      <c r="O72" s="6" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="P72" s="7" t="inlineStr">
         <is>
@@ -5939,7 +5868,7 @@
       <c r="Q72" s="2" t="inlineStr"/>
       <c r="R72" s="2" t="inlineStr">
         <is>
-          <t>Food &amp; Liquor. Skate kid from Chicago with dictionary flow.</t>
+          <t>Conceptually sui generis. 'Dumb It Down' a rebuke of simplicity.</t>
         </is>
       </c>
     </row>
@@ -6000,9 +5929,8 @@
       <c r="N73" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O73" s="6">
-        <f>AVERAGE(J73:N73)</f>
-        <v/>
+      <c r="O73" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P73" s="7" t="inlineStr">
         <is>
@@ -6012,7 +5940,7 @@
       <c r="Q73" s="2" t="inlineStr"/>
       <c r="R73" s="2" t="inlineStr">
         <is>
-          <t>The World Is Yours. Southern rap's great novelist.</t>
+          <t>Houston's great novelist. Psychological interior in gangsta rap.</t>
         </is>
       </c>
     </row>
@@ -6073,9 +6001,8 @@
       <c r="N74" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O74" s="6">
-        <f>AVERAGE(J74:N74)</f>
-        <v/>
+      <c r="O74" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P74" s="7" t="inlineStr">
         <is>
@@ -6085,7 +6012,7 @@
       <c r="Q74" s="2" t="inlineStr"/>
       <c r="R74" s="2" t="inlineStr">
         <is>
-          <t>None Shall Pass. Largest vocabulary in measured rap.</t>
+          <t>NLP-verified largest unique vocabulary in rap. Dense abstract imagery.</t>
         </is>
       </c>
     </row>
@@ -6146,9 +6073,8 @@
       <c r="N75" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O75" s="6">
-        <f>AVERAGE(J75:N75)</f>
-        <v/>
+      <c r="O75" s="6" t="n">
+        <v>8.6</v>
       </c>
       <c r="P75" s="14" t="inlineStr">
         <is>
@@ -6162,7 +6088,7 @@
       </c>
       <c r="R75" s="2" t="inlineStr">
         <is>
-          <t>Fishscale is Ghostface at peak: cinematic, dense, unmatched.</t>
+          <t>'Fishscale' is a 2000s apex. Singular stream-of-consciousness voice.</t>
         </is>
       </c>
     </row>
@@ -6223,9 +6149,8 @@
       <c r="N76" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O76" s="6">
-        <f>AVERAGE(J76:N76)</f>
-        <v/>
+      <c r="O76" s="6" t="n">
+        <v>6.8</v>
       </c>
       <c r="P76" s="14" t="inlineStr">
         <is>
@@ -6239,7 +6164,7 @@
       </c>
       <c r="R76" s="2" t="inlineStr">
         <is>
-          <t>Why? punchline king. LOX member whose grimace became iconic.</t>
+          <t>Gravelly-voiced Yonkers MC. Punchline economy and street credibility.</t>
         </is>
       </c>
     </row>
@@ -6300,9 +6225,8 @@
       <c r="N77" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O77" s="6">
-        <f>AVERAGE(J77:N77)</f>
-        <v/>
+      <c r="O77" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="P77" s="7" t="inlineStr">
         <is>
@@ -6312,7 +6236,7 @@
       <c r="Q77" s="2" t="inlineStr"/>
       <c r="R77" s="2" t="inlineStr">
         <is>
-          <t>Get Rich or Die Tryin'. Commercial domination built on street cred.</t>
+          <t>Bulletproof charisma. Street narrative over lyrical complexity.</t>
         </is>
       </c>
     </row>
@@ -6373,9 +6297,8 @@
       <c r="N78" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O78" s="6">
-        <f>AVERAGE(J78:N78)</f>
-        <v/>
+      <c r="O78" s="6" t="n">
+        <v>5.6</v>
       </c>
       <c r="P78" s="14" t="inlineStr">
         <is>
@@ -6389,7 +6312,7 @@
       </c>
       <c r="R78" s="2" t="inlineStr">
         <is>
-          <t>Tear da Club Up. Memphis horrorcore before trap existed.</t>
+          <t>Oscar-winning Southern horror-rap. Pioneered the dark triplet flow.</t>
         </is>
       </c>
     </row>
@@ -6450,9 +6373,8 @@
       <c r="N79" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O79" s="6">
-        <f>AVERAGE(J79:N79)</f>
-        <v/>
+      <c r="O79" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P79" s="7" t="inlineStr">
         <is>
@@ -6462,7 +6384,7 @@
       <c r="Q79" s="2" t="inlineStr"/>
       <c r="R79" s="2" t="inlineStr">
         <is>
-          <t>Ridin' Dirty. Bun B and Pimp C: Southern rap's purist duo.</t>
+          <t>Bun B and Pimp C. Texas's most complete rap duo.</t>
         </is>
       </c>
     </row>
@@ -6523,9 +6445,8 @@
       <c r="N80" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O80" s="6">
-        <f>AVERAGE(J80:N80)</f>
-        <v/>
+      <c r="O80" s="6" t="n">
+        <v>6.4</v>
       </c>
       <c r="P80" s="15" t="inlineStr">
         <is>
@@ -6539,7 +6460,7 @@
       </c>
       <c r="R80" s="2" t="inlineStr">
         <is>
-          <t>Restless. Houston street reporting with slow, heavy flow.</t>
+          <t>Houston's street ambassador. Chopped-and-screwed delivery as identity.</t>
         </is>
       </c>
     </row>
@@ -6600,9 +6521,8 @@
       <c r="N81" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O81" s="6">
-        <f>AVERAGE(J81:N81)</f>
-        <v/>
+      <c r="O81" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P81" s="14" t="inlineStr">
         <is>
@@ -6616,7 +6536,7 @@
       </c>
       <c r="R81" s="2" t="inlineStr">
         <is>
-          <t>All Balls Don't Bounce. Project Blowed's academic underground MC.</t>
+          <t>LA underground legend. Freestyle Fellowship's most technically gifted MC.</t>
         </is>
       </c>
     </row>
@@ -6677,9 +6597,8 @@
       <c r="N82" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O82" s="6">
-        <f>AVERAGE(J82:N82)</f>
-        <v/>
+      <c r="O82" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P82" s="7" t="inlineStr">
         <is>
@@ -6689,7 +6608,7 @@
       <c r="Q82" s="2" t="inlineStr"/>
       <c r="R82" s="2" t="inlineStr">
         <is>
-          <t>Only Built 4 Cuban Linx. Mafioso rap as cinematic epic.</t>
+          <t>'Only Built 4 Cuban Linx' — the Godfather Part II of rap albums.</t>
         </is>
       </c>
     </row>
@@ -6750,9 +6669,8 @@
       <c r="N83" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O83" s="6">
-        <f>AVERAGE(J83:N83)</f>
-        <v/>
+      <c r="O83" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P83" s="7" t="inlineStr">
         <is>
@@ -6762,7 +6680,7 @@
       <c r="Q83" s="2" t="inlineStr"/>
       <c r="R83" s="2" t="inlineStr">
         <is>
-          <t>Fantastic Damage. Dystopian industrial rap from the Def Jux era.</t>
+          <t>Company Flow / Run The Jewels architect. Dystopian sonic vision.</t>
         </is>
       </c>
     </row>
@@ -6823,9 +6741,8 @@
       <c r="N84" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O84" s="6">
-        <f>AVERAGE(J84:N84)</f>
-        <v/>
+      <c r="O84" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P84" s="14" t="inlineStr">
         <is>
@@ -6839,7 +6756,7 @@
       </c>
       <c r="R84" s="2" t="inlineStr">
         <is>
-          <t>Shadows on the Sun. Minneapolis underground social conscience.</t>
+          <t>Minneapolis conscious rapper. Raw emotional honesty over Ant's production.</t>
         </is>
       </c>
     </row>
@@ -6900,9 +6817,8 @@
       <c r="N85" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="O85" s="6">
-        <f>AVERAGE(J85:N85)</f>
-        <v/>
+      <c r="O85" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P85" s="14" t="inlineStr">
         <is>
@@ -6916,7 +6832,7 @@
       </c>
       <c r="R85" s="2" t="inlineStr">
         <is>
-          <t>Revolutionary Vol. 2. Conspiracy rap with genuine rhetorical force.</t>
+          <t>Most politically radical rapper in the genre. Conspiracy and revolution.</t>
         </is>
       </c>
     </row>
@@ -6977,9 +6893,8 @@
       <c r="N86" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="O86" s="6">
-        <f>AVERAGE(J86:N86)</f>
-        <v/>
+      <c r="O86" s="6" t="n">
+        <v>10</v>
       </c>
       <c r="P86" s="7" t="inlineStr">
         <is>
@@ -6989,7 +6904,7 @@
       <c r="Q86" s="2" t="inlineStr"/>
       <c r="R86" s="2" t="inlineStr">
         <is>
-          <t>good kid m.A.A.d city / TPAB. The most complete MC since Nas.</t>
+          <t>The complete package. Every dimension at peak. Pulitzer Prize.</t>
         </is>
       </c>
     </row>
@@ -7050,9 +6965,8 @@
       <c r="N87" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O87" s="6">
-        <f>AVERAGE(J87:N87)</f>
-        <v/>
+      <c r="O87" s="6" t="n">
+        <v>6.4</v>
       </c>
       <c r="P87" s="7" t="inlineStr">
         <is>
@@ -7062,7 +6976,7 @@
       <c r="Q87" s="2" t="inlineStr"/>
       <c r="R87" s="2" t="inlineStr">
         <is>
-          <t>Take Care. Emotional rap at massive commercial scale.</t>
+          <t>Emotional candor and commercial dominance. Lyricism secondary to feeling.</t>
         </is>
       </c>
     </row>
@@ -7123,9 +7037,8 @@
       <c r="N88" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O88" s="6">
-        <f>AVERAGE(J88:N88)</f>
-        <v/>
+      <c r="O88" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P88" s="7" t="inlineStr">
         <is>
@@ -7135,7 +7048,7 @@
       <c r="Q88" s="2" t="inlineStr"/>
       <c r="R88" s="2" t="inlineStr">
         <is>
-          <t>2014 Forest Hills Drive. Self-produced introspection at scale.</t>
+          <t>Working-class emotional intelligence. Deep narrative craft.</t>
         </is>
       </c>
     </row>
@@ -7196,9 +7109,8 @@
       <c r="N89" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O89" s="6">
-        <f>AVERAGE(J89:N89)</f>
-        <v/>
+      <c r="O89" s="6" t="n">
+        <v>5.2</v>
       </c>
       <c r="P89" s="7" t="inlineStr">
         <is>
@@ -7208,7 +7120,7 @@
       <c r="Q89" s="2" t="inlineStr"/>
       <c r="R89" s="2" t="inlineStr">
         <is>
-          <t>Barter 6. Recontextualized flow as melodic instrument.</t>
+          <t>Melody over meaning. Vocal texture as primary instrument.</t>
         </is>
       </c>
     </row>
@@ -7269,9 +7181,8 @@
       <c r="N90" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O90" s="6">
-        <f>AVERAGE(J90:N90)</f>
-        <v/>
+      <c r="O90" s="6" t="n">
+        <v>5.2</v>
       </c>
       <c r="P90" s="7" t="inlineStr">
         <is>
@@ -7281,7 +7192,7 @@
       <c r="Q90" s="2" t="inlineStr"/>
       <c r="R90" s="2" t="inlineStr">
         <is>
-          <t>DS2. Emotional ambivalence as trap subgenre.</t>
+          <t>Emotional auto-tune as confession. Vibe over lyrical architecture.</t>
         </is>
       </c>
     </row>
@@ -7342,9 +7253,8 @@
       <c r="N91" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O91" s="6">
-        <f>AVERAGE(J91:N91)</f>
-        <v/>
+      <c r="O91" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P91" s="7" t="inlineStr">
         <is>
@@ -7354,7 +7264,7 @@
       <c r="Q91" s="2" t="inlineStr"/>
       <c r="R91" s="2" t="inlineStr">
         <is>
-          <t>Coloring Book. Gospel rap from Chicago's south side.</t>
+          <t>Joyful complexity. Gospel cadences and Chicago love letters.</t>
         </is>
       </c>
     </row>
@@ -7415,9 +7325,8 @@
       <c r="N92" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O92" s="6">
-        <f>AVERAGE(J92:N92)</f>
-        <v/>
+      <c r="O92" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P92" s="7" t="inlineStr">
         <is>
@@ -7427,7 +7336,7 @@
       <c r="Q92" s="2" t="inlineStr"/>
       <c r="R92" s="2" t="inlineStr">
         <is>
-          <t>I Don't Like Shit. Dense, interior, self-lacerating.</t>
+          <t>Compression and grief as poetics. Dense abstract imagery.</t>
         </is>
       </c>
     </row>
@@ -7488,9 +7397,8 @@
       <c r="N93" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O93" s="6">
-        <f>AVERAGE(J93:N93)</f>
-        <v/>
+      <c r="O93" s="6" t="n">
+        <v>6.2</v>
       </c>
       <c r="P93" s="7" t="inlineStr">
         <is>
@@ -7500,7 +7408,7 @@
       <c r="Q93" s="2" t="inlineStr"/>
       <c r="R93" s="2" t="inlineStr">
         <is>
-          <t>Dreams and Nightmares. Philly grit at arena scale.</t>
+          <t>Visceral urgency. Philadelphia streets in raw kinetic delivery.</t>
         </is>
       </c>
     </row>
@@ -7561,9 +7469,8 @@
       <c r="N94" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O94" s="6">
-        <f>AVERAGE(J94:N94)</f>
-        <v/>
+      <c r="O94" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="P94" s="7" t="inlineStr">
         <is>
@@ -7573,7 +7480,7 @@
       <c r="Q94" s="2" t="inlineStr"/>
       <c r="R94" s="2" t="inlineStr">
         <is>
-          <t>Long.Live.ASAP. Harlem avant-garde aesthetics in rap form.</t>
+          <t>Aesthetic as content. Flow and texture over lyrical substance.</t>
         </is>
       </c>
     </row>
@@ -7634,9 +7541,8 @@
       <c r="N95" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O95" s="6">
-        <f>AVERAGE(J95:N95)</f>
-        <v/>
+      <c r="O95" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P95" s="7" t="inlineStr">
         <is>
@@ -7646,7 +7552,7 @@
       <c r="Q95" s="2" t="inlineStr"/>
       <c r="R95" s="2" t="inlineStr">
         <is>
-          <t>Pink Friday. Technical bars meet pop domination.</t>
+          <t>Technical precision and alter-ego theatrics. 'Monster' verse.</t>
         </is>
       </c>
     </row>
@@ -7707,9 +7613,8 @@
       <c r="N96" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O96" s="6">
-        <f>AVERAGE(J96:N96)</f>
-        <v/>
+      <c r="O96" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P96" s="7" t="inlineStr">
         <is>
@@ -7719,7 +7624,7 @@
       <c r="Q96" s="2" t="inlineStr"/>
       <c r="R96" s="2" t="inlineStr">
         <is>
-          <t>Summertime '06. Long Beach noir, economical and bleak.</t>
+          <t>Deadpan sociologist. Minimalist language doing maximum structural work.</t>
         </is>
       </c>
     </row>
@@ -7780,9 +7685,8 @@
       <c r="N97" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O97" s="6">
-        <f>AVERAGE(J97:N97)</f>
-        <v/>
+      <c r="O97" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P97" s="7" t="inlineStr">
         <is>
@@ -7792,7 +7696,7 @@
       <c r="Q97" s="2" t="inlineStr"/>
       <c r="R97" s="2" t="inlineStr">
         <is>
-          <t>Live from the Underground. Southern rap's self-produced soul heir.</t>
+          <t>Mississippi throwback futurist. Southern soul and lyrical ambition fused.</t>
         </is>
       </c>
     </row>
@@ -7853,9 +7757,8 @@
       <c r="N98" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O98" s="6">
-        <f>AVERAGE(J98:N98)</f>
-        <v/>
+      <c r="O98" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P98" s="7" t="inlineStr">
         <is>
@@ -7865,7 +7768,7 @@
       <c r="Q98" s="2" t="inlineStr"/>
       <c r="R98" s="2" t="inlineStr">
         <is>
-          <t>RTJ2. El-P + Killer Mike = relentless political rap.</t>
+          <t>El-P and Killer Mike. Most politically urgent rap duo since PE.</t>
         </is>
       </c>
     </row>
@@ -7926,9 +7829,8 @@
       <c r="N99" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O99" s="6">
-        <f>AVERAGE(J99:N99)</f>
-        <v/>
+      <c r="O99" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P99" s="7" t="inlineStr">
         <is>
@@ -7938,7 +7840,7 @@
       <c r="Q99" s="2" t="inlineStr"/>
       <c r="R99" s="2" t="inlineStr">
         <is>
-          <t>R.A.P. Music. Atlanta social critique at its angriest best.</t>
+          <t>RTJ's political conscience. Atlanta's most morally serious MC.</t>
         </is>
       </c>
     </row>
@@ -7999,9 +7901,8 @@
       <c r="N100" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="O100" s="6">
-        <f>AVERAGE(J100:N100)</f>
-        <v/>
+      <c r="O100" s="6" t="n">
+        <v>3.8</v>
       </c>
       <c r="P100" s="7" t="inlineStr">
         <is>
@@ -8011,7 +7912,7 @@
       <c r="Q100" s="2" t="inlineStr"/>
       <c r="R100" s="2" t="inlineStr">
         <is>
-          <t>Fancy. Commercial peak; authenticity debates dominated reception.</t>
+          <t>Commercial success masking thin lyrical foundation. Accent controversy.</t>
         </is>
       </c>
     </row>
@@ -8072,9 +7973,8 @@
       <c r="N101" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O101" s="6">
-        <f>AVERAGE(J101:N101)</f>
-        <v/>
+      <c r="O101" s="6" t="n">
+        <v>7.8</v>
       </c>
       <c r="P101" s="7" t="inlineStr">
         <is>
@@ -8084,7 +7984,7 @@
       <c r="Q101" s="2" t="inlineStr"/>
       <c r="R101" s="2" t="inlineStr">
         <is>
-          <t>Piñata. Madlib collab reinvented his career and the genre.</t>
+          <t>Gary Indiana's finest. Technical gangsta rap with jazz-rap production.</t>
         </is>
       </c>
     </row>
@@ -8145,9 +8045,8 @@
       <c r="N102" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="O102" s="6">
-        <f>AVERAGE(J102:N102)</f>
-        <v/>
+      <c r="O102" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="P102" s="7" t="inlineStr">
         <is>
@@ -8157,7 +8056,7 @@
       <c r="Q102" s="2" t="inlineStr"/>
       <c r="R102" s="2" t="inlineStr">
         <is>
-          <t>Culture. Triplet flow codified an era; lyricism secondary.</t>
+          <t>Triplet flow inventors. Cultural influence far exceeds lyrical complexity.</t>
         </is>
       </c>
     </row>
@@ -8218,9 +8117,8 @@
       <c r="N103" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O103" s="6">
-        <f>AVERAGE(J103:N103)</f>
-        <v/>
+      <c r="O103" s="6" t="n">
+        <v>5.8</v>
       </c>
       <c r="P103" s="14" t="inlineStr">
         <is>
@@ -8234,7 +8132,7 @@
       </c>
       <c r="R103" s="2" t="inlineStr">
         <is>
-          <t>I Decided. Catchy rap with occasional lyrical ambition.</t>
+          <t>Detroit MC. Punchlines over conceptual depth. 'One Man Can Change The World'.</t>
         </is>
       </c>
     </row>
@@ -8295,9 +8193,8 @@
       <c r="N104" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O104" s="6">
-        <f>AVERAGE(J104:N104)</f>
-        <v/>
+      <c r="O104" s="6" t="n">
+        <v>7.6</v>
       </c>
       <c r="P104" s="14" t="inlineStr">
         <is>
@@ -8311,7 +8208,7 @@
       </c>
       <c r="R104" s="2" t="inlineStr">
         <is>
-          <t>Whack World. 15 one-minute songs as conceptual art project.</t>
+          <t>'Whack World' — 15 one-minute songs as unified concept. Wholly original.</t>
         </is>
       </c>
     </row>
@@ -8372,9 +8269,8 @@
       <c r="N105" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O105" s="6">
-        <f>AVERAGE(J105:N105)</f>
-        <v/>
+      <c r="O105" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P105" s="7" t="inlineStr">
         <is>
@@ -8384,7 +8280,7 @@
       <c r="Q105" s="2" t="inlineStr"/>
       <c r="R105" s="2" t="inlineStr">
         <is>
-          <t>Room 25. Quiet devastation over jazz loops.</t>
+          <t>Chicago's most literary voice. Jazz cadences and political awakening.</t>
         </is>
       </c>
     </row>
@@ -8445,9 +8341,8 @@
       <c r="N106" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O106" s="6">
-        <f>AVERAGE(J106:N106)</f>
-        <v/>
+      <c r="O106" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P106" s="7" t="inlineStr">
         <is>
@@ -8457,7 +8352,7 @@
       <c r="Q106" s="2" t="inlineStr"/>
       <c r="R106" s="2" t="inlineStr">
         <is>
-          <t>CARE FOR ME. Grief album as Chicago hip-hop masterpiece.</t>
+          <t>'CARE FOR ME' — grief and Chicago violence as devastating concept album.</t>
         </is>
       </c>
     </row>
@@ -8518,9 +8413,8 @@
       <c r="N107" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O107" s="6">
-        <f>AVERAGE(J107:N107)</f>
-        <v/>
+      <c r="O107" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P107" s="7" t="inlineStr">
         <is>
@@ -8530,7 +8424,7 @@
       <c r="Q107" s="2" t="inlineStr"/>
       <c r="R107" s="2" t="inlineStr">
         <is>
-          <t>Atrocity Exhibition. Detroit's answer to post-punk sonic chaos.</t>
+          <t>Detroit's avant-garde MC. Schizophrenic flows and surreal imagery.</t>
         </is>
       </c>
     </row>
@@ -8591,9 +8485,8 @@
       <c r="N108" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O108" s="6">
-        <f>AVERAGE(J108:N108)</f>
-        <v/>
+      <c r="O108" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P108" s="7" t="inlineStr">
         <is>
@@ -8603,7 +8496,7 @@
       <c r="Q108" s="2" t="inlineStr"/>
       <c r="R108" s="2" t="inlineStr">
         <is>
-          <t>Swimming. Self-medication turned into heartbreaking art.</t>
+          <t>Arc from frat-rap to deeply personal jazz introspection. 'Swimming' a peak.</t>
         </is>
       </c>
     </row>
@@ -8664,9 +8557,8 @@
       <c r="N109" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O109" s="6">
-        <f>AVERAGE(J109:N109)</f>
-        <v/>
+      <c r="O109" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P109" s="14" t="inlineStr">
         <is>
@@ -8680,7 +8572,7 @@
       </c>
       <c r="R109" s="2" t="inlineStr">
         <is>
-          <t>DiCaprio 2. Switchable flow at a pace few can match.</t>
+          <t>Atlanta's most technically gifted rapper. 'DiCaprio 2' showed full potential.</t>
         </is>
       </c>
     </row>
@@ -8741,9 +8633,8 @@
       <c r="N110" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O110" s="6">
-        <f>AVERAGE(J110:N110)</f>
-        <v/>
+      <c r="O110" s="6" t="n">
+        <v>5.6</v>
       </c>
       <c r="P110" s="7" t="inlineStr">
         <is>
@@ -8753,7 +8644,7 @@
       <c r="Q110" s="2" t="inlineStr"/>
       <c r="R110" s="2" t="inlineStr">
         <is>
-          <t>Invasion of Privacy. Bronx bravado at Grammys level.</t>
+          <t>Unfiltered Bronx personality. Cultural force exceeds lyrical architecture.</t>
         </is>
       </c>
     </row>
@@ -8814,9 +8705,8 @@
       <c r="N111" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O111" s="6">
-        <f>AVERAGE(J111:N111)</f>
-        <v/>
+      <c r="O111" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P111" s="14" t="inlineStr">
         <is>
@@ -8830,7 +8720,7 @@
       </c>
       <c r="R111" s="2" t="inlineStr">
         <is>
-          <t>Pop Out. Melancholy Chicago trap with genuine lyrical care.</t>
+          <t>Chicago's introspective melodic trap voice. Melancholy street memoir.</t>
         </is>
       </c>
     </row>
@@ -8891,9 +8781,8 @@
       <c r="N112" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O112" s="6">
-        <f>AVERAGE(J112:N112)</f>
-        <v/>
+      <c r="O112" s="6" t="n">
+        <v>5.6</v>
       </c>
       <c r="P112" s="14" t="inlineStr">
         <is>
@@ -8907,7 +8796,7 @@
       </c>
       <c r="R112" s="2" t="inlineStr">
         <is>
-          <t>SoulFly. Florida's emotional trap meets gospel music.</t>
+          <t>Emotional vulnerability over technical precision. Florida pain made universal.</t>
         </is>
       </c>
     </row>
@@ -8968,9 +8857,8 @@
       <c r="N113" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O113" s="6">
-        <f>AVERAGE(J113:N113)</f>
-        <v/>
+      <c r="O113" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P113" s="14" t="inlineStr">
         <is>
@@ -8984,7 +8872,7 @@
       </c>
       <c r="R113" s="2" t="inlineStr">
         <is>
-          <t>Alligator Bites Never Heal. Tampa avant-garde challenging rap norms.</t>
+          <t>Tampa's theatrical polymath. Technical fire meets conceptual daring.</t>
         </is>
       </c>
     </row>
@@ -9045,9 +8933,8 @@
       <c r="N114" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O114" s="6">
-        <f>AVERAGE(J114:N114)</f>
-        <v/>
+      <c r="O114" s="6" t="n">
+        <v>4.8</v>
       </c>
       <c r="P114" s="15" t="inlineStr">
         <is>
@@ -9061,7 +8948,7 @@
       </c>
       <c r="R114" s="2" t="inlineStr">
         <is>
-          <t>FNF. Memphis energy with instant cultural resonance.</t>
+          <t>Memphis energy, unfiltered personality. New Southern feminism in party form.</t>
         </is>
       </c>
     </row>
@@ -9122,9 +9009,8 @@
       <c r="N115" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="O115" s="6">
-        <f>AVERAGE(J115:N115)</f>
-        <v/>
+      <c r="O115" s="6" t="n">
+        <v>4.2</v>
       </c>
       <c r="P115" s="14" t="inlineStr">
         <is>
@@ -9138,7 +9024,7 @@
       </c>
       <c r="R115" s="2" t="inlineStr">
         <is>
-          <t>DS4EVER. Melodic trap comfort zone never pushed.</t>
+          <t>Melodic luxury trap. Vibe and aesthetic are the art.</t>
         </is>
       </c>
     </row>
@@ -9199,9 +9085,8 @@
       <c r="N116" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O116" s="6">
-        <f>AVERAGE(J116:N116)</f>
-        <v/>
+      <c r="O116" s="6" t="n">
+        <v>5.2</v>
       </c>
       <c r="P116" s="14" t="inlineStr">
         <is>
@@ -9215,7 +9100,7 @@
       </c>
       <c r="R116" s="2" t="inlineStr">
         <is>
-          <t>My Turn. Effortless commercial dominance; artistry developing.</t>
+          <t>Authentic street narrator. Storytelling grounded in lived experience.</t>
         </is>
       </c>
     </row>
@@ -9276,9 +9161,8 @@
       <c r="N117" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O117" s="6">
-        <f>AVERAGE(J117:N117)</f>
-        <v/>
+      <c r="O117" s="6" t="n">
+        <v>8</v>
       </c>
       <c r="P117" s="7" t="inlineStr">
         <is>
@@ -9288,7 +9172,7 @@
       <c r="Q117" s="2" t="inlineStr"/>
       <c r="R117" s="2" t="inlineStr">
         <is>
-          <t>Burden of Proof. Griselda's street pulpit.</t>
+          <t>Griselda's lyrical backbone. Buffalo street narratives with East Coast precision.</t>
         </is>
       </c>
     </row>
@@ -9349,9 +9233,8 @@
       <c r="N118" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O118" s="6">
-        <f>AVERAGE(J118:N118)</f>
-        <v/>
+      <c r="O118" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P118" s="7" t="inlineStr">
         <is>
@@ -9361,7 +9244,7 @@
       <c r="Q118" s="2" t="inlineStr"/>
       <c r="R118" s="2" t="inlineStr">
         <is>
-          <t>Heavy Is the Head. UK grime at Glastonbury scale.</t>
+          <t>UK grime's political conscience. Authenticity and ambition fused.</t>
         </is>
       </c>
     </row>
@@ -9422,9 +9305,8 @@
       <c r="N119" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O119" s="6">
-        <f>AVERAGE(J119:N119)</f>
-        <v/>
+      <c r="O119" s="6" t="n">
+        <v>5.8</v>
       </c>
       <c r="P119" s="14" t="inlineStr">
         <is>
@@ -9438,7 +9320,7 @@
       </c>
       <c r="R119" s="2" t="inlineStr">
         <is>
-          <t>Un Verano Sin Ti. Latin trap global domination.</t>
+          <t>Global Latin trap superstar. Reframed what non-English rap could achieve commercially.</t>
         </is>
       </c>
     </row>
@@ -9499,9 +9381,8 @@
       <c r="N120" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O120" s="6">
-        <f>AVERAGE(J120:N120)</f>
-        <v/>
+      <c r="O120" s="6" t="n">
+        <v>4.4</v>
       </c>
       <c r="P120" s="15" t="inlineStr">
         <is>
@@ -9515,7 +9396,7 @@
       </c>
       <c r="R120" s="2" t="inlineStr">
         <is>
-          <t>Colores. Reggaeton popstar with rap adjacency.</t>
+          <t>Reggaeton crossover king. Melody and production far exceed lyrical content.</t>
         </is>
       </c>
     </row>
@@ -9576,9 +9457,8 @@
       <c r="N121" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O121" s="6">
-        <f>AVERAGE(J121:N121)</f>
-        <v/>
+      <c r="O121" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="P121" s="14" t="inlineStr">
         <is>
@@ -9592,7 +9472,7 @@
       </c>
       <c r="R121" s="2" t="inlineStr">
         <is>
-          <t>Set It Off. Post-Migos identity search ongoing.</t>
+          <t>Migos' most lyrical member. Flow variation and delivery standout in trap context.</t>
         </is>
       </c>
     </row>
@@ -9653,9 +9533,8 @@
       <c r="N122" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O122" s="6">
-        <f>AVERAGE(J122:N122)</f>
-        <v/>
+      <c r="O122" s="6" t="n">
+        <v>7</v>
       </c>
       <c r="P122" s="15" t="inlineStr">
         <is>
@@ -9669,7 +9548,7 @@
       </c>
       <c r="R122" s="2" t="inlineStr">
         <is>
-          <t>Angelic Hoodrat. Atlanta experimental underground at its weirdest.</t>
+          <t>Atlanta's punk-rap hybrid. Unconventional tonal range.</t>
         </is>
       </c>
     </row>
@@ -9730,9 +9609,8 @@
       <c r="N123" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O123" s="6">
-        <f>AVERAGE(J123:N123)</f>
-        <v/>
+      <c r="O123" s="6" t="n">
+        <v>5.8</v>
       </c>
       <c r="P123" s="14" t="inlineStr">
         <is>
@@ -9746,7 +9624,7 @@
       </c>
       <c r="R123" s="2" t="inlineStr">
         <is>
-          <t>777. Southern female rap following Cardi and Nicki's path.</t>
+          <t>Atlanta's female trap voice. Technical skill often underestimated.</t>
         </is>
       </c>
     </row>
@@ -9807,9 +9685,8 @@
       <c r="N124" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O124" s="6">
-        <f>AVERAGE(J124:N124)</f>
-        <v/>
+      <c r="O124" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P124" s="14" t="inlineStr">
         <is>
@@ -9823,7 +9700,7 @@
       </c>
       <c r="R124" s="2" t="inlineStr">
         <is>
-          <t>blkswn. Jazz-rap from St. Louis with melodic depth.</t>
+          <t>St. Louis's jazz-rap hybrid. Melodic and rhythmic sophistication.</t>
         </is>
       </c>
     </row>
@@ -9884,9 +9761,8 @@
       <c r="N125" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O125" s="6">
-        <f>AVERAGE(J125:N125)</f>
-        <v/>
+      <c r="O125" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P125" s="7" t="inlineStr">
         <is>
@@ -9896,7 +9772,7 @@
       <c r="Q125" s="2" t="inlineStr"/>
       <c r="R125" s="2" t="inlineStr">
         <is>
-          <t>It's Almost Dry. Coke rap as high art. Pharrell and Kanye dual production.</t>
+          <t>Cocaine rap's Rembrandt. 'Daytona' — maximum density, minimum waste.</t>
         </is>
       </c>
     </row>
@@ -9957,9 +9833,8 @@
       <c r="N126" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O126" s="6">
-        <f>AVERAGE(J126:N126)</f>
-        <v/>
+      <c r="O126" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P126" s="14" t="inlineStr">
         <is>
@@ -9973,7 +9848,7 @@
       </c>
       <c r="R126" s="2" t="inlineStr">
         <is>
-          <t>The Never Story / Pandemonium!. Technical rapper escaping Atlanta tropes.</t>
+          <t>Atlanta's most technically gifted. 'The Never Story' showed generational talent.</t>
         </is>
       </c>
     </row>
@@ -10034,9 +9909,8 @@
       <c r="N127" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O127" s="6">
-        <f>AVERAGE(J127:N127)</f>
-        <v/>
+      <c r="O127" s="6" t="n">
+        <v>8.4</v>
       </c>
       <c r="P127" s="7" t="inlineStr">
         <is>
@@ -10046,7 +9920,7 @@
       <c r="Q127" s="2" t="inlineStr"/>
       <c r="R127" s="2" t="inlineStr">
         <is>
-          <t>Igor / Call Me If You Get Lost. Conceptual album art as rap.</t>
+          <t>'Igor' and 'Call Me If You Get Lost' — producer-auteur. Concept album mastery.</t>
         </is>
       </c>
     </row>
@@ -10107,9 +9981,8 @@
       <c r="N128" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O128" s="6">
-        <f>AVERAGE(J128:N128)</f>
-        <v/>
+      <c r="O128" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P128" s="14" t="inlineStr">
         <is>
@@ -10123,7 +9996,7 @@
       </c>
       <c r="R128" s="2" t="inlineStr">
         <is>
-          <t>Haram. billy woods + ELUCID: dense, allusive, uncompromising.</t>
+          <t>billy woods + ELUCID. The most demanding abstract rap being made today.</t>
         </is>
       </c>
     </row>
@@ -10184,9 +10057,8 @@
       <c r="N129" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O129" s="6">
-        <f>AVERAGE(J129:N129)</f>
-        <v/>
+      <c r="O129" s="6" t="n">
+        <v>6.4</v>
       </c>
       <c r="P129" s="15" t="inlineStr">
         <is>
@@ -10200,7 +10072,7 @@
       </c>
       <c r="R129" s="2" t="inlineStr">
         <is>
-          <t>Bussin. Internet-native absurdist rapper with genuine lyrical wit.</t>
+          <t>Comedy-meets-rap. Formally interesting but body of work too small to score confidently.</t>
         </is>
       </c>
     </row>
@@ -10261,9 +10133,8 @@
       <c r="N130" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="O130" s="6">
-        <f>AVERAGE(J130:N130)</f>
-        <v/>
+      <c r="O130" s="6" t="n">
+        <v>5.2</v>
       </c>
       <c r="P130" s="14" t="inlineStr">
         <is>
@@ -10277,7 +10148,7 @@
       </c>
       <c r="R130" s="2" t="inlineStr">
         <is>
-          <t>The Voice. Chicago melodic trap emotional authenticity at scale.</t>
+          <t>Chicago drill's most commercially consistent voice.</t>
         </is>
       </c>
     </row>
@@ -10338,9 +10209,8 @@
       <c r="N131" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O131" s="6">
-        <f>AVERAGE(J131:N131)</f>
-        <v/>
+      <c r="O131" s="6" t="n">
+        <v>5</v>
       </c>
       <c r="P131" s="14" t="inlineStr">
         <is>
@@ -10354,7 +10224,7 @@
       </c>
       <c r="R131" s="2" t="inlineStr">
         <is>
-          <t>Project Baby. Florida trap originality clouded by off-mic controversies.</t>
+          <t>Florida trap's most distinctive voice. Rough-edged regional authenticity.</t>
         </is>
       </c>
     </row>
@@ -10415,9 +10285,8 @@
       <c r="N132" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O132" s="6">
-        <f>AVERAGE(J132:N132)</f>
-        <v/>
+      <c r="O132" s="6" t="n">
+        <v>6.6</v>
       </c>
       <c r="P132" s="15" t="inlineStr">
         <is>
@@ -10431,7 +10300,7 @@
       </c>
       <c r="R132" s="2" t="inlineStr">
         <is>
-          <t>Por Vida. Colombian-American bilingual artistry; rap adjacent.</t>
+          <t>Colombian-American crossover. When rapping, brings genuine bilingual lyricism.</t>
         </is>
       </c>
     </row>
@@ -10492,9 +10361,8 @@
       <c r="N133" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="O133" s="6">
-        <f>AVERAGE(J133:N133)</f>
-        <v/>
+      <c r="O133" s="6" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="P133" s="7" t="inlineStr">
         <is>
@@ -10504,7 +10372,7 @@
       <c r="Q133" s="2" t="inlineStr"/>
       <c r="R133" s="2" t="inlineStr">
         <is>
-          <t>Eve. Named every track after a Black woman. Precision and purpose.</t>
+          <t>North Carolina's most complete female MC. Lyrical depth rivals any peer.</t>
         </is>
       </c>
     </row>
@@ -10565,9 +10433,8 @@
       <c r="N134" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="O134" s="6">
-        <f>AVERAGE(J134:N134)</f>
-        <v/>
+      <c r="O134" s="6" t="n">
+        <v>8.6</v>
       </c>
       <c r="P134" s="14" t="inlineStr">
         <is>
@@ -10581,7 +10448,7 @@
       </c>
       <c r="R134" s="2" t="inlineStr">
         <is>
-          <t>Factory Baby. Post-Room 25 political radicalization era.</t>
+          <t>Noname's political radicalization phase. Most conceptually ambitious output.</t>
         </is>
       </c>
     </row>
@@ -10642,9 +10509,8 @@
       <c r="N135" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O135" s="6">
-        <f>AVERAGE(J135:N135)</f>
-        <v/>
+      <c r="O135" s="6" t="n">
+        <v>7.2</v>
       </c>
       <c r="P135" s="15" t="inlineStr">
         <is>
@@ -10658,7 +10524,7 @@
       </c>
       <c r="R135" s="2" t="inlineStr">
         <is>
-          <t>Let the Sun Talk. Introspective underground debut with cultish following.</t>
+          <t>Charlotte underground. Dense introspective abstract rap. Watch this space.</t>
         </is>
       </c>
     </row>
@@ -10719,9 +10585,8 @@
       <c r="N136" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="O136" s="6">
-        <f>AVERAGE(J136:N136)</f>
-        <v/>
+      <c r="O136" s="6" t="n">
+        <v>6.8</v>
       </c>
       <c r="P136" s="14" t="inlineStr">
         <is>
@@ -10735,7 +10600,7 @@
       </c>
       <c r="R136" s="2" t="inlineStr">
         <is>
-          <t>At the Speed of Life. West Coast boom bap craftsman.</t>
+          <t>West Coast boom bap craftsman. More respected by peers than critics.</t>
         </is>
       </c>
     </row>
@@ -10796,9 +10661,8 @@
       <c r="N137" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O137" s="6">
-        <f>AVERAGE(J137:N137)</f>
-        <v/>
+      <c r="O137" s="6" t="n">
+        <v>4.8</v>
       </c>
       <c r="P137" s="14" t="inlineStr">
         <is>
@@ -10812,7 +10676,7 @@
       </c>
       <c r="R137" s="2" t="inlineStr">
         <is>
-          <t>Pretty Summer Playlist. Bay Area trap-pop aesthetic.</t>
+          <t>Bay Area trap-pop. Ice Princess persona over lyrical substance.</t>
         </is>
       </c>
     </row>
@@ -10873,9 +10737,8 @@
       <c r="N138" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="O138" s="6">
-        <f>AVERAGE(J138:N138)</f>
-        <v/>
+      <c r="O138" s="6" t="n">
+        <v>4.6</v>
       </c>
       <c r="P138" s="15" t="inlineStr">
         <is>
@@ -10889,7 +10752,7 @@
       </c>
       <c r="R138" s="2" t="inlineStr">
         <is>
-          <t>Period. Miami hedonistic party rap duo.</t>
+          <t>Miami's hedonistic party rap duo. Energy over craft.</t>
         </is>
       </c>
     </row>
@@ -10950,9 +10813,8 @@
       <c r="N139" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="O139" s="6">
-        <f>AVERAGE(J139:N139)</f>
-        <v/>
+      <c r="O139" s="6" t="n">
+        <v>7.4</v>
       </c>
       <c r="P139" s="14" t="inlineStr">
         <is>
@@ -10966,7 +10828,7 @@
       </c>
       <c r="R139" s="2" t="inlineStr">
         <is>
-          <t>Weight of the World. Houston storytelling tradition continued.</t>
+          <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
         </is>
       </c>
     </row>
@@ -11027,9 +10889,8 @@
       <c r="N140" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="O140" s="6">
-        <f>AVERAGE(J140:N140)</f>
-        <v/>
+      <c r="O140" s="6" t="n">
+        <v>7.6</v>
       </c>
       <c r="P140" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Consolidate hip-hop data into a single source of truth
- hiphop_artists.xlsx is now the only data file, with two sheets:
  - "Artist Database" (authoritative data the site builds from)
  - "Confidence Guide" (folded in from the old 5-dimension workbook:
    scoring methodology, known biases, verification sources)
- Remove redundant HipHop_150_5Dim.xlsx. Its richer descriptions and
  composites were already merged into Artist Database last commit; its
  derived Top 30 / Era-Averages snapshots are dropped (regenerable on
  demand, and would go stale during data edits)
- Update build_table.R header comment to document the single-file layout

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Artist Database" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Confidence Guide" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Artist Database'!$A$1:$R$1</definedName>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,6 +71,9 @@
       <b val="1"/>
       <color rgb="009C0006"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="15">
@@ -157,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -203,6 +207,13 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10912,4 +10923,161 @@
   <autoFilter ref="A1:R1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Scoring Confidence Flag Guide</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>Criteria for assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>H — High</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Extensive critical record</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Artist has: (1) sustained critical and/or academic attention, (2) multiple long-form critical analyses of their lyrical craft, (3) consistent reception across multiple sources, (4) enough body of work that scores are stable across albums. Examples: Rakim, Nas, Eminem, Kendrick, Biggie, Jay-Z.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>M — Medium</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Moderate documentation</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Artist meets 1–2 of the High criteria but not all. May be: historically significant but under-analyzed (e.g. MC Lyte), recently emergent with promising but incomplete body of work (e.g. J.I.D, Doechii), subject to contested or shifting critical reception, or significant in regional/underground circles without mainstream scholarly attention. Scores should be treated as provisional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>L — Low</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Thin or contested record</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Artist has: limited formal critical analysis, very recent emergence (insufficient time for consensus), scores that rely heavily on a single source or thin evidence base, reception clouded by non-lyrical controversy, or requires critical frameworks not well-developed in English-language sources (e.g. Latin rap, non-English artists). Scores marked L should be treated as initial estimates requiring verification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="C6" s="17" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>METHODOLOGICAL NOTES</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Scoring basis</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Critical consensus synthesis</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>All scores are derived from synthesis of published music criticism, academic hip-hop scholarship (Bradley, Chang, Kajikawa, Rabaka), and documented critical consensus. They are NOT computational — no NLP analysis was run. Aesop Rock is used as the Vocab Breadth=10 anchor based on published NLP studies of unique vocabulary in rap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Known biases</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Prestige / gender / language</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>The dataset over-represents: critically acclaimed artists vs commercially dominant ones; male artists (correcting); Golden Age NYC; English-language rap. Latin, African, and non-Anglophone rap are significantly underrepresented and scores for international artists should be treated with extra caution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Recommended verification</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>For each L- and M-flagged artist</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Cross-reference against: RateYourMusic critical consensus scores, Pitchfork / The Wire artist discography reviews, academic sources via Google Scholar ('artist name' + 'lyricism' or 'hip-hop'), genre-specific publications (The Source, XXL retrospectives, Passion of the Weiss).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Start accuracy pass: structural relabels + L/M worklist
- Relabel "Nas feat. AZ" -> "AZ" (symbol AZ): the row already scored AZ
  per its own note/description; this makes it a proper standalone entry
- Rename "Ghostface / Fishscale era" -> "Ghostface Killah"
- Rename "Yvonne (Yaya Bey)" -> "Yaya Bey"
- Add hiphop/data/accuracy_worklist.md: tracked checklist of the 12 L-
  and 42 M-confidence artists, plus pending structural decisions
  (JID/Noname duplicate merges, Kali Uchis & reggaeton inclusion,
  Schoolly D region)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -5093,12 +5093,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>NR</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Nas feat. AZ</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -5154,12 +5154,12 @@
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>AZ's solo career less documented than Nas; scored as AZ</t>
+          <t>Solo career less documented than Nas; scored on his own body of work.</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t>AZ: One of the most underrated MCs of the era. 'Sugarhill' an all-time verse.</t>
+          <t>One of the era's most underrated lyricists. 'Doe or Die' (1995) a classic; his 'Life's a Bitch' verse is all-time.</t>
         </is>
       </c>
     </row>
@@ -6038,7 +6038,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Ghostface / Fishscale era</t>
+          <t>Ghostface Killah</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="R75" s="2" t="inlineStr">
         <is>
-          <t>'Fishscale' is a 2000s apex. Singular stream-of-consciousness voice.</t>
+          <t>Wu-Tang's vivid storyteller; 'Fishscale' (2006) a stream-of-consciousness apex.</t>
         </is>
       </c>
     </row>
@@ -10854,7 +10854,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Yvonne (Yaya Bey)</t>
+          <t>Yaya Bey</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Resolve duplicates and narrow scope (139 -> 134 artists)
- Merge JID duplicate: keep #108 (renamed "J.I.D" -> "JID", 2010s),
  remove #125 (identical sub-scores, no data lost)
- Merge Noname duplicate: keep #104 (H-confidence canonical entry),
  remove #133 "Noname (Ghetto Sage)"
- Remove Kali Uchis, J Balvin, Bad Bunny (scope narrowing: primarily
  R&B / reggaeton, thin rap output)
- Renumber the # column sequentially 1..134
- Make the template artist counts dynamic (subtitle + "showing X of Y")
  so they derive from the data instead of a hardcoded 139
- Regenerate accuracy_worklist.md (now 10 L / 39 M / 85 H)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R140"/>
+  <dimension ref="A1:R135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8522,7 +8522,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>J.I.D</t>
+          <t>JID</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -9265,17 +9265,17 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>OM</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Bad Bunny</t>
+          <t>Offset</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -9285,39 +9285,39 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Trap/Drill</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Reggaeton/Latin Trap</t>
+          <t>Migos Solo Trap</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Rimas</t>
+          <t>Quality Control</t>
         </is>
       </c>
       <c r="I119" s="2" t="n">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="J119" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="K119" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L119" s="9" t="n">
-        <v>6</v>
+      <c r="K119" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L119" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="M119" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N119" s="9" t="n">
-        <v>6</v>
+      <c r="N119" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O119" s="6" t="n">
-        <v>5.8</v>
+        <v>5</v>
       </c>
       <c r="P119" s="14" t="inlineStr">
         <is>
@@ -9326,12 +9326,12 @@
       </c>
       <c r="Q119" s="2" t="inlineStr">
         <is>
-          <t>Massive influence on global rap; Spanish-language scoring requires different critical frame</t>
+          <t>Solo career emerging post-Migos; scoring tentative</t>
         </is>
       </c>
       <c r="R119" s="2" t="inlineStr">
         <is>
-          <t>Global Latin trap superstar. Reframed what non-English rap could achieve commercially.</t>
+          <t>Migos' most lyrical member. Flow variation and delivery standout in trap context.</t>
         </is>
       </c>
     </row>
@@ -9341,17 +9341,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>JB</t>
+          <t>KD</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>J Balvin</t>
+          <t>Kenny Mason</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -9361,39 +9361,39 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>Reggaeton</t>
+          <t>Atlanta Punk Rap</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Capitol</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="I120" s="2" t="n">
-        <v>2007</v>
-      </c>
-      <c r="J120" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K120" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L120" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M120" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N120" s="5" t="n">
-        <v>4</v>
+        <v>2019</v>
+      </c>
+      <c r="J120" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K120" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L120" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M120" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N120" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O120" s="6" t="n">
-        <v>4.4</v>
+        <v>7</v>
       </c>
       <c r="P120" s="15" t="inlineStr">
         <is>
@@ -9402,12 +9402,12 @@
       </c>
       <c r="Q120" s="2" t="inlineStr">
         <is>
-          <t>Minimal lyrical critical record; scored on available Spanish-language criticism</t>
+          <t>Limited documentation; critical buzz building in underground circles</t>
         </is>
       </c>
       <c r="R120" s="2" t="inlineStr">
         <is>
-          <t>Reggaeton crossover king. Melody and production far exceed lyrical content.</t>
+          <t>Atlanta's punk-rap hybrid. Unconventional tonal range.</t>
         </is>
       </c>
     </row>
@@ -9417,12 +9417,12 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>OM</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Offset</t>
+          <t>Latto</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -9437,39 +9437,39 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>Trap/Drill</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Migos Solo Trap</t>
+          <t>Atlanta Female Trap</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Quality Control</t>
+          <t>RCA</t>
         </is>
       </c>
       <c r="I121" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J121" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K121" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L121" s="8" t="n">
-        <v>5</v>
+        <v>2019</v>
+      </c>
+      <c r="J121" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K121" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L121" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="M121" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="N121" s="5" t="n">
-        <v>4</v>
+      <c r="N121" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="O121" s="6" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="P121" s="14" t="inlineStr">
         <is>
@@ -9478,12 +9478,12 @@
       </c>
       <c r="Q121" s="2" t="inlineStr">
         <is>
-          <t>Solo career emerging post-Migos; scoring tentative</t>
+          <t>Recent; commercial trajectory clearer than critical consensus</t>
         </is>
       </c>
       <c r="R121" s="2" t="inlineStr">
         <is>
-          <t>Migos' most lyrical member. Flow variation and delivery standout in trap context.</t>
+          <t>Atlanta's female trap voice. Technical skill often underestimated.</t>
         </is>
       </c>
     </row>
@@ -9493,17 +9493,17 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>KD</t>
+          <t>SR</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Kenny Mason</t>
+          <t>Smino</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -9518,48 +9518,48 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Punk Rap</t>
+          <t>St. Louis Jazz Rap</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Zero Fatigue</t>
         </is>
       </c>
       <c r="I122" s="2" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="J122" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="K122" s="10" t="n">
-        <v>7</v>
+      <c r="K122" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="L122" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="M122" s="10" t="n">
-        <v>7</v>
+      <c r="M122" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="N122" s="10" t="n">
         <v>7</v>
       </c>
       <c r="O122" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P122" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
+        <v>7.4</v>
+      </c>
+      <c r="P122" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="Q122" s="2" t="inlineStr">
         <is>
-          <t>Limited documentation; critical buzz building in underground circles</t>
+          <t>Critical darling in jazz-rap circles; broader recognition still forming</t>
         </is>
       </c>
       <c r="R122" s="2" t="inlineStr">
         <is>
-          <t>Atlanta's punk-rap hybrid. Unconventional tonal range.</t>
+          <t>St. Louis's jazz-rap hybrid. Melodic and rhythmic sophistication.</t>
         </is>
       </c>
     </row>
@@ -9569,17 +9569,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Latto</t>
+          <t>Pusha T</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -9594,48 +9594,44 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Female Trap</t>
+          <t>Coke Rap Boom Bap</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>RCA</t>
+          <t>G.O.O.D.</t>
         </is>
       </c>
       <c r="I123" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="J123" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K123" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L123" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M123" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N123" s="8" t="n">
-        <v>5</v>
+        <v>2002</v>
+      </c>
+      <c r="J123" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K123" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L123" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M123" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N123" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O123" s="6" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="P123" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q123" s="2" t="inlineStr">
-        <is>
-          <t>Recent; commercial trajectory clearer than critical consensus</t>
-        </is>
-      </c>
+        <v>7.4</v>
+      </c>
+      <c r="P123" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q123" s="2" t="inlineStr"/>
       <c r="R123" s="2" t="inlineStr">
         <is>
-          <t>Atlanta's female trap voice. Technical skill often underestimated.</t>
+          <t>Cocaine rap's Rembrandt. 'Daytona' — maximum density, minimum waste.</t>
         </is>
       </c>
     </row>
@@ -9645,17 +9641,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>TY</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Smino</t>
+          <t>Tyler the Creator</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -9670,48 +9666,44 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>St. Louis Jazz Rap</t>
+          <t>Odd Future/Orchestral</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Zero Fatigue</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="I124" s="2" t="n">
-        <v>2017</v>
+        <v>2009</v>
       </c>
       <c r="J124" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="K124" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L124" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M124" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N124" s="10" t="n">
-        <v>7</v>
+      <c r="K124" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="L124" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M124" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="N124" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="O124" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="P124" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q124" s="2" t="inlineStr">
-        <is>
-          <t>Critical darling in jazz-rap circles; broader recognition still forming</t>
-        </is>
-      </c>
+        <v>8.4</v>
+      </c>
+      <c r="P124" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q124" s="2" t="inlineStr"/>
       <c r="R124" s="2" t="inlineStr">
         <is>
-          <t>St. Louis's jazz-rap hybrid. Melodic and rhythmic sophistication.</t>
+          <t>'Igor' and 'Call Me If You Get Lost' — producer-auteur. Concept album mastery.</t>
         </is>
       </c>
     </row>
@@ -9721,12 +9713,12 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>AB2</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Pusha T</t>
+          <t>Armand Hammer</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -9741,49 +9733,53 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Coke Rap Boom Bap</t>
+          <t>Abstract Boom Bap</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>G.O.O.D.</t>
+          <t>Backwoodz</t>
         </is>
       </c>
       <c r="I125" s="2" t="n">
-        <v>2002</v>
+        <v>2012</v>
       </c>
       <c r="J125" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K125" s="10" t="n">
-        <v>7</v>
+      <c r="K125" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="L125" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="M125" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N125" s="10" t="n">
-        <v>7</v>
+      <c r="M125" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="N125" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="O125" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="P125" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q125" s="2" t="inlineStr"/>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P125" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q125" s="2" t="inlineStr">
+        <is>
+          <t>Critical underground darling; thin mainstream documentation</t>
+        </is>
+      </c>
       <c r="R125" s="2" t="inlineStr">
         <is>
-          <t>Cocaine rap's Rembrandt. 'Daytona' — maximum density, minimum waste.</t>
+          <t>billy woods + ELUCID. The most demanding abstract rap being made today.</t>
         </is>
       </c>
     </row>
@@ -9793,17 +9789,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>JS</t>
+          <t>ZE</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>JID</t>
+          <t>Zach Fox</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -9813,53 +9809,53 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Technical Rap</t>
+          <t>Comedy-Abstract Rap</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Dreamville</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="I126" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J126" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="K126" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L126" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M126" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N126" s="11" t="n">
-        <v>8</v>
+        <v>2020</v>
+      </c>
+      <c r="J126" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K126" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L126" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M126" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N126" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="O126" s="6" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="P126" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
+        <v>6.4</v>
+      </c>
+      <c r="P126" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="Q126" s="2" t="inlineStr">
         <is>
-          <t>Recent; scoring likely conservative; upward trajectory clear</t>
+          <t>Very recent; extremely limited critical record</t>
         </is>
       </c>
       <c r="R126" s="2" t="inlineStr">
         <is>
-          <t>Atlanta's most technically gifted. 'The Never Story' showed generational talent.</t>
+          <t>Comedy-meets-rap. Formally interesting but body of work too small to score confidently.</t>
         </is>
       </c>
     </row>
@@ -9869,17 +9865,17 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>TY</t>
+          <t>LI</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Tyler the Creator</t>
+          <t>Lil Durk</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -9889,49 +9885,53 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Odd Future/Orchestral</t>
+          <t>Chicago Melodic Trap</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Only the Family</t>
         </is>
       </c>
       <c r="I127" s="2" t="n">
-        <v>2009</v>
-      </c>
-      <c r="J127" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K127" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="L127" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M127" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="N127" s="12" t="n">
-        <v>9</v>
+        <v>2013</v>
+      </c>
+      <c r="J127" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K127" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L127" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M127" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N127" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="O127" s="6" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="P127" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q127" s="2" t="inlineStr"/>
+        <v>5.2</v>
+      </c>
+      <c r="P127" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q127" s="2" t="inlineStr">
+        <is>
+          <t>Commercial dominance clear; critical depth limited</t>
+        </is>
+      </c>
       <c r="R127" s="2" t="inlineStr">
         <is>
-          <t>'Igor' and 'Call Me If You Get Lost' — producer-auteur. Concept album mastery.</t>
+          <t>Chicago drill's most commercially consistent voice.</t>
         </is>
       </c>
     </row>
@@ -9941,17 +9941,17 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>AB2</t>
+          <t>KS2</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Armand Hammer</t>
+          <t>Kodak Black</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -9961,39 +9961,39 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>Abstract Boom Bap</t>
+          <t>Florida Trap</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Backwoodz</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="I128" s="2" t="n">
-        <v>2012</v>
-      </c>
-      <c r="J128" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K128" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="L128" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M128" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="N128" s="11" t="n">
-        <v>8</v>
+        <v>2014</v>
+      </c>
+      <c r="J128" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K128" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L128" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M128" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N128" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O128" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>5</v>
       </c>
       <c r="P128" s="14" t="inlineStr">
         <is>
@@ -10002,12 +10002,12 @@
       </c>
       <c r="Q128" s="2" t="inlineStr">
         <is>
-          <t>Critical underground darling; thin mainstream documentation</t>
+          <t>Commercial success; thin critical framework; behavior clouds reception</t>
         </is>
       </c>
       <c r="R128" s="2" t="inlineStr">
         <is>
-          <t>billy woods + ELUCID. The most demanding abstract rap being made today.</t>
+          <t>Florida trap's most distinctive voice. Rough-edged regional authenticity.</t>
         </is>
       </c>
     </row>
@@ -10017,17 +10017,17 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>ZE</t>
+          <t>RC</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Zach Fox</t>
+          <t>Rapsody</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -10037,53 +10037,49 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Conscious/Lyrical</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Comedy-Abstract Rap</t>
+          <t>North Carolina Soul Rap</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Jamla</t>
         </is>
       </c>
       <c r="I129" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="J129" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K129" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L129" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M129" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N129" s="9" t="n">
-        <v>6</v>
+        <v>2010</v>
+      </c>
+      <c r="J129" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K129" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L129" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M129" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N129" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="O129" s="6" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="P129" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="Q129" s="2" t="inlineStr">
-        <is>
-          <t>Very recent; extremely limited critical record</t>
-        </is>
-      </c>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P129" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q129" s="2" t="inlineStr"/>
       <c r="R129" s="2" t="inlineStr">
         <is>
-          <t>Comedy-meets-rap. Formally interesting but body of work too small to score confidently.</t>
+          <t>North Carolina's most complete female MC. Lyrical depth rivals any peer.</t>
         </is>
       </c>
     </row>
@@ -10093,12 +10089,12 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>LI</t>
+          <t>MF2</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Lil Durk</t>
+          <t>Mavi</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
@@ -10113,53 +10109,53 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Chicago Melodic Trap</t>
+          <t>Underground Abstract</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Only the Family</t>
+          <t>Mutant Academy</t>
         </is>
       </c>
       <c r="I130" s="2" t="n">
-        <v>2013</v>
-      </c>
-      <c r="J130" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K130" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L130" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M130" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N130" s="8" t="n">
-        <v>5</v>
+        <v>2019</v>
+      </c>
+      <c r="J130" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K130" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L130" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M130" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N130" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O130" s="6" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="P130" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
+        <v>7.2</v>
+      </c>
+      <c r="P130" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
         <is>
-          <t>Commercial dominance clear; critical depth limited</t>
+          <t>Very limited critical documentation; underground following only</t>
         </is>
       </c>
       <c r="R130" s="2" t="inlineStr">
         <is>
-          <t>Chicago drill's most commercially consistent voice.</t>
+          <t>Charlotte underground. Dense introspective abstract rap. Watch this space.</t>
         </is>
       </c>
     </row>
@@ -10169,22 +10165,22 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>KS2</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Kodak Black</t>
+          <t>Xzibit</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>2020s</t>
+          <t>2000s</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -10194,34 +10190,34 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>Florida Trap</t>
+          <t>Hard West Coast</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Loud/Columbia</t>
         </is>
       </c>
       <c r="I131" s="2" t="n">
-        <v>2014</v>
-      </c>
-      <c r="J131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L131" s="9" t="n">
+        <v>1996</v>
+      </c>
+      <c r="J131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N131" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="M131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N131" s="5" t="n">
-        <v>4</v>
-      </c>
       <c r="O131" s="6" t="n">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="P131" s="14" t="inlineStr">
         <is>
@@ -10230,12 +10226,12 @@
       </c>
       <c r="Q131" s="2" t="inlineStr">
         <is>
-          <t>Commercial success; thin critical framework; behavior clouds reception</t>
+          <t>Well-known but limited formal critical analysis</t>
         </is>
       </c>
       <c r="R131" s="2" t="inlineStr">
         <is>
-          <t>Florida trap's most distinctive voice. Rough-edged regional authenticity.</t>
+          <t>West Coast boom bap craftsman. More respected by peers than critics.</t>
         </is>
       </c>
     </row>
@@ -10245,17 +10241,17 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>LA2</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>Lana (Kali Uchis rap)</t>
+          <t>Saweetie</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -10265,53 +10261,53 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>R&amp;B/Latin Rap Hybrid</t>
+          <t>Trap Pop</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>Virgin</t>
+          <t>Warner</t>
         </is>
       </c>
       <c r="I132" s="2" t="n">
         <v>2018</v>
       </c>
-      <c r="J132" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K132" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L132" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M132" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N132" s="10" t="n">
-        <v>7</v>
+      <c r="J132" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K132" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L132" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M132" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N132" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O132" s="6" t="n">
-        <v>6.6</v>
-      </c>
-      <c r="P132" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
+        <v>4.8</v>
+      </c>
+      <c r="P132" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="Q132" s="2" t="inlineStr">
         <is>
-          <t>Primarily R&amp;B artist; rap output limited and under-analyzed</t>
+          <t>Recent commercial success; limited critical depth</t>
         </is>
       </c>
       <c r="R132" s="2" t="inlineStr">
         <is>
-          <t>Colombian-American crossover. When rapping, brings genuine bilingual lyricism.</t>
+          <t>Bay Area trap-pop. Ice Princess persona over lyrical substance.</t>
         </is>
       </c>
     </row>
@@ -10321,12 +10317,12 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>RC</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Rapsody</t>
+          <t>City Girls</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -10341,49 +10337,53 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>North Carolina Soul Rap</t>
+          <t>Miami Trap</t>
         </is>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Jamla</t>
+          <t>Quality Control/Motown</t>
         </is>
       </c>
       <c r="I133" s="2" t="n">
-        <v>2010</v>
-      </c>
-      <c r="J133" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K133" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L133" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M133" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N133" s="12" t="n">
-        <v>9</v>
+        <v>2018</v>
+      </c>
+      <c r="J133" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K133" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L133" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M133" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N133" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O133" s="6" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="P133" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q133" s="2" t="inlineStr"/>
+        <v>4.6</v>
+      </c>
+      <c r="P133" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q133" s="2" t="inlineStr">
+        <is>
+          <t>Limited critical record; cultural impact clearer than lyrical analysis</t>
+        </is>
+      </c>
       <c r="R133" s="2" t="inlineStr">
         <is>
-          <t>North Carolina's most complete female MC. Lyrical depth rivals any peer.</t>
+          <t>Miami's hedonistic party rap duo. Energy over craft.</t>
         </is>
       </c>
     </row>
@@ -10393,17 +10393,17 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>Noname (Ghetto Sage)</t>
+          <t>Maxo Kream</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
@@ -10413,39 +10413,39 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>Political</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Political Jazz Rap</t>
+          <t>Houston Narrative Trap</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>EMPIRE</t>
         </is>
       </c>
       <c r="I134" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="J134" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K134" s="12" t="n">
+        <v>2017</v>
+      </c>
+      <c r="J134" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K134" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L134" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="L134" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M134" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N134" s="13" t="n">
-        <v>10</v>
+      <c r="M134" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N134" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O134" s="6" t="n">
-        <v>8.6</v>
+        <v>7.4</v>
       </c>
       <c r="P134" s="14" t="inlineStr">
         <is>
@@ -10454,12 +10454,12 @@
       </c>
       <c r="Q134" s="2" t="inlineStr">
         <is>
-          <t>Political evolution post-Room 25; scoring for this phase specifically</t>
+          <t>Critical acclaim in narrative rap circles; limited mainstream documentation</t>
         </is>
       </c>
       <c r="R134" s="2" t="inlineStr">
         <is>
-          <t>Noname's political radicalization phase. Most conceptually ambitious output.</t>
+          <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
         </is>
       </c>
     </row>
@@ -10469,17 +10469,17 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>MF2</t>
+          <t>YN</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Mavi</t>
+          <t>Yaya Bey</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
@@ -10489,21 +10489,21 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Underground Abstract</t>
+          <t>Neo-Soul Jazz Rap</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>Mutant Academy</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="I135" s="2" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="J135" s="10" t="n">
         <v>7</v>
@@ -10514,14 +10514,14 @@
       <c r="L135" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="M135" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N135" s="10" t="n">
-        <v>7</v>
+      <c r="M135" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N135" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="O135" s="6" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="P135" s="15" t="inlineStr">
         <is>
@@ -10530,390 +10530,10 @@
       </c>
       <c r="Q135" s="2" t="inlineStr">
         <is>
-          <t>Very limited critical documentation; underground following only</t>
+          <t>Very recent and limited documentation; genre straddles rap and R&amp;B</t>
         </is>
       </c>
       <c r="R135" s="2" t="inlineStr">
-        <is>
-          <t>Charlotte underground. Dense introspective abstract rap. Watch this space.</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="2" t="n">
-        <v>135</v>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
-        <is>
-          <t>XP</t>
-        </is>
-      </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>Xzibit</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t>2000s</t>
-        </is>
-      </c>
-      <c r="F136" s="2" t="inlineStr">
-        <is>
-          <t>Gangsta/Street</t>
-        </is>
-      </c>
-      <c r="G136" s="2" t="inlineStr">
-        <is>
-          <t>Hard West Coast</t>
-        </is>
-      </c>
-      <c r="H136" s="2" t="inlineStr">
-        <is>
-          <t>Loud/Columbia</t>
-        </is>
-      </c>
-      <c r="I136" s="2" t="n">
-        <v>1996</v>
-      </c>
-      <c r="J136" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K136" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L136" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M136" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N136" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="O136" s="6" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="P136" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q136" s="2" t="inlineStr">
-        <is>
-          <t>Well-known but limited formal critical analysis</t>
-        </is>
-      </c>
-      <c r="R136" s="2" t="inlineStr">
-        <is>
-          <t>West Coast boom bap craftsman. More respected by peers than critics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="2" t="n">
-        <v>136</v>
-      </c>
-      <c r="B137" s="2" t="inlineStr">
-        <is>
-          <t>SA</t>
-        </is>
-      </c>
-      <c r="C137" s="2" t="inlineStr">
-        <is>
-          <t>Saweetie</t>
-        </is>
-      </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="E137" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F137" s="2" t="inlineStr">
-        <is>
-          <t>Party/Pop</t>
-        </is>
-      </c>
-      <c r="G137" s="2" t="inlineStr">
-        <is>
-          <t>Trap Pop</t>
-        </is>
-      </c>
-      <c r="H137" s="2" t="inlineStr">
-        <is>
-          <t>Warner</t>
-        </is>
-      </c>
-      <c r="I137" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J137" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K137" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L137" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="M137" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N137" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O137" s="6" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="P137" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q137" s="2" t="inlineStr">
-        <is>
-          <t>Recent commercial success; limited critical depth</t>
-        </is>
-      </c>
-      <c r="R137" s="2" t="inlineStr">
-        <is>
-          <t>Bay Area trap-pop. Ice Princess persona over lyrical substance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="n">
-        <v>137</v>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>CI</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>City Girls</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="E138" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F138" s="2" t="inlineStr">
-        <is>
-          <t>Party/Pop</t>
-        </is>
-      </c>
-      <c r="G138" s="2" t="inlineStr">
-        <is>
-          <t>Miami Trap</t>
-        </is>
-      </c>
-      <c r="H138" s="2" t="inlineStr">
-        <is>
-          <t>Quality Control/Motown</t>
-        </is>
-      </c>
-      <c r="I138" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J138" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K138" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L138" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="M138" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N138" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O138" s="6" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="P138" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="Q138" s="2" t="inlineStr">
-        <is>
-          <t>Limited critical record; cultural impact clearer than lyrical analysis</t>
-        </is>
-      </c>
-      <c r="R138" s="2" t="inlineStr">
-        <is>
-          <t>Miami's hedonistic party rap duo. Energy over craft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="2" t="n">
-        <v>138</v>
-      </c>
-      <c r="B139" s="2" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="C139" s="2" t="inlineStr">
-        <is>
-          <t>Maxo Kream</t>
-        </is>
-      </c>
-      <c r="D139" s="2" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="E139" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F139" s="2" t="inlineStr">
-        <is>
-          <t>Gangsta/Street</t>
-        </is>
-      </c>
-      <c r="G139" s="2" t="inlineStr">
-        <is>
-          <t>Houston Narrative Trap</t>
-        </is>
-      </c>
-      <c r="H139" s="2" t="inlineStr">
-        <is>
-          <t>EMPIRE</t>
-        </is>
-      </c>
-      <c r="I139" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J139" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K139" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L139" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="M139" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N139" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="O139" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="P139" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q139" s="2" t="inlineStr">
-        <is>
-          <t>Critical acclaim in narrative rap circles; limited mainstream documentation</t>
-        </is>
-      </c>
-      <c r="R139" s="2" t="inlineStr">
-        <is>
-          <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="2" t="n">
-        <v>139</v>
-      </c>
-      <c r="B140" s="2" t="inlineStr">
-        <is>
-          <t>YN</t>
-        </is>
-      </c>
-      <c r="C140" s="2" t="inlineStr">
-        <is>
-          <t>Yaya Bey</t>
-        </is>
-      </c>
-      <c r="D140" s="2" t="inlineStr">
-        <is>
-          <t>NYC</t>
-        </is>
-      </c>
-      <c r="E140" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F140" s="2" t="inlineStr">
-        <is>
-          <t>Experimental</t>
-        </is>
-      </c>
-      <c r="G140" s="2" t="inlineStr">
-        <is>
-          <t>Neo-Soul Jazz Rap</t>
-        </is>
-      </c>
-      <c r="H140" s="2" t="inlineStr">
-        <is>
-          <t>Independent</t>
-        </is>
-      </c>
-      <c r="I140" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="J140" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K140" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L140" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M140" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N140" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="O140" s="6" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="P140" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="Q140" s="2" t="inlineStr">
-        <is>
-          <t>Very recent and limited documentation; genre straddles rap and R&amp;B</t>
-        </is>
-      </c>
-      <c r="R140" s="2" t="inlineStr">
         <is>
           <t>Brooklyn experimental R&amp;B-rap hybrid. Underrecognized artistic depth.</t>
         </is>

</xml_diff>

<commit_message>
Accuracy pass: L-flagged factual corrections (web-verified)
- Schoolly D: region South -> NYC (he's from Philadelphia / East Coast)
- Kenny Mason: label Independent -> RCA Records
- Zack Fox: fix name spelling (Zach -> Zack); region NYC -> South (Atlanta)
- Mavi: label Mutant Academy -> Secretly Canadian (not a Mutant Academy act)
- Yaya Bey: label Independent -> Big Dada
- Verified accurate, no change: J.J. Fad, Dana Dane, Jedi Mind Tricks,
  Trae Tha Truth, GloRilla, City Girls
- Update accuracy_worklist.md to reflect the factual pass

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>RCA Records</t>
         </is>
       </c>
       <c r="I120" s="2" t="n">
@@ -9794,12 +9794,12 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Zach Fox</t>
+          <t>Zack Fox</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -10119,7 +10119,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Mutant Academy</t>
+          <t>Secretly Canadian</t>
         </is>
       </c>
       <c r="I130" s="2" t="n">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Big Dada</t>
         </is>
       </c>
       <c r="I135" s="2" t="n">

</xml_diff>

<commit_message>
Add Philly region; drop Yaya Bey (133 artists)
- New "Philly" region with its own color (teal #4e9e94): legend, filter
  dropdown, REGION_COLORS map, and edit/add forms all updated
- Reassign Schoolly D and Jedi Mind Tricks from NYC -> Philly (both are
  from Philadelphia); room to grow as The Roots, Beanie Sigel, Meek Mill,
  etc. get added in expansion
- Drop Yaya Bey (primarily neo-soul/R&B; out of scope), renumber to 133

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R135"/>
+  <dimension ref="A1:R134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>Philly</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>Philly</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -10460,82 +10460,6 @@
       <c r="R134" s="2" t="inlineStr">
         <is>
           <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="2" t="n">
-        <v>134</v>
-      </c>
-      <c r="B135" s="2" t="inlineStr">
-        <is>
-          <t>YN</t>
-        </is>
-      </c>
-      <c r="C135" s="2" t="inlineStr">
-        <is>
-          <t>Yaya Bey</t>
-        </is>
-      </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t>NYC</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F135" s="2" t="inlineStr">
-        <is>
-          <t>Experimental</t>
-        </is>
-      </c>
-      <c r="G135" s="2" t="inlineStr">
-        <is>
-          <t>Neo-Soul Jazz Rap</t>
-        </is>
-      </c>
-      <c r="H135" s="2" t="inlineStr">
-        <is>
-          <t>Big Dada</t>
-        </is>
-      </c>
-      <c r="I135" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="J135" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K135" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L135" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M135" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N135" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="O135" s="6" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="P135" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="Q135" s="2" t="inlineStr">
-        <is>
-          <t>Very recent and limited documentation; genre straddles rap and R&amp;B</t>
-        </is>
-      </c>
-      <c r="R135" s="2" t="inlineStr">
-        <is>
-          <t>Brooklyn experimental R&amp;B-rap hybrid. Underrecognized artistic depth.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Accuracy pass: M-flagged region fixes (web-verified)
- Tierra Whack: NYC -> Philly (North Philadelphia)
- Lil Durk: South -> Midwest (Englewood, South Side Chicago)
- Saweetie: LA -> Bay Area (born Santa Clara, raised Hayward/Sacramento)
- Completes the factual audit of all 9 L- and 39 M-flagged artists;
  remaining open items (era/debut/label nits) noted in accuracy_worklist.md

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -8163,7 +8163,7 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>Philly</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -9875,7 +9875,7 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Accuracy: factual nits + Jadakiss score correction
Factual (web-verified):
- Freestyle Fellowship label Acacia -> Sun Music (1991 debut label)
- Three 6 Mafia label Sony -> Hypnotize Minds (signature label)
- Armand Hammer debut 2012 -> 2013 (Race Music)
- Xzibit era 2000s -> Late 90s (debuted 1996, matches debut-based bucketing)
- Juvenile 1994 confirmed correct (no change)

Score:
- Jadakiss 6.8 -> 7.2 (Rhyme/Metaphor 7->8): elite punchline lyricist
  was undersold on his signature dimension

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -3579,7 +3579,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Acacia</t>
+          <t>Sun Music</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -6146,7 +6146,7 @@
         <v>2001</v>
       </c>
       <c r="J76" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K76" s="10" t="n">
         <v>7</v>
@@ -6155,13 +6155,13 @@
         <v>7</v>
       </c>
       <c r="M76" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N76" s="9" t="n">
         <v>6</v>
       </c>
       <c r="O76" s="6" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
       <c r="P76" s="14" t="inlineStr">
         <is>
@@ -6287,7 +6287,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Sony</t>
+          <t>Hypnotize Minds</t>
         </is>
       </c>
       <c r="I78" s="2" t="n">
@@ -9747,7 +9747,7 @@
         </is>
       </c>
       <c r="I125" s="2" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="J125" s="11" t="n">
         <v>8</v>
@@ -10180,7 +10180,7 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>2000s</t>
+          <t>Late 90s</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Expansion batch 1: +18 artists -> 150
US-only additions (no International/UK per scope), region by label/scene
base rather than birthplace:
- Philly (4->9): Black Thought, Beanie Sigel, Lil Uzi Vert, Freeway, Eve
- Bay Area (2->5): Too $hort, Del the Funky Homosapien, Mac Dre
- NYC legends: Kool G Rap, Redman, Method Man, EPMD
- LA: The Game, Ice-T, Nipsey Hussle, DJ Quik
- Midwest: Royce da 5'9"; South: Da Brat (So So Def/Atlanta)

All composites computed from the 5 dims; symbols unique; integrity
verified (no dup names/symbols, valid regions, sequential numbering).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R133"/>
+  <dimension ref="A1:R151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10387,6 +10387,1364 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BT3</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Black Thought</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Live-Band Boom Bap</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Geffen/MCA</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>1993</v>
+      </c>
+      <c r="J134" t="n">
+        <v>10</v>
+      </c>
+      <c r="K134" t="n">
+        <v>9</v>
+      </c>
+      <c r="L134" t="n">
+        <v>8</v>
+      </c>
+      <c r="M134" t="n">
+        <v>9</v>
+      </c>
+      <c r="N134" t="n">
+        <v>8</v>
+      </c>
+      <c r="O134" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>The Roots' engine and a consensus top-tier technician. Relentless breath control and rhyme density.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Beanie Sigel</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Soul Boom Bap</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Roc-A-Fella</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J135" t="n">
+        <v>8</v>
+      </c>
+      <c r="K135" t="n">
+        <v>7</v>
+      </c>
+      <c r="L135" t="n">
+        <v>8</v>
+      </c>
+      <c r="M135" t="n">
+        <v>7</v>
+      </c>
+      <c r="N135" t="n">
+        <v>7</v>
+      </c>
+      <c r="O135" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q135" t="inlineStr">
+        <is>
+          <t>Critically respected but thinly documented outside the Roc-A-Fella context.</t>
+        </is>
+      </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>Philadelphia's hardest pen. Street narratives carried with weight and conviction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>UV</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Lil Uzi Vert</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>2010s</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Rage/Trap</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Generation Now/Atlantic</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J136" t="n">
+        <v>6</v>
+      </c>
+      <c r="K136" t="n">
+        <v>6</v>
+      </c>
+      <c r="L136" t="n">
+        <v>5</v>
+      </c>
+      <c r="M136" t="n">
+        <v>6</v>
+      </c>
+      <c r="N136" t="n">
+        <v>6</v>
+      </c>
+      <c r="O136" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q136" t="inlineStr">
+        <is>
+          <t>Melodic rage star; influence on sound outweighs lyrical scholarship.</t>
+        </is>
+      </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>Genre-bending rage pioneer. Melody and energy over lyrical density.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>FW</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Freeway</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Soul Boom Bap</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Roc-A-Fella</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>2003</v>
+      </c>
+      <c r="J137" t="n">
+        <v>7</v>
+      </c>
+      <c r="K137" t="n">
+        <v>6</v>
+      </c>
+      <c r="L137" t="n">
+        <v>6</v>
+      </c>
+      <c r="M137" t="n">
+        <v>6</v>
+      </c>
+      <c r="N137" t="n">
+        <v>5</v>
+      </c>
+      <c r="O137" t="n">
+        <v>6</v>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q137" t="inlineStr">
+        <is>
+          <t>Limited critical record; respected within State Property/Roc-A-Fella circles.</t>
+        </is>
+      </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>Distinctive raspy urgency and Philly grit. State Property standout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>EV</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Eve</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Ruff Ryders</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Ruff Ryders/Interscope</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>1999</v>
+      </c>
+      <c r="J138" t="n">
+        <v>6</v>
+      </c>
+      <c r="K138" t="n">
+        <v>6</v>
+      </c>
+      <c r="L138" t="n">
+        <v>6</v>
+      </c>
+      <c r="M138" t="n">
+        <v>6</v>
+      </c>
+      <c r="N138" t="n">
+        <v>5</v>
+      </c>
+      <c r="O138" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q138" t="inlineStr">
+        <is>
+          <t>Commercial success clearer than lyrical analysis.</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>Ruff Ryders' First Lady. Charismatic crossover with Philly roots.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>DB</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Da Brat</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>So So Def Bass</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>So So Def</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J139" t="n">
+        <v>6</v>
+      </c>
+      <c r="K139" t="n">
+        <v>6</v>
+      </c>
+      <c r="L139" t="n">
+        <v>6</v>
+      </c>
+      <c r="M139" t="n">
+        <v>6</v>
+      </c>
+      <c r="N139" t="n">
+        <v>5</v>
+      </c>
+      <c r="O139" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q139" t="inlineStr">
+        <is>
+          <t>First female solo rapper to go platinum; under-analyzed lyrically.</t>
+        </is>
+      </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>So So Def's breakout. First female solo rapper to go platinum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>TS2</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Too $hort</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Old School</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Funk/Bass</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Jive/Dangerous Music</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>1987</v>
+      </c>
+      <c r="J140" t="n">
+        <v>6</v>
+      </c>
+      <c r="K140" t="n">
+        <v>5</v>
+      </c>
+      <c r="L140" t="n">
+        <v>6</v>
+      </c>
+      <c r="M140" t="n">
+        <v>5</v>
+      </c>
+      <c r="N140" t="n">
+        <v>5</v>
+      </c>
+      <c r="O140" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q140" t="inlineStr">
+        <is>
+          <t>Pioneer status outweighs lyrical-craft documentation.</t>
+        </is>
+      </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>Oakland pioneer and pimp-rap archetype. Influence over intricacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Del the Funky Homosapien</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Hieroglyphics</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Elektra/Hiero Imperium</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>1991</v>
+      </c>
+      <c r="J141" t="n">
+        <v>7</v>
+      </c>
+      <c r="K141" t="n">
+        <v>8</v>
+      </c>
+      <c r="L141" t="n">
+        <v>6</v>
+      </c>
+      <c r="M141" t="n">
+        <v>7</v>
+      </c>
+      <c r="N141" t="n">
+        <v>7</v>
+      </c>
+      <c r="O141" t="n">
+        <v>7</v>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q141" t="inlineStr">
+        <is>
+          <t>Underground Hieroglyphics following; specialist critical attention.</t>
+        </is>
+      </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>Hieroglyphics wordsmith. Quirky vocabulary and abstract wit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>MD3</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Mac Dre</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Hyphy</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Thizz Entertainment</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J142" t="n">
+        <v>6</v>
+      </c>
+      <c r="K142" t="n">
+        <v>6</v>
+      </c>
+      <c r="L142" t="n">
+        <v>6</v>
+      </c>
+      <c r="M142" t="n">
+        <v>5</v>
+      </c>
+      <c r="N142" t="n">
+        <v>5</v>
+      </c>
+      <c r="O142" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>Regional hyphy icon; limited national critical record.</t>
+        </is>
+      </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>Hyphy movement godfather. Enduring Bay Area cult legend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Royce da 5'9"</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Detroit Boom Bap</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Shady/Independent</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>2002</v>
+      </c>
+      <c r="J143" t="n">
+        <v>9</v>
+      </c>
+      <c r="K143" t="n">
+        <v>8</v>
+      </c>
+      <c r="L143" t="n">
+        <v>7</v>
+      </c>
+      <c r="M143" t="n">
+        <v>8</v>
+      </c>
+      <c r="N143" t="n">
+        <v>7</v>
+      </c>
+      <c r="O143" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q143" t="inlineStr">
+        <is>
+          <t>Elite technician; documentation grew via Slaughterhouse and PRhyme.</t>
+        </is>
+      </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>Detroit technician. Slaughterhouse and PRhyme cornerstone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Kool G Rap</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Boom Bap</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Cold Chillin'</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>1989</v>
+      </c>
+      <c r="J144" t="n">
+        <v>9</v>
+      </c>
+      <c r="K144" t="n">
+        <v>8</v>
+      </c>
+      <c r="L144" t="n">
+        <v>9</v>
+      </c>
+      <c r="M144" t="n">
+        <v>8</v>
+      </c>
+      <c r="N144" t="n">
+        <v>7</v>
+      </c>
+      <c r="O144" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>Mafioso-rap forefather. The multisyllabic blueprint for Nas, Biggie and Jay-Z.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Redman</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Funk Boom Bap</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Def Jam</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>1992</v>
+      </c>
+      <c r="J145" t="n">
+        <v>8</v>
+      </c>
+      <c r="K145" t="n">
+        <v>7</v>
+      </c>
+      <c r="L145" t="n">
+        <v>7</v>
+      </c>
+      <c r="M145" t="n">
+        <v>7</v>
+      </c>
+      <c r="N145" t="n">
+        <v>6</v>
+      </c>
+      <c r="O145" t="n">
+        <v>7</v>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q145" t="inlineStr">
+        <is>
+          <t>Beloved and skilled; lyrical scholarship modest relative to peers.</t>
+        </is>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Newark's funkiest. Effortless flow with comedic menace.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Method Man</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Wu-Tang</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Def Jam</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J146" t="n">
+        <v>7</v>
+      </c>
+      <c r="K146" t="n">
+        <v>7</v>
+      </c>
+      <c r="L146" t="n">
+        <v>6</v>
+      </c>
+      <c r="M146" t="n">
+        <v>7</v>
+      </c>
+      <c r="N146" t="n">
+        <v>6</v>
+      </c>
+      <c r="O146" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q146" t="inlineStr">
+        <is>
+          <t>Scored solo; Wu-Tang charisma vs pure-lyric metrics.</t>
+        </is>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>Wu-Tang's charismatic star. Gravel-voiced hooks and grit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>EP</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>EPMD</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Funk Boom Bap</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Def Jam</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>1988</v>
+      </c>
+      <c r="J147" t="n">
+        <v>7</v>
+      </c>
+      <c r="K147" t="n">
+        <v>6</v>
+      </c>
+      <c r="L147" t="n">
+        <v>6</v>
+      </c>
+      <c r="M147" t="n">
+        <v>6</v>
+      </c>
+      <c r="N147" t="n">
+        <v>6</v>
+      </c>
+      <c r="O147" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q147" t="inlineStr">
+        <is>
+          <t>Influential funk-rap duo; understated lyrical documentation.</t>
+        </is>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Strictly Business. Laid-back funk and durable chemistry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>TG</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>The Game</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>West Coast</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Aftermath/G-Unit</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>2005</v>
+      </c>
+      <c r="J148" t="n">
+        <v>7</v>
+      </c>
+      <c r="K148" t="n">
+        <v>7</v>
+      </c>
+      <c r="L148" t="n">
+        <v>7</v>
+      </c>
+      <c r="M148" t="n">
+        <v>7</v>
+      </c>
+      <c r="N148" t="n">
+        <v>6</v>
+      </c>
+      <c r="O148" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q148" t="inlineStr">
+        <is>
+          <t>Commercially dominant; reference-heavy bars, mixed critical view.</t>
+        </is>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Compton revivalist. The Documentary-era West Coast resurgence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Ice-T</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Old School</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Electro/Funk</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Sire/Rhyme Syndicate</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>1987</v>
+      </c>
+      <c r="J149" t="n">
+        <v>6</v>
+      </c>
+      <c r="K149" t="n">
+        <v>6</v>
+      </c>
+      <c r="L149" t="n">
+        <v>7</v>
+      </c>
+      <c r="M149" t="n">
+        <v>6</v>
+      </c>
+      <c r="N149" t="n">
+        <v>7</v>
+      </c>
+      <c r="O149" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Gangsta-rap pioneer; influence and narrative over technical metrics.</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Gangsta-rap originator. Street reportage before the template existed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Nipsey Hussle</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2010s</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Conscious/Street</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>West Coast</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>All Money In/Atlantic</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J150" t="n">
+        <v>7</v>
+      </c>
+      <c r="K150" t="n">
+        <v>7</v>
+      </c>
+      <c r="L150" t="n">
+        <v>7</v>
+      </c>
+      <c r="M150" t="n">
+        <v>7</v>
+      </c>
+      <c r="N150" t="n">
+        <v>7</v>
+      </c>
+      <c r="O150" t="n">
+        <v>7</v>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Posthumous reappraisal ongoing; entrepreneurial legacy prominent.</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Crenshaw's marathon. Street wisdom and self-determination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>DQ</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>DJ Quik</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>G-Funk</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>1991</v>
+      </c>
+      <c r="J151" t="n">
+        <v>7</v>
+      </c>
+      <c r="K151" t="n">
+        <v>6</v>
+      </c>
+      <c r="L151" t="n">
+        <v>6</v>
+      </c>
+      <c r="M151" t="n">
+        <v>6</v>
+      </c>
+      <c r="N151" t="n">
+        <v>6</v>
+      </c>
+      <c r="O151" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>Revered as a producer; underrated as a lyricist.</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>G-funk auteur. Producer-rapper with effortless West Coast bounce.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rename Black Thought -> The Roots; remove Iggy Azalea + Stormzy
- Use the group "The Roots" (symbol RT) rather than Black Thought solo,
  matching the original intent
- Remove Iggy Azalea (International) and Stormzy (UK) per scope decision
  to keep the table US-focused; Drake (International/Canadian) left
  pending a separate decision
- 148 artists

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R151"/>
+  <dimension ref="A1:R149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7785,17 +7785,17 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Iggy Azalea</t>
+          <t>Freddie Gibbs</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>International</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -7805,39 +7805,39 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Southern Trap Pop</t>
+          <t>Gangsta Boom Bap</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Grand Hustle</t>
+          <t>ESGN</t>
         </is>
       </c>
       <c r="I99" s="2" t="n">
-        <v>2014</v>
-      </c>
-      <c r="J99" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K99" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L99" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M99" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="N99" s="3" t="n">
-        <v>3</v>
+        <v>2004</v>
+      </c>
+      <c r="J99" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K99" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L99" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="M99" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N99" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O99" s="6" t="n">
-        <v>3.8</v>
+        <v>7.8</v>
       </c>
       <c r="P99" s="7" t="inlineStr">
         <is>
@@ -7847,7 +7847,7 @@
       <c r="Q99" s="2" t="inlineStr"/>
       <c r="R99" s="2" t="inlineStr">
         <is>
-          <t>Commercial success masking thin lyrical foundation. Accent controversy.</t>
+          <t>Gary Indiana's finest. Technical gangsta rap with jazz-rap production.</t>
         </is>
       </c>
     </row>
@@ -7857,17 +7857,17 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>FS</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Freddie Gibbs</t>
+          <t>Migos</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -7877,39 +7877,39 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Trap/Drill</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Gangsta Boom Bap</t>
+          <t>Atlanta Triplet Trap</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>ESGN</t>
+          <t>Quality Control</t>
         </is>
       </c>
       <c r="I100" s="2" t="n">
-        <v>2004</v>
-      </c>
-      <c r="J100" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K100" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L100" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="M100" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N100" s="10" t="n">
-        <v>7</v>
+        <v>2013</v>
+      </c>
+      <c r="J100" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K100" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L100" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="M100" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N100" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="O100" s="6" t="n">
-        <v>7.8</v>
+        <v>4</v>
       </c>
       <c r="P100" s="7" t="inlineStr">
         <is>
@@ -7919,7 +7919,7 @@
       <c r="Q100" s="2" t="inlineStr"/>
       <c r="R100" s="2" t="inlineStr">
         <is>
-          <t>Gary Indiana's finest. Technical gangsta rap with jazz-rap production.</t>
+          <t>Triplet flow inventors. Cultural influence far exceeds lyrical complexity.</t>
         </is>
       </c>
     </row>
@@ -7929,17 +7929,17 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>BI2</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Migos</t>
+          <t>Big Sean</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -7949,49 +7949,53 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Trap/Drill</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Triplet Trap</t>
+          <t>Detroit Pop Rap</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Quality Control</t>
+          <t>G.O.O.D.</t>
         </is>
       </c>
       <c r="I101" s="2" t="n">
-        <v>2013</v>
-      </c>
-      <c r="J101" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K101" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L101" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M101" s="8" t="n">
+        <v>2011</v>
+      </c>
+      <c r="J101" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K101" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L101" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M101" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N101" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="N101" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="O101" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P101" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q101" s="2" t="inlineStr"/>
+        <v>5.8</v>
+      </c>
+      <c r="P101" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q101" s="2" t="inlineStr">
+        <is>
+          <t>Commercial success; critical reception mixed; thin formal analysis</t>
+        </is>
+      </c>
       <c r="R101" s="2" t="inlineStr">
         <is>
-          <t>Triplet flow inventors. Cultural influence far exceeds lyrical complexity.</t>
+          <t>Detroit MC. Punchlines over conceptual depth. 'One Man Can Change The World'.</t>
         </is>
       </c>
     </row>
@@ -8001,17 +8005,17 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>BI2</t>
+          <t>TR</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Big Sean</t>
+          <t>Tierra Whack</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>Philly</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -8021,39 +8025,39 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Detroit Pop Rap</t>
+          <t>Experimental Pop Rap</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>G.O.O.D.</t>
+          <t>Interscope</t>
         </is>
       </c>
       <c r="I102" s="2" t="n">
-        <v>2011</v>
-      </c>
-      <c r="J102" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K102" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L102" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M102" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N102" s="8" t="n">
-        <v>5</v>
+        <v>2018</v>
+      </c>
+      <c r="J102" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K102" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L102" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M102" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N102" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="O102" s="6" t="n">
-        <v>5.8</v>
+        <v>7.6</v>
       </c>
       <c r="P102" s="14" t="inlineStr">
         <is>
@@ -8062,12 +8066,12 @@
       </c>
       <c r="Q102" s="2" t="inlineStr">
         <is>
-          <t>Commercial success; critical reception mixed; thin formal analysis</t>
+          <t>Breakout 2018; critical buzz high but career short; scoring may shift</t>
         </is>
       </c>
       <c r="R102" s="2" t="inlineStr">
         <is>
-          <t>Detroit MC. Punchlines over conceptual depth. 'One Man Can Change The World'.</t>
+          <t>'Whack World' — 15 one-minute songs as unified concept. Wholly original.</t>
         </is>
       </c>
     </row>
@@ -8077,17 +8081,17 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>TR</t>
+          <t>NL</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Tierra Whack</t>
+          <t>Noname</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -8097,53 +8101,49 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Conscious/Lyrical</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Experimental Pop Rap</t>
+          <t>Chicago Jazz Rap</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Interscope</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="I103" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J103" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K103" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L103" s="10" t="n">
-        <v>7</v>
+        <v>2016</v>
+      </c>
+      <c r="J103" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K103" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="L103" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="M103" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="N103" s="11" t="n">
-        <v>8</v>
+      <c r="N103" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="O103" s="6" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="P103" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q103" s="2" t="inlineStr">
-        <is>
-          <t>Breakout 2018; critical buzz high but career short; scoring may shift</t>
-        </is>
-      </c>
+        <v>8.4</v>
+      </c>
+      <c r="P103" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q103" s="2" t="inlineStr"/>
       <c r="R103" s="2" t="inlineStr">
         <is>
-          <t>'Whack World' — 15 one-minute songs as unified concept. Wholly original.</t>
+          <t>Chicago's most literary voice. Jazz cadences and political awakening.</t>
         </is>
       </c>
     </row>
@@ -8153,12 +8153,12 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Noname</t>
+          <t>Saba</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -8178,34 +8178,34 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Chicago Jazz Rap</t>
+          <t>Chicago Boom Bap</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Pivot Gang</t>
         </is>
       </c>
       <c r="I104" s="2" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="J104" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K104" s="12" t="n">
+      <c r="K104" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L104" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="L104" s="11" t="n">
-        <v>8</v>
-      </c>
       <c r="M104" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="N104" s="12" t="n">
-        <v>9</v>
+      <c r="N104" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="O104" s="6" t="n">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="P104" s="7" t="inlineStr">
         <is>
@@ -8215,7 +8215,7 @@
       <c r="Q104" s="2" t="inlineStr"/>
       <c r="R104" s="2" t="inlineStr">
         <is>
-          <t>Chicago's most literary voice. Jazz cadences and political awakening.</t>
+          <t>'CARE FOR ME' — grief and Chicago violence as devastating concept album.</t>
         </is>
       </c>
     </row>
@@ -8225,12 +8225,12 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>SZ</t>
+          <t>DC</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Saba</t>
+          <t>Danny Brown</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -8245,33 +8245,33 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Chicago Boom Bap</t>
+          <t>Detroit Noise Rap</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Pivot Gang</t>
+          <t>Fool's Gold</t>
         </is>
       </c>
       <c r="I105" s="2" t="n">
-        <v>2014</v>
+        <v>2010</v>
       </c>
       <c r="J105" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K105" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L105" s="12" t="n">
+      <c r="K105" s="12" t="n">
         <v>9</v>
       </c>
-      <c r="M105" s="11" t="n">
-        <v>8</v>
+      <c r="L105" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M105" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="N105" s="11" t="n">
         <v>8</v>
@@ -8287,7 +8287,7 @@
       <c r="Q105" s="2" t="inlineStr"/>
       <c r="R105" s="2" t="inlineStr">
         <is>
-          <t>'CARE FOR ME' — grief and Chicago violence as devastating concept album.</t>
+          <t>Detroit's avant-garde MC. Schizophrenic flows and surreal imagery.</t>
         </is>
       </c>
     </row>
@@ -8297,12 +8297,12 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>DC</t>
+          <t>MH</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Danny Brown</t>
+          <t>Mac Miller</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -8317,39 +8317,39 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Conscious/Lyrical</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Detroit Noise Rap</t>
+          <t>Pittsburgh Soul Rap</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Fool's Gold</t>
+          <t>Rostrum</t>
         </is>
       </c>
       <c r="I106" s="2" t="n">
         <v>2010</v>
       </c>
-      <c r="J106" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K106" s="12" t="n">
-        <v>9</v>
+      <c r="J106" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K106" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="L106" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="M106" s="12" t="n">
-        <v>9</v>
+      <c r="M106" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="N106" s="11" t="n">
         <v>8</v>
       </c>
       <c r="O106" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="P106" s="7" t="inlineStr">
         <is>
@@ -8359,7 +8359,7 @@
       <c r="Q106" s="2" t="inlineStr"/>
       <c r="R106" s="2" t="inlineStr">
         <is>
-          <t>Detroit's avant-garde MC. Schizophrenic flows and surreal imagery.</t>
+          <t>Arc from frat-rap to deeply personal jazz introspection. 'Swimming' a peak.</t>
         </is>
       </c>
     </row>
@@ -8369,17 +8369,17 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>MH</t>
+          <t>JD2</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Mac Miller</t>
+          <t>JID</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -8394,44 +8394,48 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Pittsburgh Soul Rap</t>
+          <t>Atlanta Jazz Rap</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Rostrum</t>
+          <t>Dreamville</t>
         </is>
       </c>
       <c r="I107" s="2" t="n">
-        <v>2010</v>
-      </c>
-      <c r="J107" s="10" t="n">
-        <v>7</v>
+        <v>2017</v>
+      </c>
+      <c r="J107" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="K107" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L107" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M107" s="10" t="n">
-        <v>7</v>
+      <c r="L107" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M107" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="N107" s="11" t="n">
         <v>8</v>
       </c>
       <c r="O107" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="P107" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q107" s="2" t="inlineStr"/>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P107" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q107" s="2" t="inlineStr">
+        <is>
+          <t>Late-decade emergence; critical acclaim building; may rescore upward</t>
+        </is>
+      </c>
       <c r="R107" s="2" t="inlineStr">
         <is>
-          <t>Arc from frat-rap to deeply personal jazz introspection. 'Swimming' a peak.</t>
+          <t>Atlanta's most technically gifted rapper. 'DiCaprio 2' showed full potential.</t>
         </is>
       </c>
     </row>
@@ -8441,17 +8445,17 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>JD2</t>
+          <t>CD</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>JID</t>
+          <t>Cardi B</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -8461,53 +8465,49 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Jazz Rap</t>
+          <t>Bronx Trap Pop</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Dreamville</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="I108" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J108" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="K108" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L108" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M108" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N108" s="11" t="n">
-        <v>8</v>
+        <v>2018</v>
+      </c>
+      <c r="J108" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K108" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L108" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M108" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N108" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O108" s="6" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="P108" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q108" s="2" t="inlineStr">
-        <is>
-          <t>Late-decade emergence; critical acclaim building; may rescore upward</t>
-        </is>
-      </c>
+        <v>5.6</v>
+      </c>
+      <c r="P108" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q108" s="2" t="inlineStr"/>
       <c r="R108" s="2" t="inlineStr">
         <is>
-          <t>Atlanta's most technically gifted rapper. 'DiCaprio 2' showed full potential.</t>
+          <t>Unfiltered Bronx personality. Cultural force exceeds lyrical architecture.</t>
         </is>
       </c>
     </row>
@@ -8517,69 +8517,73 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>PG</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Cardi B</t>
+          <t>Polo G</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>2010s</t>
+          <t>2020s</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Bronx Trap Pop</t>
+          <t>Chicago Melodic Trap</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="I109" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J109" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K109" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L109" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M109" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N109" s="5" t="n">
-        <v>4</v>
+        <v>2019</v>
+      </c>
+      <c r="J109" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K109" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L109" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M109" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N109" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O109" s="6" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="P109" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q109" s="2" t="inlineStr"/>
+        <v>7.2</v>
+      </c>
+      <c r="P109" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q109" s="2" t="inlineStr">
+        <is>
+          <t>Recent emergence; trajectory still forming</t>
+        </is>
+      </c>
       <c r="R109" s="2" t="inlineStr">
         <is>
-          <t>Unfiltered Bronx personality. Cultural force exceeds lyrical architecture.</t>
+          <t>Chicago's introspective melodic trap voice. Melancholy street memoir.</t>
         </is>
       </c>
     </row>
@@ -8589,17 +8593,17 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Polo G</t>
+          <t>Rod Wave</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
@@ -8609,39 +8613,39 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Chicago Melodic Trap</t>
+          <t>Florida Soul Trap</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Alamo</t>
         </is>
       </c>
       <c r="I110" s="2" t="n">
         <v>2019</v>
       </c>
-      <c r="J110" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K110" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L110" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M110" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N110" s="10" t="n">
-        <v>7</v>
+      <c r="J110" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K110" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L110" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M110" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N110" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="O110" s="6" t="n">
-        <v>7.2</v>
+        <v>5.6</v>
       </c>
       <c r="P110" s="14" t="inlineStr">
         <is>
@@ -8650,12 +8654,12 @@
       </c>
       <c r="Q110" s="2" t="inlineStr">
         <is>
-          <t>Recent emergence; trajectory still forming</t>
+          <t>Recent; critical consensus not yet settled</t>
         </is>
       </c>
       <c r="R110" s="2" t="inlineStr">
         <is>
-          <t>Chicago's introspective melodic trap voice. Melancholy street memoir.</t>
+          <t>Emotional vulnerability over technical precision. Florida pain made universal.</t>
         </is>
       </c>
     </row>
@@ -8665,12 +8669,12 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>DO</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Rod Wave</t>
+          <t>Doechii</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -8690,34 +8694,34 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Florida Soul Trap</t>
+          <t>Tampa Art Rap</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Alamo</t>
+          <t>Capitol</t>
         </is>
       </c>
       <c r="I111" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="J111" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K111" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L111" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M111" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N111" s="8" t="n">
-        <v>5</v>
+        <v>2021</v>
+      </c>
+      <c r="J111" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K111" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L111" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M111" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N111" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="O111" s="6" t="n">
-        <v>5.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="P111" s="14" t="inlineStr">
         <is>
@@ -8726,12 +8730,12 @@
       </c>
       <c r="Q111" s="2" t="inlineStr">
         <is>
-          <t>Recent; critical consensus not yet settled</t>
+          <t>Breakout recent; scoring may shift upward as body of work grows</t>
         </is>
       </c>
       <c r="R111" s="2" t="inlineStr">
         <is>
-          <t>Emotional vulnerability over technical precision. Florida pain made universal.</t>
+          <t>Tampa's theatrical polymath. Technical fire meets conceptual daring.</t>
         </is>
       </c>
     </row>
@@ -8741,12 +8745,12 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>DO</t>
+          <t>GG2</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Doechii</t>
+          <t>GloRilla</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -8761,53 +8765,53 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Tampa Art Rap</t>
+          <t>Memphis Trap</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Capitol</t>
+          <t>CMG</t>
         </is>
       </c>
       <c r="I112" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="J112" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K112" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L112" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M112" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N112" s="12" t="n">
-        <v>9</v>
+        <v>2022</v>
+      </c>
+      <c r="J112" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K112" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L112" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M112" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N112" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O112" s="6" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="P112" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
+        <v>4.8</v>
+      </c>
+      <c r="P112" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="Q112" s="2" t="inlineStr">
         <is>
-          <t>Breakout recent; scoring may shift upward as body of work grows</t>
+          <t>Very recent; limited critical record; commercial impact clear</t>
         </is>
       </c>
       <c r="R112" s="2" t="inlineStr">
         <is>
-          <t>Tampa's theatrical polymath. Technical fire meets conceptual daring.</t>
+          <t>Memphis energy, unfiltered personality. New Southern feminism in party form.</t>
         </is>
       </c>
     </row>
@@ -8817,12 +8821,12 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>GG2</t>
+          <t>GN</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>GloRilla</t>
+          <t>Gunna</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -8837,53 +8841,53 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Trap/Drill</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Memphis Trap</t>
+          <t>Atlanta Melodic Trap</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>CMG</t>
+          <t>Young Stoner Life</t>
         </is>
       </c>
       <c r="I113" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="J113" s="8" t="n">
-        <v>5</v>
+        <v>2018</v>
+      </c>
+      <c r="J113" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="K113" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="L113" s="8" t="n">
-        <v>5</v>
+      <c r="L113" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="M113" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="N113" s="5" t="n">
-        <v>4</v>
+      <c r="N113" s="3" t="n">
+        <v>3</v>
       </c>
       <c r="O113" s="6" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="P113" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
+        <v>4.2</v>
+      </c>
+      <c r="P113" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="Q113" s="2" t="inlineStr">
         <is>
-          <t>Very recent; limited critical record; commercial impact clear</t>
+          <t>Significant commercial presence; thin critical analysis</t>
         </is>
       </c>
       <c r="R113" s="2" t="inlineStr">
         <is>
-          <t>Memphis energy, unfiltered personality. New Southern feminism in party form.</t>
+          <t>Melodic luxury trap. Vibe and aesthetic are the art.</t>
         </is>
       </c>
     </row>
@@ -8893,12 +8897,12 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>GN</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Gunna</t>
+          <t>Lil Baby</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -8913,39 +8917,39 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>Trap/Drill</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Melodic Trap</t>
+          <t>Atlanta Slime Trap</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Young Stoner Life</t>
+          <t>Quality Control</t>
         </is>
       </c>
       <c r="I114" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J114" s="5" t="n">
-        <v>4</v>
+        <v>2017</v>
+      </c>
+      <c r="J114" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="K114" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="L114" s="5" t="n">
-        <v>4</v>
+      <c r="L114" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="M114" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="N114" s="3" t="n">
-        <v>3</v>
+      <c r="N114" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="O114" s="6" t="n">
-        <v>4.2</v>
+        <v>5.2</v>
       </c>
       <c r="P114" s="14" t="inlineStr">
         <is>
@@ -8954,12 +8958,12 @@
       </c>
       <c r="Q114" s="2" t="inlineStr">
         <is>
-          <t>Significant commercial presence; thin critical analysis</t>
+          <t>Recent; commercial dominance clear; critical depth forming</t>
         </is>
       </c>
       <c r="R114" s="2" t="inlineStr">
         <is>
-          <t>Melodic luxury trap. Vibe and aesthetic are the art.</t>
+          <t>Authentic street narrator. Storytelling grounded in lived experience.</t>
         </is>
       </c>
     </row>
@@ -8969,17 +8973,17 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>BT</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Lil Baby</t>
+          <t>Benny the Butcher</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
@@ -8994,48 +8998,44 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Slime Trap</t>
+          <t>Buffalo Boom Bap</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Quality Control</t>
+          <t>Griselda</t>
         </is>
       </c>
       <c r="I115" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J115" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K115" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L115" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M115" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N115" s="8" t="n">
-        <v>5</v>
+        <v>2012</v>
+      </c>
+      <c r="J115" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K115" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L115" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="M115" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N115" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O115" s="6" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="P115" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q115" s="2" t="inlineStr">
-        <is>
-          <t>Recent; commercial dominance clear; critical depth forming</t>
-        </is>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="P115" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q115" s="2" t="inlineStr"/>
       <c r="R115" s="2" t="inlineStr">
         <is>
-          <t>Authentic street narrator. Storytelling grounded in lived experience.</t>
+          <t>Griselda's lyrical backbone. Buffalo street narratives with East Coast precision.</t>
         </is>
       </c>
     </row>
@@ -9045,17 +9045,17 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>BT</t>
+          <t>OM</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Benny the Butcher</t>
+          <t>Offset</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -9065,49 +9065,53 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Trap/Drill</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Buffalo Boom Bap</t>
+          <t>Migos Solo Trap</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Griselda</t>
+          <t>Quality Control</t>
         </is>
       </c>
       <c r="I116" s="2" t="n">
-        <v>2012</v>
-      </c>
-      <c r="J116" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K116" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L116" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="M116" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N116" s="10" t="n">
-        <v>7</v>
+        <v>2017</v>
+      </c>
+      <c r="J116" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K116" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L116" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M116" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N116" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O116" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="P116" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q116" s="2" t="inlineStr"/>
+        <v>5</v>
+      </c>
+      <c r="P116" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q116" s="2" t="inlineStr">
+        <is>
+          <t>Solo career emerging post-Migos; scoring tentative</t>
+        </is>
+      </c>
       <c r="R116" s="2" t="inlineStr">
         <is>
-          <t>Griselda's lyrical backbone. Buffalo street narratives with East Coast precision.</t>
+          <t>Migos' most lyrical member. Flow variation and delivery standout in trap context.</t>
         </is>
       </c>
     </row>
@@ -9117,17 +9121,17 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>ST</t>
+          <t>KD</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Stormzy</t>
+          <t>Kenny Mason</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -9137,21 +9141,21 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Political</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>UK Grime/Gospel</t>
+          <t>Atlanta Punk Rap</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>#Merky</t>
+          <t>RCA Records</t>
         </is>
       </c>
       <c r="I117" s="2" t="n">
-        <v>2015</v>
+        <v>2019</v>
       </c>
       <c r="J117" s="10" t="n">
         <v>7</v>
@@ -9165,21 +9169,25 @@
       <c r="M117" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="N117" s="11" t="n">
-        <v>8</v>
+      <c r="N117" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O117" s="6" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="P117" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q117" s="2" t="inlineStr"/>
+        <v>7</v>
+      </c>
+      <c r="P117" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q117" s="2" t="inlineStr">
+        <is>
+          <t>Limited documentation; critical buzz building in underground circles</t>
+        </is>
+      </c>
       <c r="R117" s="2" t="inlineStr">
         <is>
-          <t>UK grime's political conscience. Authenticity and ambition fused.</t>
+          <t>Atlanta's punk-rap hybrid. Unconventional tonal range.</t>
         </is>
       </c>
     </row>
@@ -9189,12 +9197,12 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>OM</t>
+          <t>LT</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Offset</t>
+          <t>Latto</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -9209,39 +9217,39 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Trap/Drill</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Migos Solo Trap</t>
+          <t>Atlanta Female Trap</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Quality Control</t>
+          <t>RCA</t>
         </is>
       </c>
       <c r="I118" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J118" s="8" t="n">
+        <v>2019</v>
+      </c>
+      <c r="J118" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K118" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L118" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M118" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="N118" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="K118" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L118" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="M118" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N118" s="5" t="n">
-        <v>4</v>
-      </c>
       <c r="O118" s="6" t="n">
-        <v>5</v>
+        <v>5.8</v>
       </c>
       <c r="P118" s="14" t="inlineStr">
         <is>
@@ -9250,12 +9258,12 @@
       </c>
       <c r="Q118" s="2" t="inlineStr">
         <is>
-          <t>Solo career emerging post-Migos; scoring tentative</t>
+          <t>Recent; commercial trajectory clearer than critical consensus</t>
         </is>
       </c>
       <c r="R118" s="2" t="inlineStr">
         <is>
-          <t>Migos' most lyrical member. Flow variation and delivery standout in trap context.</t>
+          <t>Atlanta's female trap voice. Technical skill often underestimated.</t>
         </is>
       </c>
     </row>
@@ -9265,17 +9273,17 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>KD</t>
+          <t>SR</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Kenny Mason</t>
+          <t>Smino</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -9290,48 +9298,48 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Punk Rap</t>
+          <t>St. Louis Jazz Rap</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>RCA Records</t>
+          <t>Zero Fatigue</t>
         </is>
       </c>
       <c r="I119" s="2" t="n">
-        <v>2019</v>
+        <v>2017</v>
       </c>
       <c r="J119" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="K119" s="10" t="n">
-        <v>7</v>
+      <c r="K119" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="L119" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="M119" s="10" t="n">
-        <v>7</v>
+      <c r="M119" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="N119" s="10" t="n">
         <v>7</v>
       </c>
       <c r="O119" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="P119" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
+        <v>7.4</v>
+      </c>
+      <c r="P119" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="Q119" s="2" t="inlineStr">
         <is>
-          <t>Limited documentation; critical buzz building in underground circles</t>
+          <t>Critical darling in jazz-rap circles; broader recognition still forming</t>
         </is>
       </c>
       <c r="R119" s="2" t="inlineStr">
         <is>
-          <t>Atlanta's punk-rap hybrid. Unconventional tonal range.</t>
+          <t>St. Louis's jazz-rap hybrid. Melodic and rhythmic sophistication.</t>
         </is>
       </c>
     </row>
@@ -9341,17 +9349,17 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>LT</t>
+          <t>PZ</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>Latto</t>
+          <t>Pusha T</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -9366,48 +9374,44 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>Atlanta Female Trap</t>
+          <t>Coke Rap Boom Bap</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>RCA</t>
+          <t>G.O.O.D.</t>
         </is>
       </c>
       <c r="I120" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="J120" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K120" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="L120" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M120" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="N120" s="8" t="n">
-        <v>5</v>
+        <v>2002</v>
+      </c>
+      <c r="J120" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K120" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L120" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M120" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N120" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O120" s="6" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="P120" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q120" s="2" t="inlineStr">
-        <is>
-          <t>Recent; commercial trajectory clearer than critical consensus</t>
-        </is>
-      </c>
+        <v>7.4</v>
+      </c>
+      <c r="P120" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q120" s="2" t="inlineStr"/>
       <c r="R120" s="2" t="inlineStr">
         <is>
-          <t>Atlanta's female trap voice. Technical skill often underestimated.</t>
+          <t>Cocaine rap's Rembrandt. 'Daytona' — maximum density, minimum waste.</t>
         </is>
       </c>
     </row>
@@ -9417,17 +9421,17 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>SR</t>
+          <t>TY</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>Smino</t>
+          <t>Tyler the Creator</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -9442,48 +9446,44 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>St. Louis Jazz Rap</t>
+          <t>Odd Future/Orchestral</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Zero Fatigue</t>
+          <t>Columbia</t>
         </is>
       </c>
       <c r="I121" s="2" t="n">
-        <v>2017</v>
+        <v>2009</v>
       </c>
       <c r="J121" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="K121" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L121" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M121" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N121" s="10" t="n">
-        <v>7</v>
+      <c r="K121" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="L121" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M121" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="N121" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="O121" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="P121" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q121" s="2" t="inlineStr">
-        <is>
-          <t>Critical darling in jazz-rap circles; broader recognition still forming</t>
-        </is>
-      </c>
+        <v>8.4</v>
+      </c>
+      <c r="P121" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q121" s="2" t="inlineStr"/>
       <c r="R121" s="2" t="inlineStr">
         <is>
-          <t>St. Louis's jazz-rap hybrid. Melodic and rhythmic sophistication.</t>
+          <t>'Igor' and 'Call Me If You Get Lost' — producer-auteur. Concept album mastery.</t>
         </is>
       </c>
     </row>
@@ -9493,12 +9493,12 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>PZ</t>
+          <t>AB2</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Pusha T</t>
+          <t>Armand Hammer</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -9513,49 +9513,53 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Coke Rap Boom Bap</t>
+          <t>Abstract Boom Bap</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>G.O.O.D.</t>
+          <t>Backwoodz</t>
         </is>
       </c>
       <c r="I122" s="2" t="n">
-        <v>2002</v>
+        <v>2013</v>
       </c>
       <c r="J122" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="K122" s="10" t="n">
-        <v>7</v>
+      <c r="K122" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="L122" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="M122" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N122" s="10" t="n">
-        <v>7</v>
+      <c r="M122" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="N122" s="11" t="n">
+        <v>8</v>
       </c>
       <c r="O122" s="6" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="P122" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q122" s="2" t="inlineStr"/>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P122" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
+          <t>Critical underground darling; thin mainstream documentation</t>
+        </is>
+      </c>
       <c r="R122" s="2" t="inlineStr">
         <is>
-          <t>Cocaine rap's Rembrandt. 'Daytona' — maximum density, minimum waste.</t>
+          <t>billy woods + ELUCID. The most demanding abstract rap being made today.</t>
         </is>
       </c>
     </row>
@@ -9565,17 +9569,17 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>TY</t>
+          <t>ZE</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Tyler the Creator</t>
+          <t>Zack Fox</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -9585,49 +9589,53 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>Odd Future/Orchestral</t>
+          <t>Comedy-Abstract Rap</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="I123" s="2" t="n">
-        <v>2009</v>
-      </c>
-      <c r="J123" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K123" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="L123" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M123" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="N123" s="12" t="n">
-        <v>9</v>
+        <v>2020</v>
+      </c>
+      <c r="J123" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="K123" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L123" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M123" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N123" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="O123" s="6" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="P123" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q123" s="2" t="inlineStr"/>
+        <v>6.4</v>
+      </c>
+      <c r="P123" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q123" s="2" t="inlineStr">
+        <is>
+          <t>Very recent; extremely limited critical record</t>
+        </is>
+      </c>
       <c r="R123" s="2" t="inlineStr">
         <is>
-          <t>'Igor' and 'Call Me If You Get Lost' — producer-auteur. Concept album mastery.</t>
+          <t>Comedy-meets-rap. Formally interesting but body of work too small to score confidently.</t>
         </is>
       </c>
     </row>
@@ -9637,17 +9645,17 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>AB2</t>
+          <t>LI</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>Armand Hammer</t>
+          <t>Lil Durk</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
@@ -9657,39 +9665,39 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>Abstract Boom Bap</t>
+          <t>Chicago Melodic Trap</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Backwoodz</t>
+          <t>Only the Family</t>
         </is>
       </c>
       <c r="I124" s="2" t="n">
         <v>2013</v>
       </c>
-      <c r="J124" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K124" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="L124" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M124" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="N124" s="11" t="n">
-        <v>8</v>
+      <c r="J124" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K124" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L124" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="M124" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N124" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="O124" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>5.2</v>
       </c>
       <c r="P124" s="14" t="inlineStr">
         <is>
@@ -9698,12 +9706,12 @@
       </c>
       <c r="Q124" s="2" t="inlineStr">
         <is>
-          <t>Critical underground darling; thin mainstream documentation</t>
+          <t>Commercial dominance clear; critical depth limited</t>
         </is>
       </c>
       <c r="R124" s="2" t="inlineStr">
         <is>
-          <t>billy woods + ELUCID. The most demanding abstract rap being made today.</t>
+          <t>Chicago drill's most commercially consistent voice.</t>
         </is>
       </c>
     </row>
@@ -9713,12 +9721,12 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>ZE</t>
+          <t>KS2</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Zack Fox</t>
+          <t>Kodak Black</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
@@ -9733,53 +9741,53 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Comedy-Abstract Rap</t>
+          <t>Florida Trap</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Atlantic</t>
         </is>
       </c>
       <c r="I125" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="J125" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="K125" s="10" t="n">
-        <v>7</v>
+        <v>2014</v>
+      </c>
+      <c r="J125" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K125" s="8" t="n">
+        <v>5</v>
       </c>
       <c r="L125" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="M125" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N125" s="9" t="n">
-        <v>6</v>
+      <c r="M125" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N125" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O125" s="6" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="P125" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
+        <v>5</v>
+      </c>
+      <c r="P125" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="Q125" s="2" t="inlineStr">
         <is>
-          <t>Very recent; extremely limited critical record</t>
+          <t>Commercial success; thin critical framework; behavior clouds reception</t>
         </is>
       </c>
       <c r="R125" s="2" t="inlineStr">
         <is>
-          <t>Comedy-meets-rap. Formally interesting but body of work too small to score confidently.</t>
+          <t>Florida trap's most distinctive voice. Rough-edged regional authenticity.</t>
         </is>
       </c>
     </row>
@@ -9789,17 +9797,17 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>LI</t>
+          <t>RC</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>Lil Durk</t>
+          <t>Rapsody</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
@@ -9809,53 +9817,49 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Conscious/Lyrical</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Chicago Melodic Trap</t>
+          <t>North Carolina Soul Rap</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Only the Family</t>
+          <t>Jamla</t>
         </is>
       </c>
       <c r="I126" s="2" t="n">
-        <v>2013</v>
-      </c>
-      <c r="J126" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K126" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L126" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M126" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N126" s="8" t="n">
-        <v>5</v>
+        <v>2010</v>
+      </c>
+      <c r="J126" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K126" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L126" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M126" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="N126" s="12" t="n">
+        <v>9</v>
       </c>
       <c r="O126" s="6" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="P126" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q126" s="2" t="inlineStr">
-        <is>
-          <t>Commercial dominance clear; critical depth limited</t>
-        </is>
-      </c>
+        <v>8.199999999999999</v>
+      </c>
+      <c r="P126" s="7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q126" s="2" t="inlineStr"/>
       <c r="R126" s="2" t="inlineStr">
         <is>
-          <t>Chicago drill's most commercially consistent voice.</t>
+          <t>North Carolina's most complete female MC. Lyrical depth rivals any peer.</t>
         </is>
       </c>
     </row>
@@ -9865,12 +9869,12 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>KS2</t>
+          <t>MF2</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>Kodak Black</t>
+          <t>Mavi</t>
         </is>
       </c>
       <c r="D127" s="2" t="inlineStr">
@@ -9885,53 +9889,53 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>Florida Trap</t>
+          <t>Underground Abstract</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Atlantic</t>
+          <t>Secretly Canadian</t>
         </is>
       </c>
       <c r="I127" s="2" t="n">
-        <v>2014</v>
-      </c>
-      <c r="J127" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K127" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L127" s="9" t="n">
-        <v>6</v>
-      </c>
-      <c r="M127" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N127" s="5" t="n">
-        <v>4</v>
+        <v>2019</v>
+      </c>
+      <c r="J127" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K127" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L127" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M127" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N127" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O127" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="P127" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
+        <v>7.2</v>
+      </c>
+      <c r="P127" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="Q127" s="2" t="inlineStr">
         <is>
-          <t>Commercial success; thin critical framework; behavior clouds reception</t>
+          <t>Very limited critical documentation; underground following only</t>
         </is>
       </c>
       <c r="R127" s="2" t="inlineStr">
         <is>
-          <t>Florida trap's most distinctive voice. Rough-edged regional authenticity.</t>
+          <t>Charlotte underground. Dense introspective abstract rap. Watch this space.</t>
         </is>
       </c>
     </row>
@@ -9941,69 +9945,73 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>RC</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>Rapsody</t>
+          <t>Xzibit</t>
         </is>
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>2020s</t>
+          <t>Late 90s</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>North Carolina Soul Rap</t>
+          <t>Hard West Coast</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Jamla</t>
+          <t>Loud/Columbia</t>
         </is>
       </c>
       <c r="I128" s="2" t="n">
-        <v>2010</v>
-      </c>
-      <c r="J128" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="K128" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L128" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="M128" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="N128" s="12" t="n">
-        <v>9</v>
+        <v>1996</v>
+      </c>
+      <c r="J128" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K128" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L128" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M128" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N128" s="9" t="n">
+        <v>6</v>
       </c>
       <c r="O128" s="6" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="P128" s="7" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="Q128" s="2" t="inlineStr"/>
+        <v>6.8</v>
+      </c>
+      <c r="P128" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q128" s="2" t="inlineStr">
+        <is>
+          <t>Well-known but limited formal critical analysis</t>
+        </is>
+      </c>
       <c r="R128" s="2" t="inlineStr">
         <is>
-          <t>North Carolina's most complete female MC. Lyrical depth rivals any peer.</t>
+          <t>West Coast boom bap craftsman. More respected by peers than critics.</t>
         </is>
       </c>
     </row>
@@ -10013,17 +10021,17 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>MF2</t>
+          <t>SA</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>Mavi</t>
+          <t>Saweetie</t>
         </is>
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
@@ -10033,53 +10041,53 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Underground Abstract</t>
+          <t>Trap Pop</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Secretly Canadian</t>
+          <t>Warner</t>
         </is>
       </c>
       <c r="I129" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="J129" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K129" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L129" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M129" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N129" s="10" t="n">
-        <v>7</v>
+        <v>2018</v>
+      </c>
+      <c r="J129" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K129" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L129" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M129" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N129" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O129" s="6" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="P129" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
+        <v>4.8</v>
+      </c>
+      <c r="P129" s="14" t="inlineStr">
+        <is>
+          <t>M</t>
         </is>
       </c>
       <c r="Q129" s="2" t="inlineStr">
         <is>
-          <t>Very limited critical documentation; underground following only</t>
+          <t>Recent commercial success; limited critical depth</t>
         </is>
       </c>
       <c r="R129" s="2" t="inlineStr">
         <is>
-          <t>Charlotte underground. Dense introspective abstract rap. Watch this space.</t>
+          <t>Bay Area trap-pop. Ice Princess persona over lyrical substance.</t>
         </is>
       </c>
     </row>
@@ -10089,73 +10097,73 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>XP</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Xzibit</t>
+          <t>City Girls</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>Late 90s</t>
+          <t>2020s</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Hard West Coast</t>
+          <t>Miami Trap</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Loud/Columbia</t>
+          <t>Quality Control/Motown</t>
         </is>
       </c>
       <c r="I130" s="2" t="n">
-        <v>1996</v>
-      </c>
-      <c r="J130" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K130" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L130" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="M130" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N130" s="9" t="n">
-        <v>6</v>
+        <v>2018</v>
+      </c>
+      <c r="J130" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="K130" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="L130" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M130" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N130" s="5" t="n">
+        <v>4</v>
       </c>
       <c r="O130" s="6" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="P130" s="14" t="inlineStr">
-        <is>
-          <t>M</t>
+        <v>4.6</v>
+      </c>
+      <c r="P130" s="15" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="Q130" s="2" t="inlineStr">
         <is>
-          <t>Well-known but limited formal critical analysis</t>
+          <t>Limited critical record; cultural impact clearer than lyrical analysis</t>
         </is>
       </c>
       <c r="R130" s="2" t="inlineStr">
         <is>
-          <t>West Coast boom bap craftsman. More respected by peers than critics.</t>
+          <t>Miami's hedonistic party rap duo. Energy over craft.</t>
         </is>
       </c>
     </row>
@@ -10165,17 +10173,17 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>SA</t>
+          <t>MX</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Saweetie</t>
+          <t>Maxo Kream</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
@@ -10185,39 +10193,39 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>Trap Pop</t>
+          <t>Houston Narrative Trap</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>Warner</t>
+          <t>EMPIRE</t>
         </is>
       </c>
       <c r="I131" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="K131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="M131" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N131" s="5" t="n">
-        <v>4</v>
+        <v>2017</v>
+      </c>
+      <c r="J131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="K131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="L131" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="M131" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N131" s="10" t="n">
+        <v>7</v>
       </c>
       <c r="O131" s="6" t="n">
-        <v>4.8</v>
+        <v>7.4</v>
       </c>
       <c r="P131" s="14" t="inlineStr">
         <is>
@@ -10226,164 +10234,159 @@
       </c>
       <c r="Q131" s="2" t="inlineStr">
         <is>
-          <t>Recent commercial success; limited critical depth</t>
+          <t>Critical acclaim in narrative rap circles; limited mainstream documentation</t>
         </is>
       </c>
       <c r="R131" s="2" t="inlineStr">
         <is>
-          <t>Bay Area trap-pop. Ice Princess persona over lyrical substance.</t>
+          <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n">
+      <c r="A132" t="n">
         <v>131</v>
       </c>
-      <c r="B132" s="2" t="inlineStr">
-        <is>
-          <t>CI</t>
-        </is>
-      </c>
-      <c r="C132" s="2" t="inlineStr">
-        <is>
-          <t>City Girls</t>
-        </is>
-      </c>
-      <c r="D132" s="2" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="E132" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F132" s="2" t="inlineStr">
-        <is>
-          <t>Party/Pop</t>
-        </is>
-      </c>
-      <c r="G132" s="2" t="inlineStr">
-        <is>
-          <t>Miami Trap</t>
-        </is>
-      </c>
-      <c r="H132" s="2" t="inlineStr">
-        <is>
-          <t>Quality Control/Motown</t>
-        </is>
-      </c>
-      <c r="I132" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="J132" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="K132" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L132" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="M132" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N132" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O132" s="6" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="P132" s="15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="Q132" s="2" t="inlineStr">
-        <is>
-          <t>Limited critical record; cultural impact clearer than lyrical analysis</t>
-        </is>
-      </c>
-      <c r="R132" s="2" t="inlineStr">
-        <is>
-          <t>Miami's hedonistic party rap duo. Energy over craft.</t>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>The Roots</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Live-Band Boom Bap</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Geffen/MCA</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>1993</v>
+      </c>
+      <c r="J132" t="n">
+        <v>10</v>
+      </c>
+      <c r="K132" t="n">
+        <v>9</v>
+      </c>
+      <c r="L132" t="n">
+        <v>8</v>
+      </c>
+      <c r="M132" t="n">
+        <v>9</v>
+      </c>
+      <c r="N132" t="n">
+        <v>8</v>
+      </c>
+      <c r="O132" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>Philadelphia's live-band institution; Black Thought's relentless technique anchors a peerless catalog.</t>
         </is>
       </c>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n">
+      <c r="A133" t="n">
         <v>132</v>
       </c>
-      <c r="B133" s="2" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="C133" s="2" t="inlineStr">
-        <is>
-          <t>Maxo Kream</t>
-        </is>
-      </c>
-      <c r="D133" s="2" t="inlineStr">
-        <is>
-          <t>South</t>
-        </is>
-      </c>
-      <c r="E133" s="2" t="inlineStr">
-        <is>
-          <t>2020s</t>
-        </is>
-      </c>
-      <c r="F133" s="2" t="inlineStr">
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Beanie Sigel</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
         <is>
           <t>Gangsta/Street</t>
         </is>
       </c>
-      <c r="G133" s="2" t="inlineStr">
-        <is>
-          <t>Houston Narrative Trap</t>
-        </is>
-      </c>
-      <c r="H133" s="2" t="inlineStr">
-        <is>
-          <t>EMPIRE</t>
-        </is>
-      </c>
-      <c r="I133" s="2" t="n">
-        <v>2017</v>
-      </c>
-      <c r="J133" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="K133" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="L133" s="12" t="n">
-        <v>9</v>
-      </c>
-      <c r="M133" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="N133" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="O133" s="6" t="n">
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Soul Boom Bap</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Roc-A-Fella</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J133" t="n">
+        <v>8</v>
+      </c>
+      <c r="K133" t="n">
+        <v>7</v>
+      </c>
+      <c r="L133" t="n">
+        <v>8</v>
+      </c>
+      <c r="M133" t="n">
+        <v>7</v>
+      </c>
+      <c r="N133" t="n">
+        <v>7</v>
+      </c>
+      <c r="O133" t="n">
         <v>7.4</v>
       </c>
-      <c r="P133" s="14" t="inlineStr">
+      <c r="P133" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="Q133" s="2" t="inlineStr">
-        <is>
-          <t>Critical acclaim in narrative rap circles; limited mainstream documentation</t>
-        </is>
-      </c>
-      <c r="R133" s="2" t="inlineStr">
-        <is>
-          <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
+      <c r="Q133" t="inlineStr">
+        <is>
+          <t>Critically respected but thinly documented outside the Roc-A-Fella context.</t>
+        </is>
+      </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>Philadelphia's hardest pen. Street narratives carried with weight and conviction.</t>
         </is>
       </c>
     </row>
@@ -10393,12 +10396,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>BT3</t>
+          <t>UV</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Black Thought</t>
+          <t>Lil Uzi Vert</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10408,53 +10411,58 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Golden Age</t>
+          <t>2010s</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Experimental</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Live-Band Boom Bap</t>
+          <t>Rage/Trap</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>Geffen/MCA</t>
+          <t>Generation Now/Atlantic</t>
         </is>
       </c>
       <c r="I134" t="n">
-        <v>1993</v>
+        <v>2016</v>
       </c>
       <c r="J134" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K134" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L134" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M134" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N134" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="O134" t="n">
-        <v>8.800000000000001</v>
+        <v>5.8</v>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q134" t="inlineStr">
+        <is>
+          <t>Melodic rage star; influence on sound outweighs lyrical scholarship.</t>
         </is>
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>The Roots' engine and a consensus top-tier technician. Relentless breath control and rhyme density.</t>
+          <t>Genre-bending rage pioneer. Melody and energy over lyrical density.</t>
         </is>
       </c>
     </row>
@@ -10464,12 +10472,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>BS</t>
+          <t>FW</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Beanie Sigel</t>
+          <t>Freeway</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -10498,39 +10506,39 @@
         </is>
       </c>
       <c r="I135" t="n">
-        <v>2000</v>
+        <v>2003</v>
       </c>
       <c r="J135" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K135" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L135" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M135" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N135" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O135" t="n">
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>Critically respected but thinly documented outside the Roc-A-Fella context.</t>
+          <t>Limited critical record; respected within State Property/Roc-A-Fella circles.</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>Philadelphia's hardest pen. Street narratives carried with weight and conviction.</t>
+          <t>Distinctive raspy urgency and Philly grit. State Property standout.</t>
         </is>
       </c>
     </row>
@@ -10540,12 +10548,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>UV</t>
+          <t>EV</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Lil Uzi Vert</t>
+          <t>Eve</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10555,26 +10563,26 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2010s</t>
+          <t>2000s</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Experimental</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Rage/Trap</t>
+          <t>Ruff Ryders</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Generation Now/Atlantic</t>
+          <t>Ruff Ryders/Interscope</t>
         </is>
       </c>
       <c r="I136" t="n">
-        <v>2016</v>
+        <v>1999</v>
       </c>
       <c r="J136" t="n">
         <v>6</v>
@@ -10583,30 +10591,30 @@
         <v>6</v>
       </c>
       <c r="L136" t="n">
+        <v>6</v>
+      </c>
+      <c r="M136" t="n">
+        <v>6</v>
+      </c>
+      <c r="N136" t="n">
         <v>5</v>
-      </c>
-      <c r="M136" t="n">
-        <v>6</v>
-      </c>
-      <c r="N136" t="n">
-        <v>6</v>
       </c>
       <c r="O136" t="n">
         <v>5.8</v>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Melodic rage star; influence on sound outweighs lyrical scholarship.</t>
+          <t>Commercial success clearer than lyrical analysis.</t>
         </is>
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>Genre-bending rage pioneer. Melody and energy over lyrical density.</t>
+          <t>Ruff Ryders' First Lady. Charismatic crossover with Philly roots.</t>
         </is>
       </c>
     </row>
@@ -10616,44 +10624,44 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>FW</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Freeway</t>
+          <t>Da Brat</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>South</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2000s</t>
+          <t>Golden Age</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Soul Boom Bap</t>
+          <t>So So Def Bass</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Roc-A-Fella</t>
+          <t>So So Def</t>
         </is>
       </c>
       <c r="I137" t="n">
-        <v>2003</v>
+        <v>1994</v>
       </c>
       <c r="J137" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K137" t="n">
         <v>6</v>
@@ -10668,21 +10676,21 @@
         <v>5</v>
       </c>
       <c r="O137" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>Limited critical record; respected within State Property/Roc-A-Fella circles.</t>
+          <t>First female solo rapper to go platinum; under-analyzed lyrically.</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
         <is>
-          <t>Distinctive raspy urgency and Philly grit. State Property standout.</t>
+          <t>So So Def's breakout. First female solo rapper to go platinum.</t>
         </is>
       </c>
     </row>
@@ -10692,73 +10700,73 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>EV</t>
+          <t>TS2</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Eve</t>
+          <t>Too $hort</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2000s</t>
+          <t>Old School</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Ruff Ryders</t>
+          <t>Funk/Bass</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Ruff Ryders/Interscope</t>
+          <t>Jive/Dangerous Music</t>
         </is>
       </c>
       <c r="I138" t="n">
-        <v>1999</v>
+        <v>1987</v>
       </c>
       <c r="J138" t="n">
         <v>6</v>
       </c>
       <c r="K138" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L138" t="n">
         <v>6</v>
       </c>
       <c r="M138" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N138" t="n">
         <v>5</v>
       </c>
       <c r="O138" t="n">
-        <v>5.8</v>
+        <v>5.4</v>
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>M</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>Commercial success clearer than lyrical analysis.</t>
+          <t>Pioneer status outweighs lyrical-craft documentation.</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
         <is>
-          <t>Ruff Ryders' First Lady. Charismatic crossover with Philly roots.</t>
+          <t>Oakland pioneer and pimp-rap archetype. Influence over intricacy.</t>
         </is>
       </c>
     </row>
@@ -10768,17 +10776,17 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Da Brat</t>
+          <t>Del the Funky Homosapien</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>South</t>
+          <t>Bay Area</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -10788,39 +10796,39 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Abstract</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>So So Def Bass</t>
+          <t>Hieroglyphics</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>So So Def</t>
+          <t>Elektra/Hiero Imperium</t>
         </is>
       </c>
       <c r="I139" t="n">
-        <v>1994</v>
+        <v>1991</v>
       </c>
       <c r="J139" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K139" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L139" t="n">
         <v>6</v>
       </c>
       <c r="M139" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N139" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O139" t="n">
-        <v>5.8</v>
+        <v>7</v>
       </c>
       <c r="P139" t="inlineStr">
         <is>
@@ -10829,12 +10837,12 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>First female solo rapper to go platinum; under-analyzed lyrically.</t>
+          <t>Underground Hieroglyphics following; specialist critical attention.</t>
         </is>
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>So So Def's breakout. First female solo rapper to go platinum.</t>
+          <t>Hieroglyphics wordsmith. Quirky vocabulary and abstract wit.</t>
         </is>
       </c>
     </row>
@@ -10844,12 +10852,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>TS2</t>
+          <t>MD3</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Too $hort</t>
+          <t>Mac Dre</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -10859,32 +10867,32 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Old School</t>
+          <t>2000s</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Party/Pop</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Funk/Bass</t>
+          <t>Hyphy</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>Jive/Dangerous Music</t>
+          <t>Thizz Entertainment</t>
         </is>
       </c>
       <c r="I140" t="n">
-        <v>1987</v>
+        <v>1989</v>
       </c>
       <c r="J140" t="n">
         <v>6</v>
       </c>
       <c r="K140" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L140" t="n">
         <v>6</v>
@@ -10896,21 +10904,21 @@
         <v>5</v>
       </c>
       <c r="O140" t="n">
-        <v>5.4</v>
+        <v>5.6</v>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>L</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>Pioneer status outweighs lyrical-craft documentation.</t>
+          <t>Regional hyphy icon; limited national critical record.</t>
         </is>
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>Oakland pioneer and pimp-rap archetype. Influence over intricacy.</t>
+          <t>Hyphy movement godfather. Enduring Bay Area cult legend.</t>
         </is>
       </c>
     </row>
@@ -10920,59 +10928,59 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Del the Funky Homosapien</t>
+          <t>Royce da 5'9"</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>Midwest</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Golden Age</t>
+          <t>2000s</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Abstract</t>
+          <t>Conscious/Lyrical</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Hieroglyphics</t>
+          <t>Detroit Boom Bap</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Elektra/Hiero Imperium</t>
+          <t>Shady/Independent</t>
         </is>
       </c>
       <c r="I141" t="n">
-        <v>1991</v>
+        <v>2002</v>
       </c>
       <c r="J141" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K141" t="n">
         <v>8</v>
       </c>
       <c r="L141" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M141" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N141" t="n">
         <v>7</v>
       </c>
       <c r="O141" t="n">
-        <v>7</v>
+        <v>7.8</v>
       </c>
       <c r="P141" t="inlineStr">
         <is>
@@ -10981,12 +10989,12 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>Underground Hieroglyphics following; specialist critical attention.</t>
+          <t>Elite technician; documentation grew via Slaughterhouse and PRhyme.</t>
         </is>
       </c>
       <c r="R141" t="inlineStr">
         <is>
-          <t>Hieroglyphics wordsmith. Quirky vocabulary and abstract wit.</t>
+          <t>Detroit technician. Slaughterhouse and PRhyme cornerstone.</t>
         </is>
       </c>
     </row>
@@ -10996,73 +11004,68 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>MD3</t>
+          <t>KG</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Mac Dre</t>
+          <t>Kool G Rap</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2000s</t>
+          <t>Golden Age</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Party/Pop</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Hyphy</t>
+          <t>Boom Bap</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Thizz Entertainment</t>
+          <t>Cold Chillin'</t>
         </is>
       </c>
       <c r="I142" t="n">
         <v>1989</v>
       </c>
       <c r="J142" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K142" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L142" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M142" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N142" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O142" t="n">
-        <v>5.6</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="Q142" t="inlineStr">
-        <is>
-          <t>Regional hyphy icon; limited national critical record.</t>
+          <t>H</t>
         </is>
       </c>
       <c r="R142" t="inlineStr">
         <is>
-          <t>Hyphy movement godfather. Enduring Bay Area cult legend.</t>
+          <t>Mafioso-rap forefather. The multisyllabic blueprint for Nas, Biggie and Jay-Z.</t>
         </is>
       </c>
     </row>
@@ -11072,22 +11075,22 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>RM</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Royce da 5'9"</t>
+          <t>Redman</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Midwest</t>
+          <t>NYC</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2000s</t>
+          <t>Golden Age</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -11097,34 +11100,34 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Detroit Boom Bap</t>
+          <t>Funk Boom Bap</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Shady/Independent</t>
+          <t>Def Jam</t>
         </is>
       </c>
       <c r="I143" t="n">
-        <v>2002</v>
+        <v>1992</v>
       </c>
       <c r="J143" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K143" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L143" t="n">
         <v>7</v>
       </c>
       <c r="M143" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N143" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O143" t="n">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="P143" t="inlineStr">
         <is>
@@ -11133,12 +11136,12 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>Elite technician; documentation grew via Slaughterhouse and PRhyme.</t>
+          <t>Beloved and skilled; lyrical scholarship modest relative to peers.</t>
         </is>
       </c>
       <c r="R143" t="inlineStr">
         <is>
-          <t>Detroit technician. Slaughterhouse and PRhyme cornerstone.</t>
+          <t>Newark's funkiest. Effortless flow with comedic menace.</t>
         </is>
       </c>
     </row>
@@ -11148,12 +11151,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>KG</t>
+          <t>ME</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Kool G Rap</t>
+          <t>Method Man</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11163,53 +11166,58 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Golden Age</t>
+          <t>Late 90s</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Conscious/Lyrical</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Boom Bap</t>
+          <t>Wu-Tang</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>Cold Chillin'</t>
+          <t>Def Jam</t>
         </is>
       </c>
       <c r="I144" t="n">
-        <v>1989</v>
+        <v>1994</v>
       </c>
       <c r="J144" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K144" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L144" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M144" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N144" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O144" t="n">
-        <v>8.199999999999999</v>
+        <v>6.6</v>
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q144" t="inlineStr">
+        <is>
+          <t>Scored solo; Wu-Tang charisma vs pure-lyric metrics.</t>
         </is>
       </c>
       <c r="R144" t="inlineStr">
         <is>
-          <t>Mafioso-rap forefather. The multisyllabic blueprint for Nas, Biggie and Jay-Z.</t>
+          <t>Wu-Tang's charismatic star. Gravel-voiced hooks and grit.</t>
         </is>
       </c>
     </row>
@@ -11219,12 +11227,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>EP</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Redman</t>
+          <t>EPMD</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11253,25 +11261,25 @@
         </is>
       </c>
       <c r="I145" t="n">
-        <v>1992</v>
+        <v>1988</v>
       </c>
       <c r="J145" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N145" t="n">
         <v>6</v>
       </c>
       <c r="O145" t="n">
-        <v>7</v>
+        <v>6.2</v>
       </c>
       <c r="P145" t="inlineStr">
         <is>
@@ -11280,12 +11288,12 @@
       </c>
       <c r="Q145" t="inlineStr">
         <is>
-          <t>Beloved and skilled; lyrical scholarship modest relative to peers.</t>
+          <t>Influential funk-rap duo; understated lyrical documentation.</t>
         </is>
       </c>
       <c r="R145" t="inlineStr">
         <is>
-          <t>Newark's funkiest. Effortless flow with comedic menace.</t>
+          <t>Strictly Business. Laid-back funk and durable chemistry.</t>
         </is>
       </c>
     </row>
@@ -11295,41 +11303,41 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>ME</t>
+          <t>TG</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Method Man</t>
+          <t>The Game</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Late 90s</t>
+          <t>2000s</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Wu-Tang</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>Def Jam</t>
+          <t>Aftermath/G-Unit</t>
         </is>
       </c>
       <c r="I146" t="n">
-        <v>1994</v>
+        <v>2005</v>
       </c>
       <c r="J146" t="n">
         <v>7</v>
@@ -11338,7 +11346,7 @@
         <v>7</v>
       </c>
       <c r="L146" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M146" t="n">
         <v>7</v>
@@ -11347,7 +11355,7 @@
         <v>6</v>
       </c>
       <c r="O146" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
       <c r="P146" t="inlineStr">
         <is>
@@ -11356,12 +11364,12 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>Scored solo; Wu-Tang charisma vs pure-lyric metrics.</t>
+          <t>Commercially dominant; reference-heavy bars, mixed critical view.</t>
         </is>
       </c>
       <c r="R146" t="inlineStr">
         <is>
-          <t>Wu-Tang's charismatic star. Gravel-voiced hooks and grit.</t>
+          <t>Compton revivalist. The Documentary-era West Coast resurgence.</t>
         </is>
       </c>
     </row>
@@ -11371,59 +11379,59 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EP</t>
+          <t>IT</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>EPMD</t>
+          <t>Ice-T</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Golden Age</t>
+          <t>Old School</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Conscious/Lyrical</t>
+          <t>Gangsta/Street</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Funk Boom Bap</t>
+          <t>Electro/Funk</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Def Jam</t>
+          <t>Sire/Rhyme Syndicate</t>
         </is>
       </c>
       <c r="I147" t="n">
-        <v>1988</v>
+        <v>1987</v>
       </c>
       <c r="J147" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K147" t="n">
         <v>6</v>
       </c>
       <c r="L147" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M147" t="n">
         <v>6</v>
       </c>
       <c r="N147" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O147" t="n">
-        <v>6.2</v>
+        <v>6.4</v>
       </c>
       <c r="P147" t="inlineStr">
         <is>
@@ -11432,12 +11440,12 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Influential funk-rap duo; understated lyrical documentation.</t>
+          <t>Gangsta-rap pioneer; influence and narrative over technical metrics.</t>
         </is>
       </c>
       <c r="R147" t="inlineStr">
         <is>
-          <t>Strictly Business. Laid-back funk and durable chemistry.</t>
+          <t>Gangsta-rap originator. Street reportage before the template existed.</t>
         </is>
       </c>
     </row>
@@ -11447,12 +11455,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>TG</t>
+          <t>NH</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>The Game</t>
+          <t>Nipsey Hussle</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11462,12 +11470,12 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2000s</t>
+          <t>2010s</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Gangsta/Street</t>
+          <t>Conscious/Street</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -11477,11 +11485,11 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>Aftermath/G-Unit</t>
+          <t>All Money In/Atlantic</t>
         </is>
       </c>
       <c r="I148" t="n">
-        <v>2005</v>
+        <v>2010</v>
       </c>
       <c r="J148" t="n">
         <v>7</v>
@@ -11496,10 +11504,10 @@
         <v>7</v>
       </c>
       <c r="N148" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O148" t="n">
-        <v>6.8</v>
+        <v>7</v>
       </c>
       <c r="P148" t="inlineStr">
         <is>
@@ -11508,12 +11516,12 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>Commercially dominant; reference-heavy bars, mixed critical view.</t>
+          <t>Posthumous reappraisal ongoing; entrepreneurial legacy prominent.</t>
         </is>
       </c>
       <c r="R148" t="inlineStr">
         <is>
-          <t>Compton revivalist. The Documentary-era West Coast resurgence.</t>
+          <t>Crenshaw's marathon. Street wisdom and self-determination.</t>
         </is>
       </c>
     </row>
@@ -11523,12 +11531,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>IT</t>
+          <t>DQ</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Ice-T</t>
+          <t>DJ Quik</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -11538,7 +11546,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Old School</t>
+          <t>Golden Age</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -11548,34 +11556,34 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Electro/Funk</t>
+          <t>G-Funk</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>Sire/Rhyme Syndicate</t>
+          <t>Profile</t>
         </is>
       </c>
       <c r="I149" t="n">
-        <v>1987</v>
+        <v>1991</v>
       </c>
       <c r="J149" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K149" t="n">
         <v>6</v>
       </c>
       <c r="L149" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M149" t="n">
         <v>6</v>
       </c>
       <c r="N149" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O149" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="P149" t="inlineStr">
         <is>
@@ -11584,162 +11592,10 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>Gangsta-rap pioneer; influence and narrative over technical metrics.</t>
+          <t>Revered as a producer; underrated as a lyricist.</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
-        <is>
-          <t>Gangsta-rap originator. Street reportage before the template existed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="n">
-        <v>149</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>NH</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Nipsey Hussle</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>2010s</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>Conscious/Street</t>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>West Coast</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr">
-        <is>
-          <t>All Money In/Atlantic</t>
-        </is>
-      </c>
-      <c r="I150" t="n">
-        <v>2010</v>
-      </c>
-      <c r="J150" t="n">
-        <v>7</v>
-      </c>
-      <c r="K150" t="n">
-        <v>7</v>
-      </c>
-      <c r="L150" t="n">
-        <v>7</v>
-      </c>
-      <c r="M150" t="n">
-        <v>7</v>
-      </c>
-      <c r="N150" t="n">
-        <v>7</v>
-      </c>
-      <c r="O150" t="n">
-        <v>7</v>
-      </c>
-      <c r="P150" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q150" t="inlineStr">
-        <is>
-          <t>Posthumous reappraisal ongoing; entrepreneurial legacy prominent.</t>
-        </is>
-      </c>
-      <c r="R150" t="inlineStr">
-        <is>
-          <t>Crenshaw's marathon. Street wisdom and self-determination.</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="n">
-        <v>150</v>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>DQ</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>DJ Quik</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Golden Age</t>
-        </is>
-      </c>
-      <c r="F151" t="inlineStr">
-        <is>
-          <t>Gangsta/Street</t>
-        </is>
-      </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>G-Funk</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>Profile</t>
-        </is>
-      </c>
-      <c r="I151" t="n">
-        <v>1991</v>
-      </c>
-      <c r="J151" t="n">
-        <v>7</v>
-      </c>
-      <c r="K151" t="n">
-        <v>6</v>
-      </c>
-      <c r="L151" t="n">
-        <v>6</v>
-      </c>
-      <c r="M151" t="n">
-        <v>6</v>
-      </c>
-      <c r="N151" t="n">
-        <v>6</v>
-      </c>
-      <c r="O151" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="P151" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="Q151" t="inlineStr">
-        <is>
-          <t>Revered as a producer; underrated as a lyricist.</t>
-        </is>
-      </c>
-      <c r="R151" t="inlineStr">
         <is>
           <t>G-funk auteur. Producer-rapper with effortless West Coast bounce.</t>
         </is>

</xml_diff>

<commit_message>
Add Compounds table for groups; tidy region UI
- New "Type" column (Element/Compound) tags the 26 groups vs 121 solo acts
- Template now renders a second "Compounds" periodic table below the main
  one (groups & crews), sharing styling, era grouping, region colors,
  filters, and the artist modal. Main-table stats/subtitle now count
  Elements; Compounds section shows its own count.
- This cleanly resolves the group-vs-individual overlap: Wu-Tang lives in
  Compounds while Method Man/Ghostface/Raekwon remain Elements.
- Remove now-empty International/UK chips from the legend, region filter,
  and add/edit forms (US-only scope)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011ryeTrcgR6UHuGZSMwMMAG
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -580,7 +580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R148"/>
+  <dimension ref="A1:S148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -694,6 +694,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -766,6 +771,11 @@
           <t>Father of hip-hop. Innovated breakbeat DJing. His voice was the party, not the page.</t>
         </is>
       </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -838,6 +848,11 @@
           <t>Turntablism pioneer. Set template for social commentary rap.</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -910,6 +925,11 @@
           <t>'The Message' — first truly serious rap lyric. Dark imagery of urban decay.</t>
         </is>
       </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -982,6 +1002,11 @@
           <t>Brought hip-hop mainstream with 'Rapper's Delight'.</t>
         </is>
       </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1054,6 +1079,11 @@
           <t>'Planet Rock' visionary. Pan-African ideology in party form.</t>
         </is>
       </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1126,6 +1156,11 @@
           <t>Def Jam's first star. Swagger as technique.</t>
         </is>
       </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1198,6 +1233,11 @@
           <t>Merged rock and rap. Iconic minimalism.</t>
         </is>
       </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1268,6 +1308,11 @@
       <c r="R9" s="2" t="inlineStr">
         <is>
           <t>Frenetic cultural collage. Grew into genuine experimental sophistication.</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Compound</t>
         </is>
       </c>
     </row>
@@ -1342,6 +1387,11 @@
           <t>'The Teacha.' Hip-hop philosopher-MC.</t>
         </is>
       </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1414,6 +1464,11 @@
           <t>Maximum political rage. Bomb Squad production as sonic warfare.</t>
         </is>
       </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1490,6 +1545,11 @@
           <t>Pioneer female MC. Battle rap legend at age 14. Foundational for women in hip-hop.</t>
         </is>
       </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1566,6 +1626,11 @@
           <t>First solo female rapper to release a full album. Sharp, authoritative delivery.</t>
         </is>
       </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1642,6 +1707,11 @@
           <t>Philadelphia proto-gangsta rapper. Predates N.W.A's gangsta template.</t>
         </is>
       </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1718,6 +1788,11 @@
           <t>First rap group Grammy-nominated. Female-fronted electro-hop novelty hit.</t>
         </is>
       </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1794,6 +1869,11 @@
           <t>Early electro-rap crossover. Bridged disco and hip-hop aesthetics.</t>
         </is>
       </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1870,6 +1950,11 @@
           <t>Human beatbox pioneer. 'La Di Da Di' a canonical party rap text.</t>
         </is>
       </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1942,6 +2027,11 @@
           <t>Master storyteller. Cockney-inflected delivery, vivid street fables.</t>
         </is>
       </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -2018,6 +2108,11 @@
           <t>Storytelling peer to Slick Rick. Underrated narrative rapper.</t>
         </is>
       </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2090,6 +2185,11 @@
           <t>Velvet-glove delivery hiding razor-sharp multisyllabic patterns.</t>
         </is>
       </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2162,6 +2262,11 @@
           <t>Invented internal rhyme as default mode. The God MC.</t>
         </is>
       </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2234,6 +2339,11 @@
           <t>Regal feminist authority. Foundational for women in rap.</t>
         </is>
       </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2306,6 +2416,11 @@
           <t>Invented gangsta rap. Vérité street journalism.</t>
         </is>
       </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2378,6 +2493,11 @@
           <t>N.W.A's sharpest writer. Furious precision.</t>
         </is>
       </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2450,6 +2570,11 @@
           <t>Playful polymaths. Vast vocabulary with absurdist wit.</t>
         </is>
       </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2522,6 +2647,11 @@
           <t>Q-Tip's conversational genius. Jazz improvisation in verse.</t>
         </is>
       </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2594,6 +2724,11 @@
           <t>'Illmatic' distilled Queensbridge into literary art.</t>
         </is>
       </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2666,6 +2801,11 @@
           <t>Greatest natural storyteller. Cinematic scenes, effortless charisma.</t>
         </is>
       </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2738,6 +2878,11 @@
           <t>Nine MCs, nine styles. Martial mythology meets grim NY street.</t>
         </is>
       </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2810,6 +2955,11 @@
           <t>Flow as personality. Delivery transcends lyrical content.</t>
         </is>
       </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2882,6 +3032,11 @@
           <t>Producer-first. Lyricism secondary to sonic architecture.</t>
         </is>
       </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2954,6 +3109,11 @@
           <t>Acrobatic, joyful wordplay. LA's alternative answer to De La Soul.</t>
         </is>
       </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3026,6 +3186,11 @@
           <t>Prodigy's paranoid poetry over Havoc's glacial loops.</t>
         </is>
       </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3098,6 +3263,11 @@
           <t>Slang inventor. Vocabulary innovation as primary art form.</t>
         </is>
       </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3174,6 +3344,11 @@
           <t>Pete Rock's jazz-inflected production plus CL Smooth's introspective flows.</t>
         </is>
       </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3246,6 +3421,11 @@
           <t>Guru's monotone wisdom over DJ Premier's crate-dug perfection.</t>
         </is>
       </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3322,6 +3502,11 @@
           <t>5 Percenter theology meets Afrocentric fury. Sadat X and Grand Puba.</t>
         </is>
       </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3398,6 +3583,11 @@
           <t>Black nationalist imagery and Afrocentric symbolism at maximum.</t>
         </is>
       </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3470,6 +3660,11 @@
           <t>Punchline architect. Harlem's greatest. Wordplay density rivals anyone.</t>
         </is>
       </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3542,6 +3737,11 @@
           <t>Pioneered Southern horror-gangsta. Scarface's lyrical foundation.</t>
         </is>
       </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3618,6 +3818,11 @@
           <t>LA's jazz-rap underground. Aceyalone among the most technically gifted MCs ever.</t>
         </is>
       </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3694,6 +3899,11 @@
           <t>Cool jazz-rap fusion. Ladybug Mecca one of the era's sharpest female voices.</t>
         </is>
       </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3770,6 +3980,11 @@
           <t>Launched Busta Rhymes. Charlie Brown and Dinco D also strong voices.</t>
         </is>
       </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3842,6 +4057,11 @@
           <t>Hyper-kinetic delivery and flow complexity. One of the fastest MCs ever.</t>
         </is>
       </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -3914,6 +4134,11 @@
           <t>Raw emotional intelligence. Political rage and personal vulnerability.</t>
         </is>
       </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -3986,6 +4211,11 @@
           <t>Effortless mastery. Hustler's autobiography as album architecture.</t>
         </is>
       </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -4058,6 +4288,11 @@
           <t>Most technically precise rapper. Internal rhyme density off the charts.</t>
         </is>
       </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -4130,6 +4365,11 @@
           <t>Primal confessional fury. Power through raw emotional delivery.</t>
         </is>
       </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -4202,6 +4442,11 @@
           <t>'Miseducation' — radical emotional honesty + technical precision.</t>
         </is>
       </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -4274,6 +4519,11 @@
           <t>Flow as futurist sculpture. Rhythm manipulation over traditional lyricism.</t>
         </is>
       </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -4346,6 +4596,11 @@
           <t>'Black on Both Sides' — blues, jazz, politics in one voice.</t>
         </is>
       </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -4418,6 +4673,11 @@
           <t>Brooklyn's dense intellectual. Every bar packed with history.</t>
         </is>
       </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -4490,6 +4750,11 @@
           <t>Andre 3000: genre-defying poet. Big Boi: underrated technical master.</t>
         </is>
       </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -4562,6 +4827,11 @@
           <t>Mogul over MC. Influence is business, not bars.</t>
         </is>
       </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -4638,6 +4908,11 @@
           <t>Pink fur and slant rhymes. Harlem's most stylistically eccentric MC.</t>
         </is>
       </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -4714,6 +4989,11 @@
           <t>Aggressive feminine sexuality as lyrical weapon. Def Jam's answer to Lil Kim.</t>
         </is>
       </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -4786,6 +5066,11 @@
           <t>Radical sexual candor. Graphic feminism that rewrote what women could say in rap.</t>
         </is>
       </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -4862,6 +5147,11 @@
           <t>Cash Money's first star. New Orleans bounce meets street narrative.</t>
         </is>
       </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -4938,6 +5228,11 @@
           <t>Battle rap legend. Technical skill occasionally undermined by ego.</t>
         </is>
       </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -5014,6 +5309,11 @@
           <t>Philadelphia underground. Vinnie Paz's dense, conspiratorial lyricism.</t>
         </is>
       </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -5086,6 +5386,11 @@
           <t>First Latin rapper to go platinum solo. Multisyllabic rhyme virtuoso.</t>
         </is>
       </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -5162,6 +5467,11 @@
           <t>One of the era's most underrated lyricists. 'Doe or Die' (1995) a classic; his 'Life's a Bitch' verse is all-time.</t>
         </is>
       </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -5234,6 +5544,11 @@
           <t>Conceptual ambition as primary engine. Each album a reinvention.</t>
         </is>
       </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -5306,6 +5621,11 @@
           <t>Simile machine at peak. Abstract metaphor-stacking as freestyle sport.</t>
         </is>
       </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -5378,6 +5698,11 @@
           <t>King of the South. Trap's emotional architect.</t>
         </is>
       </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -5450,6 +5775,11 @@
           <t>Vibe and charisma over craft. Trap music's spiritual godfather.</t>
         </is>
       </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -5522,6 +5852,11 @@
           <t>Stream-of-consciousness genius. Dense slang, vivid scene-painting.</t>
         </is>
       </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -5594,6 +5929,11 @@
           <t>The supervillain. Labyrinths of internal rhyme no one has fully mapped.</t>
         </is>
       </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -5666,6 +6006,11 @@
           <t>Chicago's philosopher-MC. Ernie Barnes paintings in verse form.</t>
         </is>
       </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -5738,6 +6083,11 @@
           <t>Comic virtuosity. Punchline timing as precision instrument.</t>
         </is>
       </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -5810,6 +6160,11 @@
           <t>Trap's motivational orator. Delivery and charisma over craft.</t>
         </is>
       </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -5882,6 +6237,11 @@
           <t>Conceptually sui generis. 'Dumb It Down' a rebuke of simplicity.</t>
         </is>
       </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -5954,6 +6314,11 @@
           <t>Houston's great novelist. Psychological interior in gangsta rap.</t>
         </is>
       </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -6026,6 +6391,11 @@
           <t>NLP-verified largest unique vocabulary in rap. Dense abstract imagery.</t>
         </is>
       </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -6102,6 +6472,11 @@
           <t>Gravelly-voiced Yonkers MC. Punchline economy and street credibility.</t>
         </is>
       </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -6174,6 +6549,11 @@
           <t>Bulletproof charisma. Street narrative over lyrical complexity.</t>
         </is>
       </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -6250,6 +6630,11 @@
           <t>Oscar-winning Southern horror-rap. Pioneered the dark triplet flow.</t>
         </is>
       </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -6322,6 +6707,11 @@
           <t>Bun B and Pimp C. Texas's most complete rap duo.</t>
         </is>
       </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -6398,6 +6788,11 @@
           <t>Houston's street ambassador. Chopped-and-screwed delivery as identity.</t>
         </is>
       </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -6474,6 +6869,11 @@
           <t>LA underground legend. Freestyle Fellowship's most technically gifted MC.</t>
         </is>
       </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -6546,6 +6946,11 @@
           <t>'Only Built 4 Cuban Linx' — the Godfather Part II of rap albums.</t>
         </is>
       </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -6618,6 +7023,11 @@
           <t>Company Flow / Run The Jewels architect. Dystopian sonic vision.</t>
         </is>
       </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -6694,6 +7104,11 @@
           <t>Minneapolis conscious rapper. Raw emotional honesty over Ant's production.</t>
         </is>
       </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -6770,6 +7185,11 @@
           <t>Most politically radical rapper in the genre. Conspiracy and revolution.</t>
         </is>
       </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -6842,6 +7262,11 @@
           <t>The complete package. Every dimension at peak. Pulitzer Prize.</t>
         </is>
       </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -6914,6 +7339,11 @@
           <t>Working-class emotional intelligence. Deep narrative craft.</t>
         </is>
       </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -6986,6 +7416,11 @@
           <t>Melody over meaning. Vocal texture as primary instrument.</t>
         </is>
       </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -7058,6 +7493,11 @@
           <t>Emotional auto-tune as confession. Vibe over lyrical architecture.</t>
         </is>
       </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -7130,6 +7570,11 @@
           <t>Joyful complexity. Gospel cadences and Chicago love letters.</t>
         </is>
       </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -7202,6 +7647,11 @@
           <t>Compression and grief as poetics. Dense abstract imagery.</t>
         </is>
       </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -7274,6 +7724,11 @@
           <t>Visceral urgency. Philadelphia streets in raw kinetic delivery.</t>
         </is>
       </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -7346,6 +7801,11 @@
           <t>Aesthetic as content. Flow and texture over lyrical substance.</t>
         </is>
       </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -7418,6 +7878,11 @@
           <t>Technical precision and alter-ego theatrics. 'Monster' verse.</t>
         </is>
       </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -7490,6 +7955,11 @@
           <t>Deadpan sociologist. Minimalist language doing maximum structural work.</t>
         </is>
       </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -7562,6 +8032,11 @@
           <t>Mississippi throwback futurist. Southern soul and lyrical ambition fused.</t>
         </is>
       </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -7634,6 +8109,11 @@
           <t>El-P and Killer Mike. Most politically urgent rap duo since PE.</t>
         </is>
       </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -7706,6 +8186,11 @@
           <t>RTJ's political conscience. Atlanta's most morally serious MC.</t>
         </is>
       </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -7778,6 +8263,11 @@
           <t>Gary Indiana's finest. Technical gangsta rap with jazz-rap production.</t>
         </is>
       </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -7850,6 +8340,11 @@
           <t>Triplet flow inventors. Cultural influence far exceeds lyrical complexity.</t>
         </is>
       </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -7926,6 +8421,11 @@
           <t>Detroit MC. Punchlines over conceptual depth. 'One Man Can Change The World'.</t>
         </is>
       </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -8002,6 +8502,11 @@
           <t>'Whack World' — 15 one-minute songs as unified concept. Wholly original.</t>
         </is>
       </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -8074,6 +8579,11 @@
           <t>Chicago's most literary voice. Jazz cadences and political awakening.</t>
         </is>
       </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -8146,6 +8656,11 @@
           <t>'CARE FOR ME' — grief and Chicago violence as devastating concept album.</t>
         </is>
       </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -8218,6 +8733,11 @@
           <t>Detroit's avant-garde MC. Schizophrenic flows and surreal imagery.</t>
         </is>
       </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -8290,6 +8810,11 @@
           <t>Arc from frat-rap to deeply personal jazz introspection. 'Swimming' a peak.</t>
         </is>
       </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -8366,6 +8891,11 @@
           <t>Atlanta's most technically gifted rapper. 'DiCaprio 2' showed full potential.</t>
         </is>
       </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -8438,6 +8968,11 @@
           <t>Unfiltered Bronx personality. Cultural force exceeds lyrical architecture.</t>
         </is>
       </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -8514,6 +9049,11 @@
           <t>Chicago's introspective melodic trap voice. Melancholy street memoir.</t>
         </is>
       </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -8590,6 +9130,11 @@
           <t>Emotional vulnerability over technical precision. Florida pain made universal.</t>
         </is>
       </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -8666,6 +9211,11 @@
           <t>Tampa's theatrical polymath. Technical fire meets conceptual daring.</t>
         </is>
       </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -8742,6 +9292,11 @@
           <t>Memphis energy, unfiltered personality. New Southern feminism in party form.</t>
         </is>
       </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -8818,6 +9373,11 @@
           <t>Melodic luxury trap. Vibe and aesthetic are the art.</t>
         </is>
       </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -8894,6 +9454,11 @@
           <t>Authentic street narrator. Storytelling grounded in lived experience.</t>
         </is>
       </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -8966,6 +9531,11 @@
           <t>Griselda's lyrical backbone. Buffalo street narratives with East Coast precision.</t>
         </is>
       </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -9042,6 +9612,11 @@
           <t>Migos' most lyrical member. Flow variation and delivery standout in trap context.</t>
         </is>
       </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -9118,6 +9693,11 @@
           <t>Atlanta's punk-rap hybrid. Unconventional tonal range.</t>
         </is>
       </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -9194,6 +9774,11 @@
           <t>Atlanta's female trap voice. Technical skill often underestimated.</t>
         </is>
       </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -9270,6 +9855,11 @@
           <t>St. Louis's jazz-rap hybrid. Melodic and rhythmic sophistication.</t>
         </is>
       </c>
+      <c r="S118" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -9342,6 +9932,11 @@
           <t>Cocaine rap's Rembrandt. 'Daytona' — maximum density, minimum waste.</t>
         </is>
       </c>
+      <c r="S119" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -9414,6 +10009,11 @@
           <t>'Igor' and 'Call Me If You Get Lost' — producer-auteur. Concept album mastery.</t>
         </is>
       </c>
+      <c r="S120" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -9490,6 +10090,11 @@
           <t>billy woods + ELUCID. The most demanding abstract rap being made today.</t>
         </is>
       </c>
+      <c r="S121" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -9566,6 +10171,11 @@
           <t>Comedy-meets-rap. Formally interesting but body of work too small to score confidently.</t>
         </is>
       </c>
+      <c r="S122" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -9642,6 +10252,11 @@
           <t>Chicago drill's most commercially consistent voice.</t>
         </is>
       </c>
+      <c r="S123" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -9718,6 +10333,11 @@
           <t>Florida trap's most distinctive voice. Rough-edged regional authenticity.</t>
         </is>
       </c>
+      <c r="S124" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -9790,6 +10410,11 @@
           <t>North Carolina's most complete female MC. Lyrical depth rivals any peer.</t>
         </is>
       </c>
+      <c r="S125" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -9866,6 +10491,11 @@
           <t>Charlotte underground. Dense introspective abstract rap. Watch this space.</t>
         </is>
       </c>
+      <c r="S126" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -9942,6 +10572,11 @@
           <t>West Coast boom bap craftsman. More respected by peers than critics.</t>
         </is>
       </c>
+      <c r="S127" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -10018,6 +10653,11 @@
           <t>Bay Area trap-pop. Ice Princess persona over lyrical substance.</t>
         </is>
       </c>
+      <c r="S128" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -10094,6 +10734,11 @@
           <t>Miami's hedonistic party rap duo. Energy over craft.</t>
         </is>
       </c>
+      <c r="S129" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -10170,6 +10815,11 @@
           <t>Houston storytelling tradition continued. 'Weight of the World' deeply affecting.</t>
         </is>
       </c>
+      <c r="S130" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -10241,6 +10891,11 @@
           <t>Philadelphia's live-band institution; Black Thought's relentless technique anchors a peerless catalog.</t>
         </is>
       </c>
+      <c r="S131" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -10317,6 +10972,11 @@
           <t>Philadelphia's hardest pen. Street narratives carried with weight and conviction.</t>
         </is>
       </c>
+      <c r="S132" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -10393,6 +11053,11 @@
           <t>Genre-bending rage pioneer. Melody and energy over lyrical density.</t>
         </is>
       </c>
+      <c r="S133" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -10469,6 +11134,11 @@
           <t>Distinctive raspy urgency and Philly grit. State Property standout.</t>
         </is>
       </c>
+      <c r="S134" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -10545,6 +11215,11 @@
           <t>Ruff Ryders' First Lady. Charismatic crossover with Philly roots.</t>
         </is>
       </c>
+      <c r="S135" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -10621,6 +11296,11 @@
           <t>So So Def's breakout. First female solo rapper to go platinum.</t>
         </is>
       </c>
+      <c r="S136" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -10697,6 +11377,11 @@
           <t>Oakland pioneer and pimp-rap archetype. Influence over intricacy.</t>
         </is>
       </c>
+      <c r="S137" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -10773,6 +11458,11 @@
           <t>Hieroglyphics wordsmith. Quirky vocabulary and abstract wit.</t>
         </is>
       </c>
+      <c r="S138" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -10849,6 +11539,11 @@
           <t>Hyphy movement godfather. Enduring Bay Area cult legend.</t>
         </is>
       </c>
+      <c r="S139" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -10925,6 +11620,11 @@
           <t>Detroit technician. Slaughterhouse and PRhyme cornerstone.</t>
         </is>
       </c>
+      <c r="S140" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -10996,6 +11696,11 @@
           <t>Mafioso-rap forefather. The multisyllabic blueprint for Nas, Biggie and Jay-Z.</t>
         </is>
       </c>
+      <c r="S141" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -11072,6 +11777,11 @@
           <t>Newark's funkiest. Effortless flow with comedic menace.</t>
         </is>
       </c>
+      <c r="S142" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -11148,6 +11858,11 @@
           <t>Wu-Tang's charismatic star. Gravel-voiced hooks and grit.</t>
         </is>
       </c>
+      <c r="S143" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -11224,6 +11939,11 @@
           <t>Strictly Business. Laid-back funk and durable chemistry.</t>
         </is>
       </c>
+      <c r="S144" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -11300,6 +12020,11 @@
           <t>Compton revivalist. The Documentary-era West Coast resurgence.</t>
         </is>
       </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -11376,6 +12101,11 @@
           <t>Gangsta-rap originator. Street reportage before the template existed.</t>
         </is>
       </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -11452,6 +12182,11 @@
           <t>Crenshaw's marathon. Street wisdom and self-determination.</t>
         </is>
       </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -11526,6 +12261,11 @@
       <c r="R148" t="inlineStr">
         <is>
           <t>G-funk auteur. Producer-rapper with effortless West Coast bounce.</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>Element</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cleanup pass: data-driven gender column, workbook hygiene, dead code
- Add a Gender column (Male/Female/Mixed) to the Artist Database sheet and
  a matching Data Dictionary entry; the dashboard's gender-representation
  chart now reads it instead of a hardcoded artist-name vector
- Normalize Composite Score cached values to 1 decimal (removes float
  artifacts like 8.800000000000001 from the workbook)
- Update the static bias-table gender figure to ~15% (18/120)
- Remove dead template code: --uk/--intl CSS vars, unused
  .tile-conf/.conf-H/M/L rules, 'Late 99s' typo-tolerance checks, and
  stale hardcoded-count comments in buildEraLayout

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AYwyGjCcrmQGUKZPhS1uD8
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S148"/>
+  <dimension ref="A1:T148"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -705,6 +705,11 @@
           <t>Type</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -782,6 +787,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -859,6 +869,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -936,6 +951,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1013,6 +1033,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1090,6 +1115,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1167,6 +1197,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1244,6 +1279,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1319,6 +1359,11 @@
       <c r="S9" t="inlineStr">
         <is>
           <t>Compound</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -1398,6 +1443,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1475,6 +1525,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1556,6 +1611,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1637,6 +1697,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1718,6 +1783,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1799,6 +1869,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1880,6 +1955,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1961,6 +2041,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -2038,6 +2123,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -2119,6 +2209,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -2196,6 +2291,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -2255,7 +2355,7 @@
         <v>8</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>8.800000000000001</v>
+        <v>8.8</v>
       </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
@@ -2271,6 +2371,11 @@
       <c r="S21" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -2350,6 +2455,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2427,6 +2537,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2486,7 +2601,7 @@
         <v>8</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P24" s="7" t="inlineStr">
         <is>
@@ -2502,6 +2617,11 @@
       <c r="S24" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -2581,6 +2701,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2658,6 +2783,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -2735,6 +2865,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2812,6 +2947,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -2889,6 +3029,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2966,6 +3111,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -3043,6 +3193,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -3120,6 +3275,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -3197,6 +3357,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3274,6 +3439,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -3355,6 +3525,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3432,6 +3607,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3513,6 +3693,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3594,6 +3779,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3653,7 +3843,7 @@
         <v>7</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
@@ -3669,6 +3859,11 @@
       <c r="S39" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -3748,6 +3943,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3829,6 +4029,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3910,6 +4115,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -3991,6 +4201,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -4068,6 +4283,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -4145,6 +4365,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -4222,6 +4447,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -4281,7 +4511,7 @@
         <v>8</v>
       </c>
       <c r="O47" s="6" t="n">
-        <v>9.199999999999999</v>
+        <v>9.2</v>
       </c>
       <c r="P47" s="7" t="inlineStr">
         <is>
@@ -4297,6 +4527,11 @@
       <c r="S47" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -4376,6 +4611,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -4435,7 +4675,7 @@
         <v>9</v>
       </c>
       <c r="O49" s="6" t="n">
-        <v>8.800000000000001</v>
+        <v>8.8</v>
       </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
@@ -4451,6 +4691,11 @@
       <c r="S49" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>Female</t>
         </is>
       </c>
     </row>
@@ -4530,6 +4775,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -4607,6 +4857,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -4684,6 +4939,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -4761,6 +5021,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -4838,6 +5103,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -4919,6 +5189,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -5000,6 +5275,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -5077,6 +5357,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -5158,6 +5443,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -5239,6 +5529,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -5320,6 +5615,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -5379,7 +5679,7 @@
         <v>7</v>
       </c>
       <c r="O61" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P61" s="7" t="inlineStr">
         <is>
@@ -5395,6 +5695,11 @@
       <c r="S61" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5761,7 @@
         <v>8</v>
       </c>
       <c r="O62" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P62" s="14" t="inlineStr">
         <is>
@@ -5476,6 +5781,11 @@
       <c r="S62" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -5555,6 +5865,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -5632,6 +5947,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -5709,6 +6029,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -5786,6 +6111,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -5863,6 +6193,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -5922,7 +6257,7 @@
         <v>8</v>
       </c>
       <c r="O68" s="6" t="n">
-        <v>9.199999999999999</v>
+        <v>9.2</v>
       </c>
       <c r="P68" s="7" t="inlineStr">
         <is>
@@ -5938,6 +6273,11 @@
       <c r="S68" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -6017,6 +6357,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -6094,6 +6439,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -6171,6 +6521,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -6230,7 +6585,7 @@
         <v>10</v>
       </c>
       <c r="O72" s="6" t="n">
-        <v>8.800000000000001</v>
+        <v>8.8</v>
       </c>
       <c r="P72" s="7" t="inlineStr">
         <is>
@@ -6246,6 +6601,11 @@
       <c r="S72" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6667,7 @@
         <v>8</v>
       </c>
       <c r="O73" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P73" s="7" t="inlineStr">
         <is>
@@ -6323,6 +6683,11 @@
       <c r="S73" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -6402,6 +6767,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -6483,6 +6853,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -6560,6 +6935,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -6641,6 +7021,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -6718,6 +7103,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -6799,6 +7189,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -6880,6 +7275,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -6957,6 +7357,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -7034,6 +7439,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -7115,6 +7525,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -7196,6 +7611,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -7273,6 +7693,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -7350,6 +7775,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -7427,6 +7857,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -7504,6 +7939,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -7563,7 +8003,7 @@
         <v>9</v>
       </c>
       <c r="O89" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P89" s="7" t="inlineStr">
         <is>
@@ -7579,6 +8019,11 @@
       <c r="S89" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -7658,6 +8103,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -7735,6 +8185,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -7812,6 +8267,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -7889,6 +8349,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -7966,6 +8431,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -8043,6 +8513,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -8120,6 +8595,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -8179,7 +8659,7 @@
         <v>9</v>
       </c>
       <c r="O97" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P97" s="7" t="inlineStr">
         <is>
@@ -8195,6 +8675,11 @@
       <c r="S97" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -8274,6 +8759,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -8351,6 +8841,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -8432,6 +8927,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -8513,6 +9013,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -8590,6 +9095,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -8649,7 +9159,7 @@
         <v>8</v>
       </c>
       <c r="O103" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P103" s="7" t="inlineStr">
         <is>
@@ -8665,6 +9175,11 @@
       <c r="S103" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -8726,7 +9241,7 @@
         <v>8</v>
       </c>
       <c r="O104" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P104" s="7" t="inlineStr">
         <is>
@@ -8742,6 +9257,11 @@
       <c r="S104" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -8821,6 +9341,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -8880,7 +9405,7 @@
         <v>8</v>
       </c>
       <c r="O106" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P106" s="14" t="inlineStr">
         <is>
@@ -8900,6 +9425,11 @@
       <c r="S106" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -8979,6 +9509,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -9060,6 +9595,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -9141,6 +9681,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -9200,7 +9745,7 @@
         <v>9</v>
       </c>
       <c r="O110" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P110" s="14" t="inlineStr">
         <is>
@@ -9220,6 +9765,11 @@
       <c r="S110" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Female</t>
         </is>
       </c>
     </row>
@@ -9303,6 +9853,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -9384,6 +9939,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -9465,6 +10025,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -9542,6 +10107,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
@@ -9623,6 +10193,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -9704,6 +10279,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -9785,6 +10365,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -9866,6 +10451,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -9943,6 +10533,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -10020,6 +10615,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -10079,7 +10679,7 @@
         <v>8</v>
       </c>
       <c r="O121" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P121" s="14" t="inlineStr">
         <is>
@@ -10099,6 +10699,11 @@
       <c r="S121" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -10182,6 +10787,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -10263,6 +10873,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -10344,6 +10959,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -10403,7 +11023,7 @@
         <v>9</v>
       </c>
       <c r="O125" s="6" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P125" s="7" t="inlineStr">
         <is>
@@ -10419,6 +11039,11 @@
       <c r="S125" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>Female</t>
         </is>
       </c>
     </row>
@@ -10502,6 +11127,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -10583,6 +11213,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -10664,6 +11299,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -10745,6 +11385,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -10826,6 +11471,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -10885,7 +11535,7 @@
         <v>8</v>
       </c>
       <c r="O131" t="n">
-        <v>8.800000000000001</v>
+        <v>8.8</v>
       </c>
       <c r="P131" t="inlineStr">
         <is>
@@ -10900,6 +11550,11 @@
       <c r="S131" t="inlineStr">
         <is>
           <t>Compound</t>
+        </is>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -10983,6 +11638,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -11064,6 +11724,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -11145,6 +11810,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -11226,6 +11896,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -11307,6 +11982,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -11388,6 +12068,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -11469,6 +12154,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -11550,6 +12240,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -11631,6 +12326,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -11690,7 +12390,7 @@
         <v>7</v>
       </c>
       <c r="O141" t="n">
-        <v>8.199999999999999</v>
+        <v>8.2</v>
       </c>
       <c r="P141" t="inlineStr">
         <is>
@@ -11705,6 +12405,11 @@
       <c r="S141" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -11788,6 +12493,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -11869,6 +12579,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -11950,6 +12665,11 @@
           <t>Compound</t>
         </is>
       </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -12031,6 +12751,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -12112,6 +12837,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -12193,6 +12923,11 @@
           <t>Element</t>
         </is>
       </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -12272,6 +13007,11 @@
       <c r="S148" t="inlineStr">
         <is>
           <t>Element</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Male</t>
         </is>
       </c>
     </row>
@@ -12444,7 +13184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12995,18 +13735,34 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="n"/>
-      <c r="B21" s="17" t="n"/>
-      <c r="C21" s="17" t="n"/>
-      <c r="D21" s="17" t="n"/>
-      <c r="E21" s="17" t="n"/>
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>Male, Female, Mixed</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>Gender of the act as publicly identified. Mixed = group with members of more than one gender. Drives the dashboard’s gender-representation chart.</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>Public record; entered at data entry.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
-        </is>
-      </c>
+      <c r="A22" s="17" t="n"/>
       <c r="B22" s="17" t="n"/>
       <c r="C22" s="17" t="n"/>
       <c r="D22" s="17" t="n"/>
@@ -13015,14 +13771,10 @@
     <row r="23">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
-        </is>
-      </c>
+          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="n"/>
       <c r="C23" s="17" t="n"/>
       <c r="D23" s="17" t="n"/>
       <c r="E23" s="17" t="n"/>
@@ -13030,12 +13782,12 @@
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>Inclusion</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
+          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
         </is>
       </c>
       <c r="C24" s="17" t="n"/>
@@ -13045,12 +13797,12 @@
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t>Exclusion</t>
+          <t>Inclusion</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
+          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
         </is>
       </c>
       <c r="C25" s="17" t="n"/>
@@ -13060,12 +13812,12 @@
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t>Unit of analysis</t>
+          <t>Exclusion</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
+          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
         </is>
       </c>
       <c r="C26" s="17" t="n"/>
@@ -13075,17 +13827,32 @@
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>Known frame biases</t>
+          <t>Unit of analysis</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
         </is>
       </c>
       <c r="C27" s="17" t="n"/>
       <c r="D27" s="17" t="n"/>
       <c r="E27" s="17" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Known frame biases</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="17" t="n"/>
+      <c r="E28" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Expansion batch 2: 16 acts targeting documented dataset gaps
Adds 12 Elements and 4 Compounds to the Artist Database sheet (147 -> 163
acts), scored per the codebook's critical-consensus methodology with
confidence notes on every M/L act:

- Gender gap: Salt-N-Pepa, Megan Thee Stallion, Yo-Yo, Bahamadia,
  Jean Grae, Trina, Mia X (female Elements now 24/132 = 18%)
- Geography/craft: Bone Thugs-N-Harmony, 8Ball & MJG, Souls of Mischief,
  Twista, Tech N9ne (Midwest, Bay Area, Memphis depth)
- Prestige-bias cases: Nelly, Chief Keef
- Modern underground: Roc Marciano, Denzel Curry

Updates the hardcoded counts in projects page copy, the dashboard bias
table (~18% female), and the internal worklist (totals, style
distribution, done log).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AYwyGjCcrmQGUKZPhS1uD8
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T148"/>
+  <dimension ref="A1:T164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13015,6 +13015,1378 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Salt-N-Pepa</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>New Jack/Pop Rap</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Next Plateau</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>1985</v>
+      </c>
+      <c r="J149" t="n">
+        <v>5</v>
+      </c>
+      <c r="K149" t="n">
+        <v>5</v>
+      </c>
+      <c r="L149" t="n">
+        <v>5</v>
+      </c>
+      <c r="M149" t="n">
+        <v>5</v>
+      </c>
+      <c r="N149" t="n">
+        <v>6</v>
+      </c>
+      <c r="O149" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q149" t="inlineStr">
+        <is>
+          <t>Extensively covered historically; close lyrical analysis thinner than cultural impact</t>
+        </is>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>Best-selling female rap act of their era. Sex-positive anthems that moved the mainstream.</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Megan Thee Stallion</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2020s</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Houston Trap</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>1501 Certified/300</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J150" t="n">
+        <v>7</v>
+      </c>
+      <c r="K150" t="n">
+        <v>6</v>
+      </c>
+      <c r="L150" t="n">
+        <v>5</v>
+      </c>
+      <c r="M150" t="n">
+        <v>7</v>
+      </c>
+      <c r="N150" t="n">
+        <v>5</v>
+      </c>
+      <c r="O150" t="n">
+        <v>6</v>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q150" t="inlineStr">
+        <is>
+          <t>Recent; awards and commercial dominance clear; long-form lyrical analysis still accumulating</t>
+        </is>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Houston hot-girl anthems built on genuine freestyle technique. Grammy Best New Artist.</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>YY</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Yo-Yo</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>West Coast Funk</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>East West</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>1991</v>
+      </c>
+      <c r="J151" t="n">
+        <v>6</v>
+      </c>
+      <c r="K151" t="n">
+        <v>6</v>
+      </c>
+      <c r="L151" t="n">
+        <v>6</v>
+      </c>
+      <c r="M151" t="n">
+        <v>5</v>
+      </c>
+      <c r="N151" t="n">
+        <v>7</v>
+      </c>
+      <c r="O151" t="n">
+        <v>6</v>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q151" t="inlineStr">
+        <is>
+          <t>Cited in histories of women in rap; limited close lyrical analysis</t>
+        </is>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Ice Cube protégée and IBWC founder. Feminist counterpoint inside gangsta-era LA.</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Bahamadia</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Philly</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Jazz Boom Bap</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Chrysalis/EMI</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>1995</v>
+      </c>
+      <c r="J152" t="n">
+        <v>8</v>
+      </c>
+      <c r="K152" t="n">
+        <v>8</v>
+      </c>
+      <c r="L152" t="n">
+        <v>6</v>
+      </c>
+      <c r="M152" t="n">
+        <v>7</v>
+      </c>
+      <c r="N152" t="n">
+        <v>7</v>
+      </c>
+      <c r="O152" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q152" t="inlineStr">
+        <is>
+          <t>Revered in underground and DJ circles; scant mainstream scholarship</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Philly's smoothest technician. Kollage a cult classic of low-key precision flow.</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Jean Grae</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Underground Boom Bap</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Blacksmith</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>2002</v>
+      </c>
+      <c r="J153" t="n">
+        <v>8</v>
+      </c>
+      <c r="K153" t="n">
+        <v>8</v>
+      </c>
+      <c r="L153" t="n">
+        <v>7</v>
+      </c>
+      <c r="M153" t="n">
+        <v>8</v>
+      </c>
+      <c r="N153" t="n">
+        <v>7</v>
+      </c>
+      <c r="O153" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q153" t="inlineStr">
+        <is>
+          <t>Peer-acclaimed technician; coverage concentrated in underground press</t>
+        </is>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Punchline surgeon and satirist. One of underground New York's most complete pens.</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Trina</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Miami Bass/Trap</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Slip-n-Slide</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>1998</v>
+      </c>
+      <c r="J154" t="n">
+        <v>5</v>
+      </c>
+      <c r="K154" t="n">
+        <v>5</v>
+      </c>
+      <c r="L154" t="n">
+        <v>4</v>
+      </c>
+      <c r="M154" t="n">
+        <v>5</v>
+      </c>
+      <c r="N154" t="n">
+        <v>4</v>
+      </c>
+      <c r="O154" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr">
+        <is>
+          <t>Commercial longevity clear; almost no formal lyrical analysis</t>
+        </is>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>Miami mainstay. Two decades of unapologetic Southern raunch rap and resilience.</t>
+        </is>
+      </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Mia X</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>No Limit Bounce</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>No Limit</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>1995</v>
+      </c>
+      <c r="J155" t="n">
+        <v>6</v>
+      </c>
+      <c r="K155" t="n">
+        <v>5</v>
+      </c>
+      <c r="L155" t="n">
+        <v>7</v>
+      </c>
+      <c r="M155" t="n">
+        <v>5</v>
+      </c>
+      <c r="N155" t="n">
+        <v>5</v>
+      </c>
+      <c r="O155" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="Q155" t="inlineStr">
+        <is>
+          <t>No Limit's first lady; regional significance with minimal national critical record</t>
+        </is>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>No Limit's first female star. New Orleans street matriarch with real narrative weight.</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>BTH</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Bone Thugs-N-Harmony</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Melodic Midwest G-Funk</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Ruthless</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J156" t="n">
+        <v>9</v>
+      </c>
+      <c r="K156" t="n">
+        <v>6</v>
+      </c>
+      <c r="L156" t="n">
+        <v>7</v>
+      </c>
+      <c r="M156" t="n">
+        <v>6</v>
+      </c>
+      <c r="N156" t="n">
+        <v>7</v>
+      </c>
+      <c r="O156" t="n">
+        <v>7</v>
+      </c>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q156" t="inlineStr"/>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>Cleveland's melodic-speed innovators. Harmonized double-time no one has replicated.</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>8B</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>8Ball &amp; MJG</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Memphis Funk</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Suave House</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>1993</v>
+      </c>
+      <c r="J157" t="n">
+        <v>7</v>
+      </c>
+      <c r="K157" t="n">
+        <v>6</v>
+      </c>
+      <c r="L157" t="n">
+        <v>8</v>
+      </c>
+      <c r="M157" t="n">
+        <v>6</v>
+      </c>
+      <c r="N157" t="n">
+        <v>6</v>
+      </c>
+      <c r="O157" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q157" t="inlineStr">
+        <is>
+          <t>Well-cited in Southern rap histories; close analysis thinner</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>Memphis's founding duo. Country-fried pimp narratives that drew the South's blueprint.</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Souls of Mischief</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Golden Age</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>Jazz-Rap</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Hieroglyphics Jazz Sample</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Jive</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>1993</v>
+      </c>
+      <c r="J158" t="n">
+        <v>8</v>
+      </c>
+      <c r="K158" t="n">
+        <v>8</v>
+      </c>
+      <c r="L158" t="n">
+        <v>6</v>
+      </c>
+      <c r="M158" t="n">
+        <v>7</v>
+      </c>
+      <c r="N158" t="n">
+        <v>7</v>
+      </c>
+      <c r="O158" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q158" t="inlineStr">
+        <is>
+          <t>'93 til Infinity canonical; group-level scholarship thinner than the single's fame</t>
+        </is>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>Hieroglyphics' teenage virtuosos. '93 til Infinity is the Bay's jazz-rap landmark.</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Twista</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Chicago Chopper/Soul</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Atlantic</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>1992</v>
+      </c>
+      <c r="J159" t="n">
+        <v>9</v>
+      </c>
+      <c r="K159" t="n">
+        <v>6</v>
+      </c>
+      <c r="L159" t="n">
+        <v>6</v>
+      </c>
+      <c r="M159" t="n">
+        <v>6</v>
+      </c>
+      <c r="N159" t="n">
+        <v>5</v>
+      </c>
+      <c r="O159" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q159" t="inlineStr">
+        <is>
+          <t>Speed technique widely celebrated; substantive analysis of the writing thinner</t>
+        </is>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>Chicago chopper pioneer. Once Guinness-fastest; precision at absurd tempo.</t>
+        </is>
+      </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Tech N9ne</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Strange Music Horrorcore</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Strange Music</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>1999</v>
+      </c>
+      <c r="J160" t="n">
+        <v>9</v>
+      </c>
+      <c r="K160" t="n">
+        <v>7</v>
+      </c>
+      <c r="L160" t="n">
+        <v>6</v>
+      </c>
+      <c r="M160" t="n">
+        <v>6</v>
+      </c>
+      <c r="N160" t="n">
+        <v>6</v>
+      </c>
+      <c r="O160" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q160" t="inlineStr">
+        <is>
+          <t>Independent institution; peer-revered technique with little academic attention</t>
+        </is>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>Kansas City's independent empire. Chopper virtuosity meets horrorcore theatricality.</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Nelly</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>Party/Pop</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>St. Louis Pop Rap</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>Universal</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J161" t="n">
+        <v>5</v>
+      </c>
+      <c r="K161" t="n">
+        <v>5</v>
+      </c>
+      <c r="L161" t="n">
+        <v>5</v>
+      </c>
+      <c r="M161" t="n">
+        <v>5</v>
+      </c>
+      <c r="N161" t="n">
+        <v>4</v>
+      </c>
+      <c r="O161" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q161" t="inlineStr">
+        <is>
+          <t>Diamond-selling; critical framework mostly dismissive — a prestige-bias test case</t>
+        </is>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>St. Louis's melodic hitmaker. Country Grammar went diamond; craft chronically under-analyzed.</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>CK</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Chief Keef</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2010s</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Trap/Drill</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Chicago Drill</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>Glory Boyz/Interscope</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>2012</v>
+      </c>
+      <c r="J162" t="n">
+        <v>4</v>
+      </c>
+      <c r="K162" t="n">
+        <v>4</v>
+      </c>
+      <c r="L162" t="n">
+        <v>4</v>
+      </c>
+      <c r="M162" t="n">
+        <v>5</v>
+      </c>
+      <c r="N162" t="n">
+        <v>5</v>
+      </c>
+      <c r="O162" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q162" t="inlineStr">
+        <is>
+          <t>Drill progenitor; reappraisal ongoing — influence far exceeds documented analysis</t>
+        </is>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>Drill's teenage architect. A Chicago sound that reshaped a decade of rap worldwide.</t>
+        </is>
+      </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>ROC</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Roc Marciano</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2010s</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Drumless Loop Minimalism</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>Marci Enterprises</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>2010</v>
+      </c>
+      <c r="J163" t="n">
+        <v>8</v>
+      </c>
+      <c r="K163" t="n">
+        <v>8</v>
+      </c>
+      <c r="L163" t="n">
+        <v>7</v>
+      </c>
+      <c r="M163" t="n">
+        <v>9</v>
+      </c>
+      <c r="N163" t="n">
+        <v>7</v>
+      </c>
+      <c r="O163" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q163" t="inlineStr">
+        <is>
+          <t>Underground canon (Marcberg, Reloaded); specialist-press documentation only</t>
+        </is>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>Rebuilt New York minimalism. Slang-dense mafioso poetry; the modern underground's blueprint.</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>DZ</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Denzel Curry</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2010s</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Florida Punk Trap</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Loma Vista</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>2013</v>
+      </c>
+      <c r="J164" t="n">
+        <v>8</v>
+      </c>
+      <c r="K164" t="n">
+        <v>7</v>
+      </c>
+      <c r="L164" t="n">
+        <v>6</v>
+      </c>
+      <c r="M164" t="n">
+        <v>7</v>
+      </c>
+      <c r="N164" t="n">
+        <v>8</v>
+      </c>
+      <c r="O164" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q164" t="inlineStr">
+        <is>
+          <t>Strong critical reception; scholarship still forming for the late-2010s class</t>
+        </is>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>Carol City shape-shifter. TA13OO fused punk energy with conceptual architecture.</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Roll Region up to coast-level taxonomy; preserve scenes in new column
Region becomes the four categories the culture itself uses — East Coast
(NYC + Philly), West Coast (LA + Bay Area), South, Midwest — replacing
the mixed local/broad six. The finer scene detail is not lost: a new
Scene column keeps NYC/Philly/LA/Bay Area/South/Midwest, the modal and
tile tooltips show it as "East Coast (NYC)", and the Data Dictionary
sheet documents both variables (Region now derived from Scene).

Dashboard palettes, factor levels, and bias-table/prose references
updated to the new taxonomy; periodic-table filter, legend, and shape
glyphs reduced to four regions.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AYwyGjCcrmQGUKZPhS1uD8
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T164"/>
+  <dimension ref="A1:U164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -710,6 +710,11 @@
           <t>Gender</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Scene</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -727,7 +732,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -790,6 +795,11 @@
       <c r="T2" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -809,7 +819,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -872,6 +882,11 @@
       <c r="T3" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -891,7 +906,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -954,6 +969,11 @@
       <c r="T4" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -973,7 +993,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1036,6 +1056,11 @@
       <c r="T5" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1080,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1118,6 +1143,11 @@
       <c r="T6" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1167,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1202,6 +1232,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1219,7 +1254,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1284,6 +1319,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1301,7 +1341,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1364,6 +1404,11 @@
       <c r="T9" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1428,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1446,6 +1491,11 @@
       <c r="T10" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1515,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1528,6 +1578,11 @@
       <c r="T11" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1602,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1614,6 +1669,11 @@
       <c r="T12" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1693,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1700,6 +1760,11 @@
       <c r="T13" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1784,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1786,6 +1851,11 @@
       <c r="T14" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1875,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1872,6 +1942,11 @@
       <c r="T15" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -1891,7 +1966,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1958,6 +2033,11 @@
       <c r="T16" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -1977,7 +2057,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -2044,6 +2124,11 @@
       <c r="T17" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2148,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2126,6 +2211,11 @@
       <c r="T18" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2235,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -2212,6 +2302,11 @@
       <c r="T19" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2326,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -2294,6 +2389,11 @@
       <c r="T20" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2413,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2376,6 +2476,11 @@
       <c r="T21" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2395,7 +2500,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -2458,6 +2563,11 @@
       <c r="T22" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2587,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2540,6 +2650,11 @@
       <c r="T23" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2674,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2622,6 +2737,11 @@
       <c r="T24" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2761,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2704,6 +2824,11 @@
       <c r="T25" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2848,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -2786,6 +2911,11 @@
       <c r="T26" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2935,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -2868,6 +2998,11 @@
       <c r="T27" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2887,7 +3022,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -2950,6 +3085,11 @@
       <c r="T28" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -2969,7 +3109,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -3032,6 +3172,11 @@
       <c r="T29" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3196,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -3114,6 +3259,11 @@
       <c r="T30" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -3133,7 +3283,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -3196,6 +3346,11 @@
       <c r="T31" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -3215,7 +3370,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -3278,6 +3433,11 @@
       <c r="T32" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3457,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -3360,6 +3520,11 @@
       <c r="T33" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3544,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -3442,6 +3607,11 @@
       <c r="T34" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
         </is>
       </c>
     </row>
@@ -3461,7 +3631,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -3528,6 +3698,11 @@
       <c r="T35" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3722,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -3610,6 +3785,11 @@
       <c r="T36" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3809,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -3696,6 +3876,11 @@
       <c r="T37" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3900,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -3782,6 +3967,11 @@
       <c r="T38" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3991,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -3864,6 +4054,11 @@
       <c r="T39" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -3948,6 +4143,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3965,7 +4165,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -4032,6 +4232,11 @@
       <c r="T41" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4256,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -4118,6 +4323,11 @@
       <c r="T42" t="inlineStr">
         <is>
           <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4137,7 +4347,7 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
@@ -4204,6 +4414,11 @@
       <c r="T43" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4438,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -4286,6 +4501,11 @@
       <c r="T44" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4305,7 +4525,7 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -4368,6 +4588,11 @@
       <c r="T45" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4612,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -4450,6 +4675,11 @@
       <c r="T46" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4534,6 +4764,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -4551,7 +4786,7 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -4614,6 +4849,11 @@
       <c r="T48" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4633,7 +4873,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -4696,6 +4936,11 @@
       <c r="T49" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4780,6 +5025,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -4797,7 +5047,7 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -4860,6 +5110,11 @@
       <c r="T51" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -4879,7 +5134,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -4942,6 +5197,11 @@
       <c r="T52" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5026,6 +5286,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -5108,6 +5373,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -5125,7 +5395,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -5192,6 +5462,11 @@
       <c r="T55" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5211,7 +5486,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -5278,6 +5553,11 @@
       <c r="T56" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5297,7 +5577,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -5360,6 +5640,11 @@
       <c r="T57" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5448,6 +5733,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -5465,7 +5755,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -5532,6 +5822,11 @@
       <c r="T59" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5846,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -5618,6 +5913,11 @@
       <c r="T60" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5937,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -5700,6 +6000,11 @@
       <c r="T61" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5719,7 +6024,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -5786,6 +6091,11 @@
       <c r="T62" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -5870,6 +6180,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -5952,6 +6267,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -6034,6 +6354,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -6116,6 +6441,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -6133,7 +6463,7 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -6196,6 +6526,11 @@
       <c r="T67" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -6215,7 +6550,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -6278,6 +6613,11 @@
       <c r="T68" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -6362,6 +6702,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -6444,6 +6789,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -6526,6 +6876,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -6608,6 +6963,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -6690,6 +7050,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -6707,7 +7072,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -6770,6 +7135,11 @@
       <c r="T74" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -6789,7 +7159,7 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -6856,6 +7226,11 @@
       <c r="T75" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -6875,7 +7250,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -6938,6 +7313,11 @@
       <c r="T76" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -7026,6 +7406,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -7108,6 +7493,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -7194,6 +7584,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -7211,7 +7606,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -7278,6 +7673,11 @@
       <c r="T80" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7697,7 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -7360,6 +7760,11 @@
       <c r="T81" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7784,7 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -7442,6 +7847,11 @@
       <c r="T82" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -7530,6 +7940,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -7547,7 +7962,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -7614,6 +8029,11 @@
       <c r="T84" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -7633,7 +8053,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -7696,6 +8116,11 @@
       <c r="T85" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -7780,6 +8205,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -7862,6 +8292,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -7944,6 +8379,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -8026,6 +8466,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -8043,7 +8488,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -8106,6 +8551,11 @@
       <c r="T90" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -8125,7 +8575,7 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -8188,6 +8638,11 @@
       <c r="T91" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -8207,7 +8662,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -8270,6 +8725,11 @@
       <c r="T92" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -8289,7 +8749,7 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -8352,6 +8812,11 @@
       <c r="T93" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -8371,7 +8836,7 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -8434,6 +8899,11 @@
       <c r="T94" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -8518,6 +8988,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -8600,6 +9075,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -8682,6 +9162,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -8764,6 +9249,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -8846,6 +9336,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -8932,6 +9427,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -8949,7 +9449,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -9016,6 +9516,11 @@
       <c r="T101" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -9100,6 +9605,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -9182,6 +9692,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -9264,6 +9779,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -9346,6 +9866,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -9432,6 +9957,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -9449,7 +9979,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -9512,6 +10042,11 @@
       <c r="T107" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -9600,6 +10135,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -9686,6 +10226,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -9772,6 +10317,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
@@ -9858,6 +10408,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
@@ -9944,6 +10499,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -10030,6 +10590,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -10047,7 +10612,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -10110,6 +10675,11 @@
       <c r="T114" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -10198,6 +10768,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
@@ -10284,6 +10859,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
@@ -10370,6 +10950,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -10456,6 +11041,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U118" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -10473,7 +11063,7 @@
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
@@ -10536,6 +11126,11 @@
       <c r="T119" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U119" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -10555,7 +11150,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -10618,6 +11213,11 @@
       <c r="T120" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U120" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -10637,7 +11237,7 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
@@ -10704,6 +11304,11 @@
       <c r="T121" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U121" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -10792,6 +11397,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U122" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -10878,6 +11488,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U123" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
@@ -10964,6 +11579,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U124" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -11046,6 +11666,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U125" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -11132,6 +11757,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U126" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -11149,7 +11779,7 @@
       </c>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -11216,6 +11846,11 @@
       <c r="T127" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U127" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -11235,7 +11870,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
@@ -11302,6 +11937,11 @@
       <c r="T128" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U128" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
         </is>
       </c>
     </row>
@@ -11390,6 +12030,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U129" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -11476,6 +12121,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U130" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -11493,7 +12143,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -11555,6 +12205,11 @@
       <c r="T131" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U131" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -11574,7 +12229,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
@@ -11641,6 +12296,11 @@
       <c r="T132" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U132" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -11660,7 +12320,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -11727,6 +12387,11 @@
       <c r="T133" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U133" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -11746,7 +12411,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -11813,6 +12478,11 @@
       <c r="T134" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U134" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -11832,7 +12502,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -11899,6 +12569,11 @@
       <c r="T135" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U135" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -11987,6 +12662,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U136" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12004,7 +12684,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -12071,6 +12751,11 @@
       <c r="T137" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U137" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
         </is>
       </c>
     </row>
@@ -12090,7 +12775,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -12157,6 +12842,11 @@
       <c r="T138" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U138" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
         </is>
       </c>
     </row>
@@ -12176,7 +12866,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -12243,6 +12933,11 @@
       <c r="T139" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U139" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
         </is>
       </c>
     </row>
@@ -12331,6 +13026,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U140" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -12348,7 +13048,7 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
@@ -12410,6 +13110,11 @@
       <c r="T141" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U141" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -12429,7 +13134,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -12496,6 +13201,11 @@
       <c r="T142" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U142" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -12515,7 +13225,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -12582,6 +13292,11 @@
       <c r="T143" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U143" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -12601,7 +13316,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -12668,6 +13383,11 @@
       <c r="T144" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U144" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -12687,7 +13407,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -12754,6 +13474,11 @@
       <c r="T145" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -12773,7 +13498,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -12840,6 +13565,11 @@
       <c r="T146" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -12859,7 +13589,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -12926,6 +13656,11 @@
       <c r="T147" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -12945,7 +13680,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -13012,6 +13747,11 @@
       <c r="T148" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -13031,7 +13771,7 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
@@ -13098,6 +13838,11 @@
       <c r="T149" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -13186,6 +13931,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U150" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -13203,7 +13953,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>LA</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
@@ -13270,6 +14020,11 @@
       <c r="T151" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr">
+        <is>
+          <t>LA</t>
         </is>
       </c>
     </row>
@@ -13289,7 +14044,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Philly</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
@@ -13356,6 +14111,11 @@
       <c r="T152" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr">
+        <is>
+          <t>Philly</t>
         </is>
       </c>
     </row>
@@ -13375,7 +14135,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
@@ -13442,6 +14202,11 @@
       <c r="T153" t="inlineStr">
         <is>
           <t>Female</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -13530,6 +14295,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U154" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -13616,6 +14386,11 @@
           <t>Female</t>
         </is>
       </c>
+      <c r="U155" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -13698,6 +14473,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U156" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -13784,6 +14564,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U157" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -13801,7 +14586,7 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Bay Area</t>
+          <t>West Coast</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
@@ -13868,6 +14653,11 @@
       <c r="T158" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
         </is>
       </c>
     </row>
@@ -13956,6 +14746,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U159" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -14042,6 +14837,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U160" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -14128,6 +14928,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U161" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -14214,6 +15019,11 @@
           <t>Male</t>
         </is>
       </c>
+      <c r="U162" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -14231,7 +15041,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>NYC</t>
+          <t>East Coast</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
@@ -14298,6 +15108,11 @@
       <c r="T163" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>
@@ -14384,6 +15199,11 @@
       <c r="T164" t="inlineStr">
         <is>
           <t>Male</t>
+        </is>
+      </c>
+      <c r="U164" t="inlineStr">
+        <is>
+          <t>South</t>
         </is>
       </c>
     </row>
@@ -14556,7 +15376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -14687,17 +15507,17 @@
       </c>
       <c r="C5" s="17" t="inlineStr">
         <is>
-          <t>NYC, Philly, LA, South, Midwest, Bay Area</t>
+          <t>East Coast, West Coast, South, Midwest</t>
         </is>
       </c>
       <c r="D5" s="17" t="inlineStr">
         <is>
-          <t>US scene the act is professionally rooted in. Assigned by label home / scene affiliation, NOT city of birth (e.g. Da Brat = South via So So Def, though born in Chicago).</t>
+          <t>Coast-level region: East Coast = NYC + Philly scenes; West Coast = LA + Bay Area; South and Midwest map 1:1. Used by the dashboard charts and the periodic table’s shape glyph.</t>
         </is>
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
-          <t>Methods decision, documented 2026-06. International/UK acts are outside the sampling frame.</t>
+          <t>Derived from Scene; coast rollup documented 2026-07.</t>
         </is>
       </c>
     </row>
@@ -15134,18 +15954,34 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="17" t="n"/>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="17" t="n"/>
-      <c r="E22" s="17" t="n"/>
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Scene</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>NYC, Philly, LA, South, Midwest, Bay Area</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>US scene the act is professionally rooted in — label home and scene affiliation during the defining run, NOT city of birth (e.g. Da Brat = South via So So Def, though born in Chicago). Finer-grained than Region; preserved when Region was rolled up to coasts.</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>Methods decision, documented 2026-06.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
-        </is>
-      </c>
+      <c r="A23" s="17" t="n"/>
       <c r="B23" s="17" t="n"/>
       <c r="C23" s="17" t="n"/>
       <c r="D23" s="17" t="n"/>
@@ -15154,14 +15990,10 @@
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
-        </is>
-      </c>
+          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="n"/>
       <c r="C24" s="17" t="n"/>
       <c r="D24" s="17" t="n"/>
       <c r="E24" s="17" t="n"/>
@@ -15169,12 +16001,12 @@
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
         <is>
-          <t>Inclusion</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
+          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
         </is>
       </c>
       <c r="C25" s="17" t="n"/>
@@ -15184,12 +16016,12 @@
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t>Exclusion</t>
+          <t>Inclusion</t>
         </is>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
+          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
         </is>
       </c>
       <c r="C26" s="17" t="n"/>
@@ -15199,12 +16031,12 @@
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>Unit of analysis</t>
+          <t>Exclusion</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
+          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
         </is>
       </c>
       <c r="C27" s="17" t="n"/>
@@ -15214,17 +16046,32 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Known frame biases</t>
+          <t>Unit of analysis</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
         </is>
       </c>
       <c r="C28" s="17" t="n"/>
       <c r="D28" s="17" t="n"/>
       <c r="E28" s="17" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>Known frame biases</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="17" t="n"/>
+      <c r="E29" s="17" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Compounds expansion: 10 post-Golden-Age groups + 2 reclassifications
The Compounds table was 18/31 Golden Age with almost nothing after it.
Adds ten groups weighted to the later eras, scored per the documented
methodology: The Fugees, Goodie Mob, Company Flow (Late 90s); Clipse,
dead prez, Little Brother, Atmosphere, Blackalicious (2000s);
Brockhampton (2010s); Griselda (2020s). Compounds by era now
6/18/6/7/3/3.

Also reclassifies Whodini (trio) and Armand Hammer (duo) from Element
to Compound per the codebook's Type rule (J.J. Fad precedent), moving
them into the Compounds table. Totals: 173 acts = 130 Elements + 43
Compounds; projects-page copy and worklist updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AYwyGjCcrmQGUKZPhS1uD8
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U164"/>
+  <dimension ref="A1:U174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Element</t>
+          <t>Compound</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>Element</t>
+          <t>Compound</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -15204,6 +15204,908 @@
       <c r="U164" t="inlineStr">
         <is>
           <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>FG</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>The Fugees</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>East Coast</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Neo-Soul Boom Bap</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Ruffhouse</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J165" t="n">
+        <v>7</v>
+      </c>
+      <c r="K165" t="n">
+        <v>8</v>
+      </c>
+      <c r="L165" t="n">
+        <v>8</v>
+      </c>
+      <c r="M165" t="n">
+        <v>8</v>
+      </c>
+      <c r="N165" t="n">
+        <v>8</v>
+      </c>
+      <c r="O165" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q165" t="inlineStr"/>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>The Score — three voices, one landmark. Refugee soul meets New York boom bap.</t>
+        </is>
+      </c>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="U165" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Goodie Mob</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Dungeon Family Funk</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>LaFace</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>1995</v>
+      </c>
+      <c r="J166" t="n">
+        <v>6</v>
+      </c>
+      <c r="K166" t="n">
+        <v>7</v>
+      </c>
+      <c r="L166" t="n">
+        <v>7</v>
+      </c>
+      <c r="M166" t="n">
+        <v>6</v>
+      </c>
+      <c r="N166" t="n">
+        <v>8</v>
+      </c>
+      <c r="O166" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q166" t="inlineStr">
+        <is>
+          <t>Well-cited in Southern rap histories; less close analysis than OutKast</t>
+        </is>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>Soul Food coined the Dirty South. The Dungeon Family's spiritual conscience.</t>
+        </is>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Company Flow</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>East Coast</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Late 90s</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Industrial Boom Bap</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Rawkus</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>1996</v>
+      </c>
+      <c r="J167" t="n">
+        <v>8</v>
+      </c>
+      <c r="K167" t="n">
+        <v>9</v>
+      </c>
+      <c r="L167" t="n">
+        <v>6</v>
+      </c>
+      <c r="M167" t="n">
+        <v>8</v>
+      </c>
+      <c r="N167" t="n">
+        <v>8</v>
+      </c>
+      <c r="O167" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q167" t="inlineStr">
+        <is>
+          <t>Underground canon; specialist-press documentation only</t>
+        </is>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>Funcrusher Plus — independent rap's blueprint. Dense, abrasive, uncompromising.</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Clipse</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Neptunes Minimalism</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Star Trak</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>2002</v>
+      </c>
+      <c r="J168" t="n">
+        <v>8</v>
+      </c>
+      <c r="K168" t="n">
+        <v>8</v>
+      </c>
+      <c r="L168" t="n">
+        <v>8</v>
+      </c>
+      <c r="M168" t="n">
+        <v>9</v>
+      </c>
+      <c r="N168" t="n">
+        <v>7</v>
+      </c>
+      <c r="O168" t="n">
+        <v>8</v>
+      </c>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="Q168" t="inlineStr"/>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>Hell Hath No Fury — coke rap's cold masterpiece over Neptunes minimalism.</t>
+        </is>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U168" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>DP</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>dead prez</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>East Coast</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>Political</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Militant Boom Bap</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Loud</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>2000</v>
+      </c>
+      <c r="J169" t="n">
+        <v>6</v>
+      </c>
+      <c r="K169" t="n">
+        <v>7</v>
+      </c>
+      <c r="L169" t="n">
+        <v>6</v>
+      </c>
+      <c r="M169" t="n">
+        <v>6</v>
+      </c>
+      <c r="N169" t="n">
+        <v>9</v>
+      </c>
+      <c r="O169" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q169" t="inlineStr">
+        <is>
+          <t>Politically canonical; formal lyrical analysis thinner</t>
+        </is>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>Let's Get Free — revolutionary program set to rap. 'Hip-Hop' still detonates.</t>
+        </is>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U169" t="inlineStr">
+        <is>
+          <t>NYC</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>LB2</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Little Brother</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>9th Wonder Soul</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>ABB/Atlantic</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>2003</v>
+      </c>
+      <c r="J170" t="n">
+        <v>7</v>
+      </c>
+      <c r="K170" t="n">
+        <v>7</v>
+      </c>
+      <c r="L170" t="n">
+        <v>8</v>
+      </c>
+      <c r="M170" t="n">
+        <v>7</v>
+      </c>
+      <c r="N170" t="n">
+        <v>8</v>
+      </c>
+      <c r="O170" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q170" t="inlineStr">
+        <is>
+          <t>Critically beloved; scholarship modest relative to reputation</t>
+        </is>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>The Listening and The Minstrel Show — North Carolina soul-rap satire and craft.</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Atmosphere</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Ant Soul Loops</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Rhymesayers</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>1997</v>
+      </c>
+      <c r="J171" t="n">
+        <v>7</v>
+      </c>
+      <c r="K171" t="n">
+        <v>7</v>
+      </c>
+      <c r="L171" t="n">
+        <v>8</v>
+      </c>
+      <c r="M171" t="n">
+        <v>7</v>
+      </c>
+      <c r="N171" t="n">
+        <v>7</v>
+      </c>
+      <c r="O171" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q171" t="inlineStr">
+        <is>
+          <t>Independent institution; underground-press documentation</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>Slug and Ant. Minneapolis confessional rap that built an independent empire.</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr">
+        <is>
+          <t>Midwest</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>BL</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Blackalicious</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>West Coast</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2000s</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Conscious/Lyrical</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Quannum Funk</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Quannum/MCA</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>1994</v>
+      </c>
+      <c r="J172" t="n">
+        <v>9</v>
+      </c>
+      <c r="K172" t="n">
+        <v>9</v>
+      </c>
+      <c r="L172" t="n">
+        <v>6</v>
+      </c>
+      <c r="M172" t="n">
+        <v>7</v>
+      </c>
+      <c r="N172" t="n">
+        <v>7</v>
+      </c>
+      <c r="O172" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q172" t="inlineStr">
+        <is>
+          <t>Gift of Gab peer-revered; limited mainstream scholarship</t>
+        </is>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>Gift of Gab's tongue-twisting virtuosity over Chief Xcel. Alphabet Aerobics tier.</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr">
+        <is>
+          <t>Bay Area</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>BP</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Brockhampton</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>West Coast</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>2010s</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>DIY Pop Rap</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Question Everything/RCA</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J173" t="n">
+        <v>6</v>
+      </c>
+      <c r="K173" t="n">
+        <v>7</v>
+      </c>
+      <c r="L173" t="n">
+        <v>6</v>
+      </c>
+      <c r="M173" t="n">
+        <v>7</v>
+      </c>
+      <c r="N173" t="n">
+        <v>8</v>
+      </c>
+      <c r="O173" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q173" t="inlineStr">
+        <is>
+          <t>Recent; heavy press coverage, little formal analysis</t>
+        </is>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>The Saturation trilogy in one year. The streaming era's self-made boy band.</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Griselda</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>East Coast</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>2020s</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Gangsta/Street</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Drumless Boom Bap</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Griselda/Shady</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>2016</v>
+      </c>
+      <c r="J174" t="n">
+        <v>8</v>
+      </c>
+      <c r="K174" t="n">
+        <v>8</v>
+      </c>
+      <c r="L174" t="n">
+        <v>8</v>
+      </c>
+      <c r="M174" t="n">
+        <v>8</v>
+      </c>
+      <c r="N174" t="n">
+        <v>7</v>
+      </c>
+      <c r="O174" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="Q174" t="inlineStr">
+        <is>
+          <t>Crew output vast and recent; critical framework still consolidating</t>
+        </is>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>Buffalo's family business. WWCD made drumless grit the sound of underground NY.</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr">
+        <is>
+          <t>NYC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add career span + signature work dimension
Rebuilt on current main to resolve the binary workbook conflict with the
site-wide style pass (PRs 21-23): the plain-voice description edits and
dashboard rebrand are preserved, with the career dimension layered on
top.

New workbook columns for all 173 acts: Signature Work (the consensus
defining release, "Title (Year)") and Active Through (last year of new
primary-catalog output; blank = still active; 101 active, 72 concluded).
The Data Dictionary sheet documents both. The tile modal gains a
signature/active-span line, and the dashboard gains page "6 · Careers &
Longevity" (survivorship teaching prompt, career length vs composite,
years-to-signature-work distribution), renumbering the Full Data Table
to 7.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AYwyGjCcrmQGUKZPhS1uD8
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -819,6 +819,16 @@
           <t>Scene</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Signature Work</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Active Through</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
@@ -906,6 +916,9 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="W2" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
@@ -993,6 +1006,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>The Adventures of Grandmaster Flash on the Wheels of Steel (1981)</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>2009</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
@@ -1078,6 +1099,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>The Message (1982)</t>
+        </is>
+      </c>
+      <c r="W4" t="n">
+        <v>1989</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
@@ -1165,6 +1194,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>Rapper's Delight (1979)</t>
+        </is>
+      </c>
+      <c r="W5" t="n">
+        <v>1985</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="n">
@@ -1252,6 +1289,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Planet Rock (1982)</t>
+        </is>
+      </c>
+      <c r="W6" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
@@ -1339,6 +1384,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>Mama Said Knock You Out (1990)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
@@ -1426,6 +1476,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>Raising Hell (1986)</t>
+        </is>
+      </c>
+      <c r="W8" t="n">
+        <v>2002</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="n">
@@ -1512,6 +1570,14 @@
         <is>
           <t>NYC</t>
         </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Paul's Boutique (1989)</t>
+        </is>
+      </c>
+      <c r="W9" t="n">
+        <v>2012</v>
       </c>
     </row>
     <row r="10">
@@ -1600,6 +1666,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Criminal Minded (1987)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
@@ -1687,6 +1758,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>It Takes a Nation of Millions to Hold Us Back (1988)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="n">
@@ -1778,6 +1854,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Roxanne's Revenge (1984)</t>
+        </is>
+      </c>
+      <c r="W12" t="n">
+        <v>1992</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
@@ -1869,6 +1953,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Lyte as a Rock (1988)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
@@ -1960,6 +2049,14 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>P.S.K. What Does It Mean? (1985)</t>
+        </is>
+      </c>
+      <c r="W14" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
@@ -2051,6 +2148,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Supersonic (1988)</t>
+        </is>
+      </c>
+      <c r="W15" t="n">
+        <v>1992</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="14" t="n">
@@ -2142,6 +2247,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Escape (1984)</t>
+        </is>
+      </c>
+      <c r="W16" t="n">
+        <v>1996</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="n">
@@ -2233,6 +2346,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>The Show / La Di Da Di (1985)</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
@@ -2320,6 +2441,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>The Great Adventures of Slick Rick (1988)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
@@ -2411,6 +2537,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Dana Dane with Fame (1987)</t>
+        </is>
+      </c>
+      <c r="W19" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
@@ -2498,6 +2632,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>Long Live the Kane (1988)</t>
+        </is>
+      </c>
+      <c r="W20" t="n">
+        <v>1998</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
@@ -2585,6 +2727,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>Paid in Full (1987)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
@@ -2672,6 +2819,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>All Hail the Queen (1989)</t>
+        </is>
+      </c>
+      <c r="W22" t="n">
+        <v>1998</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
@@ -2759,6 +2914,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>Straight Outta Compton (1988)</t>
+        </is>
+      </c>
+      <c r="W23" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="14" t="n">
@@ -2846,6 +3009,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>AmeriKKKa's Most Wanted (1990)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
@@ -2933,6 +3101,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>3 Feet High and Rising (1989)</t>
+        </is>
+      </c>
+      <c r="W25" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="n">
@@ -3020,6 +3196,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>The Low End Theory (1991)</t>
+        </is>
+      </c>
+      <c r="W26" t="n">
+        <v>2016</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="14" t="n">
@@ -3107,6 +3291,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>Illmatic (1994)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
@@ -3194,6 +3383,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>Ready to Die (1994)</t>
+        </is>
+      </c>
+      <c r="W28" t="n">
+        <v>1997</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
@@ -3281,6 +3478,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>Enter the Wu-Tang (36 Chambers) (1993)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="n">
@@ -3368,6 +3570,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>Doggystyle (1993)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
@@ -3455,6 +3662,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>The Chronic (1992)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
@@ -3542,6 +3754,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>Bizarre Ride II the Pharcyde (1992)</t>
+        </is>
+      </c>
+      <c r="W32" t="n">
+        <v>2004</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="14" t="n">
@@ -3629,6 +3849,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>The Infamous (1995)</t>
+        </is>
+      </c>
+      <c r="W33" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="14" t="n">
@@ -3716,6 +3944,11 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>In a Major Way (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
@@ -3807,6 +4040,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Mecca and the Soul Brother (1992)</t>
+        </is>
+      </c>
+      <c r="W35" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="n">
@@ -3894,6 +4135,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>Moment of Truth (1998)</t>
+        </is>
+      </c>
+      <c r="W36" t="n">
+        <v>2003</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="n">
@@ -3985,6 +4234,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>One for All (1990)</t>
+        </is>
+      </c>
+      <c r="W37" t="n">
+        <v>2007</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="n">
@@ -4076,6 +4333,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>To the East, Blackwards (1990)</t>
+        </is>
+      </c>
+      <c r="W38" t="n">
+        <v>2007</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="14" t="n">
@@ -4163,6 +4428,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>Lifestylez ov da Poor &amp; Dangerous (1995)</t>
+        </is>
+      </c>
+      <c r="W39" t="n">
+        <v>1999</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
@@ -4250,6 +4523,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>We Can't Be Stopped (1991)</t>
+        </is>
+      </c>
+      <c r="W40" t="n">
+        <v>2005</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="14" t="n">
@@ -4341,6 +4622,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Innercity Griots (1993)</t>
+        </is>
+      </c>
+      <c r="W41" t="n">
+        <v>2011</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="n">
@@ -4432,6 +4721,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Reachin' (A New Refutation of Time and Space) (1993)</t>
+        </is>
+      </c>
+      <c r="W42" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="14" t="n">
@@ -4523,6 +4820,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>A Future Without a Past... (1991)</t>
+        </is>
+      </c>
+      <c r="W43" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="14" t="n">
@@ -4610,6 +4915,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>When Disaster Strikes... (1997)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
@@ -4697,6 +5007,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>All Eyez on Me (1996)</t>
+        </is>
+      </c>
+      <c r="W45" t="n">
+        <v>1996</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
@@ -4784,6 +5102,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>The Blueprint (2001)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
@@ -4871,6 +5194,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>The Marshall Mathers LP (2000)</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
@@ -4958,6 +5286,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>It's Dark and Hell Is Hot (1998)</t>
+        </is>
+      </c>
+      <c r="W48" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
@@ -5043,6 +5379,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>The Miseducation of Lauryn Hill (1998)</t>
+        </is>
+      </c>
+      <c r="W49" t="n">
+        <v>2002</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
@@ -5130,6 +5474,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Supa Dupa Fly (1997)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="n">
@@ -5215,6 +5564,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Black on Both Sides (1999)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
@@ -5302,6 +5656,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Quality (2002)</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
@@ -5389,6 +5748,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Aquemini (1998)</t>
+        </is>
+      </c>
+      <c r="W53" t="n">
+        <v>2006</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="14" t="n">
@@ -5476,6 +5843,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>Ghetto D (1997)</t>
+        </is>
+      </c>
+      <c r="W54" t="n">
+        <v>2005</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
@@ -5567,6 +5942,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Purple Haze (2004)</t>
+        </is>
+      </c>
+      <c r="W55" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
@@ -5658,6 +6041,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Ill Na Na (1996)</t>
+        </is>
+      </c>
+      <c r="W56" t="n">
+        <v>2008</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
@@ -5745,6 +6136,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Hard Core (1996)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
@@ -5836,6 +6232,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>400 Degreez (1998)</t>
+        </is>
+      </c>
+      <c r="W58" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
@@ -5927,6 +6331,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Can-I-Bus (1998)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
@@ -6018,6 +6427,11 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>Violent by Design (2000)</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
@@ -6105,6 +6519,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>Capital Punishment (1998)</t>
+        </is>
+      </c>
+      <c r="W61" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
@@ -6196,6 +6618,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Doe or Die (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
@@ -6283,6 +6710,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>My Beautiful Dark Twisted Fantasy (2010)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
@@ -6370,6 +6802,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Tha Carter III (2008)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
@@ -6457,6 +6894,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>Trap Muzik (2003)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
@@ -6544,6 +6986,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>The State vs. Radric Davis (2009)</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
@@ -6631,6 +7078,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Supreme Clientele (2000)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
@@ -6718,6 +7170,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Madvillainy (2004)</t>
+        </is>
+      </c>
+      <c r="W68" t="n">
+        <v>2020</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
@@ -6805,6 +7265,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Be (2005)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
@@ -6892,6 +7357,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Word of Mouf (2001)</t>
+        </is>
+      </c>
+      <c r="W70" t="n">
+        <v>2015</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
@@ -6979,6 +7452,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Let's Get It: Thug Motivation 101 (2005)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
@@ -7066,6 +7544,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>The Cool (2007)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
@@ -7153,6 +7636,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>The Diary (1994)</t>
+        </is>
+      </c>
+      <c r="W73" t="n">
+        <v>2015</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="14" t="n">
@@ -7240,6 +7731,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>Labor Days (2001)</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="14" t="n">
@@ -7331,6 +7827,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Kiss of Death (2004)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="14" t="n">
@@ -7418,6 +7919,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Get Rich or Die Tryin' (2003)</t>
+        </is>
+      </c>
+      <c r="W76" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="14" t="n">
@@ -7509,6 +8018,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Mystic Stylez (1995)</t>
+        </is>
+      </c>
+      <c r="W77" t="n">
+        <v>2008</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="14" t="n">
@@ -7596,6 +8113,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>Ridin' Dirty (1996)</t>
+        </is>
+      </c>
+      <c r="W78" t="n">
+        <v>2007</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="14" t="n">
@@ -7687,6 +8212,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>Restless (2006)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
@@ -7778,6 +8308,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>All Balls Don't Bounce (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="14" t="n">
@@ -7863,6 +8398,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>Only Built 4 Cuban Linx… (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="14" t="n">
@@ -7950,6 +8490,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Fantastic Damage (2002)</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="14" t="n">
@@ -8041,6 +8586,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>Shadows on the Sun (2003)</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="14" t="n">
@@ -8132,6 +8682,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>Revolutionary Vol. 2 (2003)</t>
+        </is>
+      </c>
+      <c r="W84" t="n">
+        <v>2011</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="14" t="n">
@@ -8219,6 +8777,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>To Pimp a Butterfly (2015)</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="14" t="n">
@@ -8306,6 +8869,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>2014 Forest Hills Drive (2014)</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="14" t="n">
@@ -8393,6 +8961,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>Jeffery (2016)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="14" t="n">
@@ -8480,6 +9053,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>DS2 (2015)</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="14" t="n">
@@ -8567,6 +9145,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>Acid Rap (2013)</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="14" t="n">
@@ -8654,6 +9237,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>Some Rap Songs (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="14" t="n">
@@ -8741,6 +9329,11 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>Dreams and Nightmares (2012)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="14" t="n">
@@ -8828,6 +9421,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>Long. Live. A$AP (2013)</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="14" t="n">
@@ -8915,6 +9513,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>Pink Friday (2010)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="n">
@@ -9002,6 +9605,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>Summertime '06 (2015)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="14" t="n">
@@ -9089,6 +9697,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>4eva Is a Mighty Long Time (2017)</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="n">
@@ -9176,6 +9789,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>Run the Jewels 2 (2014)</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="14" t="n">
@@ -9263,6 +9881,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>R.A.P. Music (2012)</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="n">
@@ -9350,6 +9973,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>Piñata (2014)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="14" t="n">
@@ -9437,6 +10065,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>Culture (2017)</t>
+        </is>
+      </c>
+      <c r="W99" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="n">
@@ -9528,6 +10164,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>Dark Sky Paradise (2015)</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="14" t="n">
@@ -9617,6 +10258,11 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>Whack World (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="n">
@@ -9704,6 +10350,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>Room 25 (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="14" t="n">
@@ -9789,6 +10440,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>CARE FOR ME (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="n">
@@ -9876,6 +10532,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>Atrocity Exhibition (2016)</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="14" t="n">
@@ -9963,6 +10624,14 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>Swimming (2018)</t>
+        </is>
+      </c>
+      <c r="W105" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="n">
@@ -10054,6 +10723,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>The Forever Story (2022)</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="14" t="n">
@@ -10141,6 +10815,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>Invasion of Privacy (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="14" t="n">
@@ -10232,6 +10911,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>Hall of Fame (2021)</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="14" t="n">
@@ -10323,6 +11007,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>SoulFly (2021)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="14" t="n">
@@ -10414,6 +11103,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>Alligator Bites Never Heal (2024)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="14" t="n">
@@ -10505,6 +11199,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>GLORIOUS (2024)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="n">
@@ -10596,6 +11295,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>WUNNA (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="14" t="n">
@@ -10687,6 +11391,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>My Turn (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="n">
@@ -10774,6 +11483,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>Tana Talk 3 (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="14" t="n">
@@ -10865,6 +11579,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>Father of 4 (2019)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="n">
@@ -10956,6 +11675,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>Angelic Hoodrat (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="14" t="n">
@@ -11047,6 +11771,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>777 (2022)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="n">
@@ -11138,6 +11867,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V118" t="inlineStr">
+        <is>
+          <t>blkswn (2017)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="14" t="n">
@@ -11223,6 +11957,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V119" t="inlineStr">
+        <is>
+          <t>Daytona (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="n">
@@ -11308,6 +12047,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V120" t="inlineStr">
+        <is>
+          <t>Igor (2019)</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="14" t="n">
@@ -11399,6 +12143,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V121" t="inlineStr">
+        <is>
+          <t>Haram (2021)</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="n">
@@ -11490,6 +12239,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V122" t="inlineStr">
+        <is>
+          <t>shut the fuck up talking to me (2021)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="14" t="n">
@@ -11581,6 +12335,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V123" t="inlineStr">
+        <is>
+          <t>The Voice (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="n">
@@ -11672,6 +12431,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V124" t="inlineStr">
+        <is>
+          <t>Painting Pictures (2017)</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="14" t="n">
@@ -11759,6 +12523,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V125" t="inlineStr">
+        <is>
+          <t>Laila's Wisdom (2017)</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="n">
@@ -11850,6 +12619,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V126" t="inlineStr">
+        <is>
+          <t>Let the Sun Talk (2019)</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="14" t="n">
@@ -11941,6 +12715,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V127" t="inlineStr">
+        <is>
+          <t>40 Dayz &amp; 40 Nightz (1998)</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="n">
@@ -12032,6 +12811,11 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V128" t="inlineStr">
+        <is>
+          <t>My Type (2019)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="14" t="n">
@@ -12123,6 +12907,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V129" t="inlineStr">
+        <is>
+          <t>Girl Code (2018)</t>
+        </is>
+      </c>
+      <c r="W129" t="n">
+        <v>2023</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="14" t="n">
@@ -12214,6 +13006,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V130" t="inlineStr">
+        <is>
+          <t>Weight of the World (2021)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -12300,6 +13097,11 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V131" t="inlineStr">
+        <is>
+          <t>Things Fall Apart (1999)</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -12391,6 +13193,14 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V132" t="inlineStr">
+        <is>
+          <t>The Truth (2000)</t>
+        </is>
+      </c>
+      <c r="W132" t="n">
+        <v>2012</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -12482,6 +13292,11 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V133" t="inlineStr">
+        <is>
+          <t>Eternal Atake (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -12573,6 +13388,14 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V134" t="inlineStr">
+        <is>
+          <t>Philadelphia Freeway (2003)</t>
+        </is>
+      </c>
+      <c r="W134" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -12664,6 +13487,14 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V135" t="inlineStr">
+        <is>
+          <t>Let There Be Eve... Ruff Ryders' First Lady (1999)</t>
+        </is>
+      </c>
+      <c r="W135" t="n">
+        <v>2013</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -12755,6 +13586,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V136" t="inlineStr">
+        <is>
+          <t>Funkdafied (1994)</t>
+        </is>
+      </c>
+      <c r="W136" t="n">
+        <v>2003</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -12846,6 +13685,11 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V137" t="inlineStr">
+        <is>
+          <t>Life Is... Too Short (1988)</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -12937,6 +13781,11 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V138" t="inlineStr">
+        <is>
+          <t>I Wish My Brother George Was Here (1991)</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -13028,6 +13877,14 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V139" t="inlineStr">
+        <is>
+          <t>Ronald Dregan: Dreganomics (2004)</t>
+        </is>
+      </c>
+      <c r="W139" t="n">
+        <v>2004</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -13119,6 +13976,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V140" t="inlineStr">
+        <is>
+          <t>Book of Ryan (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -13205,6 +14067,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V141" t="inlineStr">
+        <is>
+          <t>Live and Let Die (1992)</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -13296,6 +14163,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V142" t="inlineStr">
+        <is>
+          <t>Muddy Waters (1996)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -13387,6 +14259,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V143" t="inlineStr">
+        <is>
+          <t>Tical (1994)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -13478,6 +14355,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V144" t="inlineStr">
+        <is>
+          <t>Strictly Business (1988)</t>
+        </is>
+      </c>
+      <c r="W144" t="n">
+        <v>2008</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -13569,6 +14454,11 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V145" t="inlineStr">
+        <is>
+          <t>The Documentary (2005)</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -13660,6 +14550,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V146" t="inlineStr">
+        <is>
+          <t>O.G. Original Gangster (1991)</t>
+        </is>
+      </c>
+      <c r="W146" t="n">
+        <v>2006</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -13751,6 +14649,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V147" t="inlineStr">
+        <is>
+          <t>Victory Lap (2018)</t>
+        </is>
+      </c>
+      <c r="W147" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -13842,6 +14748,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V148" t="inlineStr">
+        <is>
+          <t>Quik Is the Name (1991)</t>
+        </is>
+      </c>
+      <c r="W148" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -13933,6 +14847,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V149" t="inlineStr">
+        <is>
+          <t>Very Necessary (1993)</t>
+        </is>
+      </c>
+      <c r="W149" t="n">
+        <v>1997</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -14024,6 +14946,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V150" t="inlineStr">
+        <is>
+          <t>Good News (2020)</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -14115,6 +15042,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V151" t="inlineStr">
+        <is>
+          <t>Make Way for the Motherlode (1991)</t>
+        </is>
+      </c>
+      <c r="W151" t="n">
+        <v>1996</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -14206,6 +15141,11 @@
           <t>Philly</t>
         </is>
       </c>
+      <c r="V152" t="inlineStr">
+        <is>
+          <t>Kollage (1996)</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -14297,6 +15237,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V153" t="inlineStr">
+        <is>
+          <t>Jeanius (2008)</t>
+        </is>
+      </c>
+      <c r="W153" t="n">
+        <v>2018</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -14388,6 +15336,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V154" t="inlineStr">
+        <is>
+          <t>Da Baddest Bitch (2000)</t>
+        </is>
+      </c>
+      <c r="W154" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -14479,6 +15435,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V155" t="inlineStr">
+        <is>
+          <t>Unlady Like (1997)</t>
+        </is>
+      </c>
+      <c r="W155" t="n">
+        <v>1998</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -14566,6 +15530,14 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V156" t="inlineStr">
+        <is>
+          <t>E. 1999 Eternal (1995)</t>
+        </is>
+      </c>
+      <c r="W156" t="n">
+        <v>2017</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -14657,6 +15629,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>On Top of the World (1995)</t>
+        </is>
+      </c>
+      <c r="W157" t="n">
+        <v>2010</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -14748,6 +15728,14 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V158" t="inlineStr">
+        <is>
+          <t>93 'til Infinity (1993)</t>
+        </is>
+      </c>
+      <c r="W158" t="n">
+        <v>2014</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -14839,6 +15827,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V159" t="inlineStr">
+        <is>
+          <t>Kamikaze (2004)</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -14930,6 +15923,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V160" t="inlineStr">
+        <is>
+          <t>All 6's and 7's (2011)</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -15019,6 +16017,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V161" t="inlineStr">
+        <is>
+          <t>Country Grammar (2000)</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -15108,6 +16111,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V162" t="inlineStr">
+        <is>
+          <t>Finally Rich (2012)</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -15199,6 +16207,11 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V163" t="inlineStr">
+        <is>
+          <t>Reloaded (2012)</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -15290,6 +16303,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V164" t="inlineStr">
+        <is>
+          <t>TA13OO (2018)</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -15375,6 +16393,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V165" t="inlineStr">
+        <is>
+          <t>The Score (1996)</t>
+        </is>
+      </c>
+      <c r="W165" t="n">
+        <v>1997</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -15466,6 +16492,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>Soul Food (1995)</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -15555,6 +16586,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V167" t="inlineStr">
+        <is>
+          <t>Funcrusher Plus (1997)</t>
+        </is>
+      </c>
+      <c r="W167" t="n">
+        <v>2000</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -15640,6 +16679,11 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V168" t="inlineStr">
+        <is>
+          <t>Hell Hath No Fury (2006)</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -15729,6 +16773,14 @@
           <t>NYC</t>
         </is>
       </c>
+      <c r="V169" t="inlineStr">
+        <is>
+          <t>Let's Get Free (2000)</t>
+        </is>
+      </c>
+      <c r="W169" t="n">
+        <v>2012</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -15818,6 +16870,14 @@
           <t>South</t>
         </is>
       </c>
+      <c r="V170" t="inlineStr">
+        <is>
+          <t>The Minstrel Show (2005)</t>
+        </is>
+      </c>
+      <c r="W170" t="n">
+        <v>2019</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -15909,6 +16969,11 @@
           <t>Midwest</t>
         </is>
       </c>
+      <c r="V171" t="inlineStr">
+        <is>
+          <t>God Loves Ugly (2002)</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -16000,6 +17065,14 @@
           <t>Bay Area</t>
         </is>
       </c>
+      <c r="V172" t="inlineStr">
+        <is>
+          <t>Blazing Arrow (2002)</t>
+        </is>
+      </c>
+      <c r="W172" t="n">
+        <v>2021</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -16091,6 +17164,14 @@
           <t>LA</t>
         </is>
       </c>
+      <c r="V173" t="inlineStr">
+        <is>
+          <t>Saturation II (2017)</t>
+        </is>
+      </c>
+      <c r="W173" t="n">
+        <v>2022</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -16180,6 +17261,11 @@
       <c r="U174" t="inlineStr">
         <is>
           <t>NYC</t>
+        </is>
+      </c>
+      <c r="V174" t="inlineStr">
+        <is>
+          <t>WWCD (2019)</t>
         </is>
       </c>
     </row>
@@ -16931,34 +18017,62 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="17"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Signature Work</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>"Title (Year)"; blank if none recorded</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>The act’s consensus defining release: an album, or a single for acts that predate albums. One per act; blank only where no recorded signature work exists (e.g. Kool Herc).</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>Critical consensus synthesis; entered 2026-07.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
-        </is>
-      </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Active Through</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>1977–present; blank = still active</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>Last year of new primary-catalog output (death, disbandment, or final album). With Debut Year, gives the active span shown on the tile modal.</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>Discographies; judgment call for gradual fade-outs.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
-        </is>
-      </c>
+      <c r="A25" s="17"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="17"/>
@@ -16966,14 +18080,10 @@
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
         <is>
-          <t>Inclusion</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
-        </is>
-      </c>
+          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
+        </is>
+      </c>
+      <c r="B26" s="17"/>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
       <c r="E26" s="17"/>
@@ -16981,12 +18091,12 @@
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>Exclusion</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
+          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
         </is>
       </c>
       <c r="C27" s="17"/>
@@ -16996,12 +18106,12 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Unit of analysis</t>
+          <t>Inclusion</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
+          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
         </is>
       </c>
       <c r="C28" s="17"/>
@@ -17011,17 +18121,47 @@
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
         <is>
-          <t>Known frame biases</t>
+          <t>Exclusion</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
         </is>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
       <c r="E29" s="17"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>Unit of analysis</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
+        </is>
+      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>Known frame biases</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+        </is>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add age dimension via Birth Year column
New Birth Year column for all 130 solo Elements (Compounds stay blank
by design: group members vary in age), documented in the Data
Dictionary. Ages derive rather than being stored: age at debut =
Debut Year - Birth Year, age at signature work = signature year -
Birth Year.

The tile modal shows "(age N)" beside the debut year for Elements. The
Careers & Longevity dashboard page gains a second chart row: age at
debut by era (boxplots + points) and age at signature work vs composite
with the median marked (26 across the dataset). Teaching prompt
extended with the age angle.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AYwyGjCcrmQGUKZPhS1uD8
</commit_message>
<xml_diff>
--- a/hiphop/data/hiphop_artists.xlsx
+++ b/hiphop/data/hiphop_artists.xlsx
@@ -829,6 +829,11 @@
           <t>Active Through</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Birth Year</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="14" t="n">
@@ -919,6 +924,9 @@
       <c r="W2" t="n">
         <v>1977</v>
       </c>
+      <c r="X2" t="n">
+        <v>1955</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="n">
@@ -1014,6 +1022,9 @@
       <c r="W3" t="n">
         <v>2009</v>
       </c>
+      <c r="X3" t="n">
+        <v>1958</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="n">
@@ -1107,6 +1118,9 @@
       <c r="W4" t="n">
         <v>1989</v>
       </c>
+      <c r="X4" t="n">
+        <v>1961</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="n">
@@ -1297,6 +1311,9 @@
       <c r="W6" t="n">
         <v>1991</v>
       </c>
+      <c r="X6" t="n">
+        <v>1957</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="n">
@@ -1389,6 +1406,9 @@
           <t>Mama Said Knock You Out (1990)</t>
         </is>
       </c>
+      <c r="X7" t="n">
+        <v>1968</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="n">
@@ -1671,6 +1691,9 @@
           <t>Criminal Minded (1987)</t>
         </is>
       </c>
+      <c r="X10" t="n">
+        <v>1965</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="n">
@@ -1862,6 +1885,9 @@
       <c r="W12" t="n">
         <v>1992</v>
       </c>
+      <c r="X12" t="n">
+        <v>1969</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="14" t="n">
@@ -1958,6 +1984,9 @@
           <t>Lyte as a Rock (1988)</t>
         </is>
       </c>
+      <c r="X13" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="14" t="n">
@@ -2057,6 +2086,9 @@
       <c r="W14" t="n">
         <v>2000</v>
       </c>
+      <c r="X14" t="n">
+        <v>1962</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="14" t="n">
@@ -2354,6 +2386,9 @@
       <c r="W17" t="n">
         <v>1995</v>
       </c>
+      <c r="X17" t="n">
+        <v>1966</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="n">
@@ -2446,6 +2481,9 @@
           <t>The Great Adventures of Slick Rick (1988)</t>
         </is>
       </c>
+      <c r="X18" t="n">
+        <v>1965</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="n">
@@ -2545,6 +2583,9 @@
       <c r="W19" t="n">
         <v>1995</v>
       </c>
+      <c r="X19" t="n">
+        <v>1965</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="n">
@@ -2640,6 +2681,9 @@
       <c r="W20" t="n">
         <v>1998</v>
       </c>
+      <c r="X20" t="n">
+        <v>1968</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="n">
@@ -2732,6 +2776,9 @@
           <t>Paid in Full (1987)</t>
         </is>
       </c>
+      <c r="X21" t="n">
+        <v>1968</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="n">
@@ -2827,6 +2874,9 @@
       <c r="W22" t="n">
         <v>1998</v>
       </c>
+      <c r="X22" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="n">
@@ -3014,6 +3064,9 @@
           <t>AmeriKKKa's Most Wanted (1990)</t>
         </is>
       </c>
+      <c r="X24" t="n">
+        <v>1969</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="n">
@@ -3296,6 +3349,9 @@
           <t>Illmatic (1994)</t>
         </is>
       </c>
+      <c r="X27" t="n">
+        <v>1973</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="n">
@@ -3391,6 +3447,9 @@
       <c r="W28" t="n">
         <v>1997</v>
       </c>
+      <c r="X28" t="n">
+        <v>1972</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="n">
@@ -3575,6 +3634,9 @@
           <t>Doggystyle (1993)</t>
         </is>
       </c>
+      <c r="X30" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="n">
@@ -3667,6 +3729,9 @@
           <t>The Chronic (1992)</t>
         </is>
       </c>
+      <c r="X31" t="n">
+        <v>1965</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="14" t="n">
@@ -3949,6 +4014,9 @@
           <t>In a Major Way (1995)</t>
         </is>
       </c>
+      <c r="X34" t="n">
+        <v>1967</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="14" t="n">
@@ -4436,6 +4504,9 @@
       <c r="W39" t="n">
         <v>1999</v>
       </c>
+      <c r="X39" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="14" t="n">
@@ -4920,6 +4991,9 @@
           <t>When Disaster Strikes... (1997)</t>
         </is>
       </c>
+      <c r="X44" t="n">
+        <v>1972</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="14" t="n">
@@ -5015,6 +5089,9 @@
       <c r="W45" t="n">
         <v>1996</v>
       </c>
+      <c r="X45" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="14" t="n">
@@ -5107,6 +5184,9 @@
           <t>The Blueprint (2001)</t>
         </is>
       </c>
+      <c r="X46" t="n">
+        <v>1969</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="14" t="n">
@@ -5199,6 +5279,9 @@
           <t>The Marshall Mathers LP (2000)</t>
         </is>
       </c>
+      <c r="X47" t="n">
+        <v>1972</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="14" t="n">
@@ -5294,6 +5377,9 @@
       <c r="W48" t="n">
         <v>2021</v>
       </c>
+      <c r="X48" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="14" t="n">
@@ -5387,6 +5473,9 @@
       <c r="W49" t="n">
         <v>2002</v>
       </c>
+      <c r="X49" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="14" t="n">
@@ -5479,6 +5568,9 @@
           <t>Supa Dupa Fly (1997)</t>
         </is>
       </c>
+      <c r="X50" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="n">
@@ -5569,6 +5661,9 @@
           <t>Black on Both Sides (1999)</t>
         </is>
       </c>
+      <c r="X51" t="n">
+        <v>1973</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="14" t="n">
@@ -5661,6 +5756,9 @@
           <t>Quality (2002)</t>
         </is>
       </c>
+      <c r="X52" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="14" t="n">
@@ -5851,6 +5949,9 @@
       <c r="W54" t="n">
         <v>2005</v>
       </c>
+      <c r="X54" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="14" t="n">
@@ -5950,6 +6051,9 @@
       <c r="W55" t="n">
         <v>2019</v>
       </c>
+      <c r="X55" t="n">
+        <v>1976</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="14" t="n">
@@ -6049,6 +6153,9 @@
       <c r="W56" t="n">
         <v>2008</v>
       </c>
+      <c r="X56" t="n">
+        <v>1978</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="14" t="n">
@@ -6141,6 +6248,9 @@
           <t>Hard Core (1996)</t>
         </is>
       </c>
+      <c r="X57" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="14" t="n">
@@ -6240,6 +6350,9 @@
       <c r="W58" t="n">
         <v>2019</v>
       </c>
+      <c r="X58" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="14" t="n">
@@ -6336,6 +6449,9 @@
           <t>Can-I-Bus (1998)</t>
         </is>
       </c>
+      <c r="X59" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="n">
@@ -6432,6 +6548,9 @@
           <t>Violent by Design (2000)</t>
         </is>
       </c>
+      <c r="X60" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="14" t="n">
@@ -6527,6 +6646,9 @@
       <c r="W61" t="n">
         <v>2000</v>
       </c>
+      <c r="X61" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="14" t="n">
@@ -6623,6 +6745,9 @@
           <t>Doe or Die (1995)</t>
         </is>
       </c>
+      <c r="X62" t="n">
+        <v>1972</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="n">
@@ -6715,6 +6840,9 @@
           <t>My Beautiful Dark Twisted Fantasy (2010)</t>
         </is>
       </c>
+      <c r="X63" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="14" t="n">
@@ -6807,6 +6935,9 @@
           <t>Tha Carter III (2008)</t>
         </is>
       </c>
+      <c r="X64" t="n">
+        <v>1982</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="14" t="n">
@@ -6899,6 +7030,9 @@
           <t>Trap Muzik (2003)</t>
         </is>
       </c>
+      <c r="X65" t="n">
+        <v>1980</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="14" t="n">
@@ -6991,6 +7125,9 @@
           <t>The State vs. Radric Davis (2009)</t>
         </is>
       </c>
+      <c r="X66" t="n">
+        <v>1980</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n">
@@ -7083,6 +7220,9 @@
           <t>Supreme Clientele (2000)</t>
         </is>
       </c>
+      <c r="X67" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n">
@@ -7178,6 +7318,9 @@
       <c r="W68" t="n">
         <v>2020</v>
       </c>
+      <c r="X68" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="14" t="n">
@@ -7270,6 +7413,9 @@
           <t>Be (2005)</t>
         </is>
       </c>
+      <c r="X69" t="n">
+        <v>1972</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="14" t="n">
@@ -7365,6 +7511,9 @@
       <c r="W70" t="n">
         <v>2015</v>
       </c>
+      <c r="X70" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="14" t="n">
@@ -7457,6 +7606,9 @@
           <t>Let's Get It: Thug Motivation 101 (2005)</t>
         </is>
       </c>
+      <c r="X71" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="14" t="n">
@@ -7549,6 +7701,9 @@
           <t>The Cool (2007)</t>
         </is>
       </c>
+      <c r="X72" t="n">
+        <v>1982</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="14" t="n">
@@ -7644,6 +7799,9 @@
       <c r="W73" t="n">
         <v>2015</v>
       </c>
+      <c r="X73" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="14" t="n">
@@ -7736,6 +7894,9 @@
           <t>Labor Days (2001)</t>
         </is>
       </c>
+      <c r="X74" t="n">
+        <v>1976</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="14" t="n">
@@ -7832,6 +7993,9 @@
           <t>Kiss of Death (2004)</t>
         </is>
       </c>
+      <c r="X75" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="14" t="n">
@@ -7927,6 +8091,9 @@
       <c r="W76" t="n">
         <v>2014</v>
       </c>
+      <c r="X76" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="14" t="n">
@@ -8217,6 +8384,9 @@
           <t>Restless (2006)</t>
         </is>
       </c>
+      <c r="X79" t="n">
+        <v>1980</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
@@ -8313,6 +8483,9 @@
           <t>All Balls Don't Bounce (1995)</t>
         </is>
       </c>
+      <c r="X80" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="14" t="n">
@@ -8403,6 +8576,9 @@
           <t>Only Built 4 Cuban Linx… (1995)</t>
         </is>
       </c>
+      <c r="X81" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="14" t="n">
@@ -8495,6 +8671,9 @@
           <t>Fantastic Damage (2002)</t>
         </is>
       </c>
+      <c r="X82" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="14" t="n">
@@ -8591,6 +8770,9 @@
           <t>Shadows on the Sun (2003)</t>
         </is>
       </c>
+      <c r="X83" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="14" t="n">
@@ -8690,6 +8872,9 @@
       <c r="W84" t="n">
         <v>2011</v>
       </c>
+      <c r="X84" t="n">
+        <v>1978</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="14" t="n">
@@ -8782,6 +8967,9 @@
           <t>To Pimp a Butterfly (2015)</t>
         </is>
       </c>
+      <c r="X85" t="n">
+        <v>1987</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="14" t="n">
@@ -8874,6 +9062,9 @@
           <t>2014 Forest Hills Drive (2014)</t>
         </is>
       </c>
+      <c r="X86" t="n">
+        <v>1985</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="14" t="n">
@@ -8966,6 +9157,9 @@
           <t>Jeffery (2016)</t>
         </is>
       </c>
+      <c r="X87" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="14" t="n">
@@ -9058,6 +9252,9 @@
           <t>DS2 (2015)</t>
         </is>
       </c>
+      <c r="X88" t="n">
+        <v>1983</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="14" t="n">
@@ -9150,6 +9347,9 @@
           <t>Acid Rap (2013)</t>
         </is>
       </c>
+      <c r="X89" t="n">
+        <v>1993</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="14" t="n">
@@ -9242,6 +9442,9 @@
           <t>Some Rap Songs (2018)</t>
         </is>
       </c>
+      <c r="X90" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="14" t="n">
@@ -9334,6 +9537,9 @@
           <t>Dreams and Nightmares (2012)</t>
         </is>
       </c>
+      <c r="X91" t="n">
+        <v>1987</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="14" t="n">
@@ -9426,6 +9632,9 @@
           <t>Long. Live. A$AP (2013)</t>
         </is>
       </c>
+      <c r="X92" t="n">
+        <v>1988</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="14" t="n">
@@ -9518,6 +9727,9 @@
           <t>Pink Friday (2010)</t>
         </is>
       </c>
+      <c r="X93" t="n">
+        <v>1982</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="n">
@@ -9610,6 +9822,9 @@
           <t>Summertime '06 (2015)</t>
         </is>
       </c>
+      <c r="X94" t="n">
+        <v>1993</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="14" t="n">
@@ -9702,6 +9917,9 @@
           <t>4eva Is a Mighty Long Time (2017)</t>
         </is>
       </c>
+      <c r="X95" t="n">
+        <v>1986</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="n">
@@ -9886,6 +10104,9 @@
           <t>R.A.P. Music (2012)</t>
         </is>
       </c>
+      <c r="X97" t="n">
+        <v>1975</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="n">
@@ -9978,6 +10199,9 @@
           <t>Piñata (2014)</t>
         </is>
       </c>
+      <c r="X98" t="n">
+        <v>1982</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="14" t="n">
@@ -10169,6 +10393,9 @@
           <t>Dark Sky Paradise (2015)</t>
         </is>
       </c>
+      <c r="X100" t="n">
+        <v>1988</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="14" t="n">
@@ -10263,6 +10490,9 @@
           <t>Whack World (2018)</t>
         </is>
       </c>
+      <c r="X101" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="n">
@@ -10355,6 +10585,9 @@
           <t>Room 25 (2018)</t>
         </is>
       </c>
+      <c r="X102" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="14" t="n">
@@ -10445,6 +10678,9 @@
           <t>CARE FOR ME (2018)</t>
         </is>
       </c>
+      <c r="X103" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="n">
@@ -10537,6 +10773,9 @@
           <t>Atrocity Exhibition (2016)</t>
         </is>
       </c>
+      <c r="X104" t="n">
+        <v>1981</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="14" t="n">
@@ -10632,6 +10871,9 @@
       <c r="W105" t="n">
         <v>2018</v>
       </c>
+      <c r="X105" t="n">
+        <v>1992</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="n">
@@ -10728,6 +10970,9 @@
           <t>The Forever Story (2022)</t>
         </is>
       </c>
+      <c r="X106" t="n">
+        <v>1990</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="14" t="n">
@@ -10820,6 +11065,9 @@
           <t>Invasion of Privacy (2018)</t>
         </is>
       </c>
+      <c r="X107" t="n">
+        <v>1992</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="14" t="n">
@@ -10916,6 +11164,9 @@
           <t>Hall of Fame (2021)</t>
         </is>
       </c>
+      <c r="X108" t="n">
+        <v>1999</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="14" t="n">
@@ -11012,6 +11263,9 @@
           <t>SoulFly (2021)</t>
         </is>
       </c>
+      <c r="X109" t="n">
+        <v>1999</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="14" t="n">
@@ -11108,6 +11362,9 @@
           <t>Alligator Bites Never Heal (2024)</t>
         </is>
       </c>
+      <c r="X110" t="n">
+        <v>1998</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="14" t="n">
@@ -11204,6 +11461,9 @@
           <t>GLORIOUS (2024)</t>
         </is>
       </c>
+      <c r="X111" t="n">
+        <v>1999</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="n">
@@ -11300,6 +11560,9 @@
           <t>WUNNA (2020)</t>
         </is>
       </c>
+      <c r="X112" t="n">
+        <v>1993</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="14" t="n">
@@ -11396,6 +11659,9 @@
           <t>My Turn (2020)</t>
         </is>
       </c>
+      <c r="X113" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="n">
@@ -11488,6 +11754,9 @@
           <t>Tana Talk 3 (2018)</t>
         </is>
       </c>
+      <c r="X114" t="n">
+        <v>1984</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="14" t="n">
@@ -11584,6 +11853,9 @@
           <t>Father of 4 (2019)</t>
         </is>
       </c>
+      <c r="X115" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="n">
@@ -11680,6 +11952,9 @@
           <t>Angelic Hoodrat (2020)</t>
         </is>
       </c>
+      <c r="X116" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="14" t="n">
@@ -11776,6 +12051,9 @@
           <t>777 (2022)</t>
         </is>
       </c>
+      <c r="X117" t="n">
+        <v>1998</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="n">
@@ -11872,6 +12150,9 @@
           <t>blkswn (2017)</t>
         </is>
       </c>
+      <c r="X118" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="14" t="n">
@@ -11962,6 +12243,9 @@
           <t>Daytona (2018)</t>
         </is>
       </c>
+      <c r="X119" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="n">
@@ -12052,6 +12336,9 @@
           <t>Igor (2019)</t>
         </is>
       </c>
+      <c r="X120" t="n">
+        <v>1991</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="14" t="n">
@@ -12244,6 +12531,9 @@
           <t>shut the fuck up talking to me (2021)</t>
         </is>
       </c>
+      <c r="X122" t="n">
+        <v>1990</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="14" t="n">
@@ -12340,6 +12630,9 @@
           <t>The Voice (2020)</t>
         </is>
       </c>
+      <c r="X123" t="n">
+        <v>1992</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="n">
@@ -12436,6 +12729,9 @@
           <t>Painting Pictures (2017)</t>
         </is>
       </c>
+      <c r="X124" t="n">
+        <v>1997</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="14" t="n">
@@ -12528,6 +12824,9 @@
           <t>Laila's Wisdom (2017)</t>
         </is>
       </c>
+      <c r="X125" t="n">
+        <v>1983</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="n">
@@ -12624,6 +12923,9 @@
           <t>Let the Sun Talk (2019)</t>
         </is>
       </c>
+      <c r="X126" t="n">
+        <v>1999</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="14" t="n">
@@ -12720,6 +13022,9 @@
           <t>40 Dayz &amp; 40 Nightz (1998)</t>
         </is>
       </c>
+      <c r="X127" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="n">
@@ -12816,6 +13121,9 @@
           <t>My Type (2019)</t>
         </is>
       </c>
+      <c r="X128" t="n">
+        <v>1993</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="14" t="n">
@@ -13011,6 +13319,9 @@
           <t>Weight of the World (2021)</t>
         </is>
       </c>
+      <c r="X130" t="n">
+        <v>1990</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -13201,6 +13512,9 @@
       <c r="W132" t="n">
         <v>2012</v>
       </c>
+      <c r="X132" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -13297,6 +13611,9 @@
           <t>Eternal Atake (2020)</t>
         </is>
       </c>
+      <c r="X133" t="n">
+        <v>1994</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -13396,6 +13713,9 @@
       <c r="W134" t="n">
         <v>2018</v>
       </c>
+      <c r="X134" t="n">
+        <v>1978</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -13495,6 +13815,9 @@
       <c r="W135" t="n">
         <v>2013</v>
       </c>
+      <c r="X135" t="n">
+        <v>1978</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -13594,6 +13917,9 @@
       <c r="W136" t="n">
         <v>2003</v>
       </c>
+      <c r="X136" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -13690,6 +14016,9 @@
           <t>Life Is... Too Short (1988)</t>
         </is>
       </c>
+      <c r="X137" t="n">
+        <v>1966</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -13786,6 +14115,9 @@
           <t>I Wish My Brother George Was Here (1991)</t>
         </is>
       </c>
+      <c r="X138" t="n">
+        <v>1972</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -13885,6 +14217,9 @@
       <c r="W139" t="n">
         <v>2004</v>
       </c>
+      <c r="X139" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -13981,6 +14316,9 @@
           <t>Book of Ryan (2018)</t>
         </is>
       </c>
+      <c r="X140" t="n">
+        <v>1977</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -14072,6 +14410,9 @@
           <t>Live and Let Die (1992)</t>
         </is>
       </c>
+      <c r="X141" t="n">
+        <v>1968</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -14168,6 +14509,9 @@
           <t>Muddy Waters (1996)</t>
         </is>
       </c>
+      <c r="X142" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -14264,6 +14608,9 @@
           <t>Tical (1994)</t>
         </is>
       </c>
+      <c r="X143" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -14459,6 +14806,9 @@
           <t>The Documentary (2005)</t>
         </is>
       </c>
+      <c r="X145" t="n">
+        <v>1979</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -14558,6 +14908,9 @@
       <c r="W146" t="n">
         <v>2006</v>
       </c>
+      <c r="X146" t="n">
+        <v>1958</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -14657,6 +15010,9 @@
       <c r="W147" t="n">
         <v>2019</v>
       </c>
+      <c r="X147" t="n">
+        <v>1985</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -14756,6 +15112,9 @@
       <c r="W148" t="n">
         <v>2017</v>
       </c>
+      <c r="X148" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -14951,6 +15310,9 @@
           <t>Good News (2020)</t>
         </is>
       </c>
+      <c r="X150" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -15050,6 +15412,9 @@
       <c r="W151" t="n">
         <v>1996</v>
       </c>
+      <c r="X151" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -15146,6 +15511,9 @@
           <t>Kollage (1996)</t>
         </is>
       </c>
+      <c r="X152" t="n">
+        <v>1966</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -15245,6 +15613,9 @@
       <c r="W153" t="n">
         <v>2018</v>
       </c>
+      <c r="X153" t="n">
+        <v>1976</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -15344,6 +15715,9 @@
       <c r="W154" t="n">
         <v>2019</v>
       </c>
+      <c r="X154" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -15443,6 +15817,9 @@
       <c r="W155" t="n">
         <v>1998</v>
       </c>
+      <c r="X155" t="n">
+        <v>1970</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -15832,6 +16209,9 @@
           <t>Kamikaze (2004)</t>
         </is>
       </c>
+      <c r="X159" t="n">
+        <v>1973</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -15928,6 +16308,9 @@
           <t>All 6's and 7's (2011)</t>
         </is>
       </c>
+      <c r="X160" t="n">
+        <v>1971</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -16022,6 +16405,9 @@
           <t>Country Grammar (2000)</t>
         </is>
       </c>
+      <c r="X161" t="n">
+        <v>1974</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -16116,6 +16502,9 @@
           <t>Finally Rich (2012)</t>
         </is>
       </c>
+      <c r="X162" t="n">
+        <v>1995</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -16212,6 +16601,9 @@
           <t>Reloaded (2012)</t>
         </is>
       </c>
+      <c r="X163" t="n">
+        <v>1978</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -16307,6 +16699,9 @@
         <is>
           <t>TA13OO (2018)</t>
         </is>
+      </c>
+      <c r="X164" t="n">
+        <v>1995</v>
       </c>
     </row>
     <row r="165">
@@ -18071,18 +18466,34 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Birth Year</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Integer</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>1955–present; Elements only (blank for Compounds)</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>Birth year of the solo artist, for age-at-debut and age-at-signature-work analysis. Group members vary in age, so Compounds are left blank.</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>Public record (documented dates of birth).</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
-        <is>
-          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
-        </is>
-      </c>
+      <c r="A26" s="17"/>
       <c r="B26" s="17"/>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -18091,14 +18502,10 @@
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
         <is>
-          <t>Population</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
-        </is>
-      </c>
+          <t>SAMPLING FRAME &amp; SCOPE RULES</t>
+        </is>
+      </c>
+      <c r="B27" s="17"/>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
@@ -18106,12 +18513,12 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>Inclusion</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
+          <t>US-based hip-hop acts with a national critical record, 1973–present.</t>
         </is>
       </c>
       <c r="C28" s="17"/>
@@ -18121,12 +18528,12 @@
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
         <is>
-          <t>Exclusion</t>
+          <t>Inclusion</t>
         </is>
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
+          <t>US-born or US-scene-based acts affiliated with a US label/scene during their defining run.</t>
         </is>
       </c>
       <c r="C29" s="17"/>
@@ -18136,12 +18543,12 @@
     <row r="30">
       <c r="A30" s="18" t="inlineStr">
         <is>
-          <t>Unit of analysis</t>
+          <t>Exclusion</t>
         </is>
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
+          <t>International and UK acts (scope decision to keep the frame tractable); acts without national critical coverage (survivorship limitation, documented).</t>
         </is>
       </c>
       <c r="C30" s="17"/>
@@ -18151,17 +18558,32 @@
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>Known frame biases</t>
+          <t>Unit of analysis</t>
         </is>
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+          <t>The act (solo artist or group). Groups are Compounds; solo careers are Elements; both may appear.</t>
         </is>
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
       <c r="E31" s="17"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
+        <is>
+          <t>Known frame biases</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Over-represents critical acclaim, NYC, Golden Age, and men. See Confidence Guide sheet for the full bias table.</t>
+        </is>
+      </c>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>